<commit_message>
SIMULATION : S a V ne s'affichent plus sur une ligne vide
Deux tests, parce qu'une restitution peut echouer des deux facons : plus
d'identite (le POV ne ramene pas la ligne) ou plus de chiffres (la ligne existe
mais la mesure est absente).

    IF(OR($C13="",COUNT($H13:$Q13)=0),"", ... )

Verifie sur trois cas : les 60 lignes remplies (60 traitees, ecart T-O
0,000000000), une restitution a 20 lignes (20 traitees, 40 blanchies, ecart
inchange sur les 20), et une ligne dont l'identite est la mais pas les mesures
(blanchie).

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01BCU7CjG5rh6esFZ9teHY6F
</commit_message>
<xml_diff>
--- a/eduservices/SIMULATION_CORRIGE.xlsx
+++ b/eduservices/SIMULATION_CORRIGE.xlsx
@@ -11908,16 +11908,16 @@
         <v>112</v>
       </c>
       <c r="S13" s="74">
-        <f>IF($R13="Fermer","",IF(SUMIFS($I$13:$I$72,$C$13:$C$72,$C13,$D$13:$D$72,$D13,$R$13:$R$72,"&lt;&gt;Fermer")=0,$M13,$M13+SUMIFS($M$13:$M$72,$C$13:$C$72,$C13,$D$13:$D$72,$D13,$R$13:$R$72,"Fermer")*$I13/SUMIFS($I$13:$I$72,$C$13:$C$72,$C13,$D$13:$D$72,$D13,$R$13:$R$72,"&lt;&gt;Fermer")))</f>
+        <f>IF(OR($C13="",COUNT($H13:$Q13)=0),"",IF($R13="Fermer","",IF(SUMIFS($I$13:$I$72,$C$13:$C$72,$C13,$D$13:$D$72,$D13,$R$13:$R$72,"&lt;&gt;Fermer")=0,$M13,$M13+SUMIFS($M$13:$M$72,$C$13:$C$72,$C13,$D$13:$D$72,$D13,$R$13:$R$72,"Fermer")*$I13/SUMIFS($I$13:$I$72,$C$13:$C$72,$C13,$D$13:$D$72,$D13,$R$13:$R$72,"&lt;&gt;Fermer"))))</f>
       </c>
       <c r="T13" s="75">
-        <f>IF($R13="Fermer","",$J13-$K13-$S13)</f>
+        <f>IF(OR($C13="",COUNT($H13:$Q13)=0),"",IF($R13="Fermer","",$J13-$K13-$S13))</f>
       </c>
       <c r="U13" s="74">
-        <f>IF($R13="Fermer",-$L13,0)</f>
+        <f>IF(OR($C13="",COUNT($H13:$Q13)=0),"",IF($R13="Fermer",-$L13,0))</f>
       </c>
       <c r="V13" s="76">
-        <f>IF($R13="Fermer","Fermer = perdre "&amp;TEXT($L13,"#,##0")&amp;" € de contribution. Le fixe, lui, reste.",IF(AND($O13&gt;=0,$T13&lt;0),"BASCULE : saine avant, en déficit à cause d'une fermeture voisine.",IF(AND($O13&lt;0,$L13&gt;0),"Déficit au coût complet mais contribution positive : ne pas fermer, c'est un artefact d'allocation.",IF($O13&lt;0,"Contribution négative : vrai point dur.","Rentable. Point mort "&amp;TEXT($P13,"#,##0")&amp;" étudiants, marge de sécurité "&amp;TEXT($Q13,"0%")&amp;"."))))</f>
+        <f>IF(OR($C13="",COUNT($H13:$Q13)=0),"",IF($R13="Fermer","Fermer = perdre "&amp;TEXT($L13,"#,##0")&amp;" € de contribution. Le fixe, lui, reste.",IF(AND($O13&gt;=0,$T13&lt;0),"BASCULE : saine avant, en déficit à cause d'une fermeture voisine.",IF(AND($O13&lt;0,$L13&gt;0),"Déficit au coût complet mais contribution positive : ne pas fermer, c'est un artefact d'allocation.",IF($O13&lt;0,"Contribution négative : vrai point dur.","Rentable. Point mort "&amp;TEXT($P13,"#,##0")&amp;" étudiants, marge de sécurité "&amp;TEXT($Q13,"0%")&amp;".")))))</f>
       </c>
       <c r="W13" s="77"/>
       <c r="X13" s="77"/>
@@ -11975,16 +11975,16 @@
         <v>115</v>
       </c>
       <c r="S14" s="74">
-        <f>IF($R14="Fermer","",IF(SUMIFS($I$13:$I$72,$C$13:$C$72,$C14,$D$13:$D$72,$D14,$R$13:$R$72,"&lt;&gt;Fermer")=0,$M14,$M14+SUMIFS($M$13:$M$72,$C$13:$C$72,$C14,$D$13:$D$72,$D14,$R$13:$R$72,"Fermer")*$I14/SUMIFS($I$13:$I$72,$C$13:$C$72,$C14,$D$13:$D$72,$D14,$R$13:$R$72,"&lt;&gt;Fermer")))</f>
+        <f>IF(OR($C14="",COUNT($H14:$Q14)=0),"",IF($R14="Fermer","",IF(SUMIFS($I$13:$I$72,$C$13:$C$72,$C14,$D$13:$D$72,$D14,$R$13:$R$72,"&lt;&gt;Fermer")=0,$M14,$M14+SUMIFS($M$13:$M$72,$C$13:$C$72,$C14,$D$13:$D$72,$D14,$R$13:$R$72,"Fermer")*$I14/SUMIFS($I$13:$I$72,$C$13:$C$72,$C14,$D$13:$D$72,$D14,$R$13:$R$72,"&lt;&gt;Fermer"))))</f>
       </c>
       <c r="T14" s="75">
-        <f>IF($R14="Fermer","",$J14-$K14-$S14)</f>
+        <f>IF(OR($C14="",COUNT($H14:$Q14)=0),"",IF($R14="Fermer","",$J14-$K14-$S14))</f>
       </c>
       <c r="U14" s="74">
-        <f>IF($R14="Fermer",-$L14,0)</f>
+        <f>IF(OR($C14="",COUNT($H14:$Q14)=0),"",IF($R14="Fermer",-$L14,0))</f>
       </c>
       <c r="V14" s="76">
-        <f>IF($R14="Fermer","Fermer = perdre "&amp;TEXT($L14,"#,##0")&amp;" € de contribution. Le fixe, lui, reste.",IF(AND($O14&gt;=0,$T14&lt;0),"BASCULE : saine avant, en déficit à cause d'une fermeture voisine.",IF(AND($O14&lt;0,$L14&gt;0),"Déficit au coût complet mais contribution positive : ne pas fermer, c'est un artefact d'allocation.",IF($O14&lt;0,"Contribution négative : vrai point dur.","Rentable. Point mort "&amp;TEXT($P14,"#,##0")&amp;" étudiants, marge de sécurité "&amp;TEXT($Q14,"0%")&amp;"."))))</f>
+        <f>IF(OR($C14="",COUNT($H14:$Q14)=0),"",IF($R14="Fermer","Fermer = perdre "&amp;TEXT($L14,"#,##0")&amp;" € de contribution. Le fixe, lui, reste.",IF(AND($O14&gt;=0,$T14&lt;0),"BASCULE : saine avant, en déficit à cause d'une fermeture voisine.",IF(AND($O14&lt;0,$L14&gt;0),"Déficit au coût complet mais contribution positive : ne pas fermer, c'est un artefact d'allocation.",IF($O14&lt;0,"Contribution négative : vrai point dur.","Rentable. Point mort "&amp;TEXT($P14,"#,##0")&amp;" étudiants, marge de sécurité "&amp;TEXT($Q14,"0%")&amp;".")))))</f>
       </c>
     </row>
     <row r="15" ht="14.25" customHeight="1">
@@ -12037,16 +12037,16 @@
         <v>115</v>
       </c>
       <c r="S15" s="74">
-        <f>IF($R15="Fermer","",IF(SUMIFS($I$13:$I$72,$C$13:$C$72,$C15,$D$13:$D$72,$D15,$R$13:$R$72,"&lt;&gt;Fermer")=0,$M15,$M15+SUMIFS($M$13:$M$72,$C$13:$C$72,$C15,$D$13:$D$72,$D15,$R$13:$R$72,"Fermer")*$I15/SUMIFS($I$13:$I$72,$C$13:$C$72,$C15,$D$13:$D$72,$D15,$R$13:$R$72,"&lt;&gt;Fermer")))</f>
+        <f>IF(OR($C15="",COUNT($H15:$Q15)=0),"",IF($R15="Fermer","",IF(SUMIFS($I$13:$I$72,$C$13:$C$72,$C15,$D$13:$D$72,$D15,$R$13:$R$72,"&lt;&gt;Fermer")=0,$M15,$M15+SUMIFS($M$13:$M$72,$C$13:$C$72,$C15,$D$13:$D$72,$D15,$R$13:$R$72,"Fermer")*$I15/SUMIFS($I$13:$I$72,$C$13:$C$72,$C15,$D$13:$D$72,$D15,$R$13:$R$72,"&lt;&gt;Fermer"))))</f>
       </c>
       <c r="T15" s="75">
-        <f>IF($R15="Fermer","",$J15-$K15-$S15)</f>
+        <f>IF(OR($C15="",COUNT($H15:$Q15)=0),"",IF($R15="Fermer","",$J15-$K15-$S15))</f>
       </c>
       <c r="U15" s="74">
-        <f>IF($R15="Fermer",-$L15,0)</f>
+        <f>IF(OR($C15="",COUNT($H15:$Q15)=0),"",IF($R15="Fermer",-$L15,0))</f>
       </c>
       <c r="V15" s="76">
-        <f>IF($R15="Fermer","Fermer = perdre "&amp;TEXT($L15,"#,##0")&amp;" € de contribution. Le fixe, lui, reste.",IF(AND($O15&gt;=0,$T15&lt;0),"BASCULE : saine avant, en déficit à cause d'une fermeture voisine.",IF(AND($O15&lt;0,$L15&gt;0),"Déficit au coût complet mais contribution positive : ne pas fermer, c'est un artefact d'allocation.",IF($O15&lt;0,"Contribution négative : vrai point dur.","Rentable. Point mort "&amp;TEXT($P15,"#,##0")&amp;" étudiants, marge de sécurité "&amp;TEXT($Q15,"0%")&amp;"."))))</f>
+        <f>IF(OR($C15="",COUNT($H15:$Q15)=0),"",IF($R15="Fermer","Fermer = perdre "&amp;TEXT($L15,"#,##0")&amp;" € de contribution. Le fixe, lui, reste.",IF(AND($O15&gt;=0,$T15&lt;0),"BASCULE : saine avant, en déficit à cause d'une fermeture voisine.",IF(AND($O15&lt;0,$L15&gt;0),"Déficit au coût complet mais contribution positive : ne pas fermer, c'est un artefact d'allocation.",IF($O15&lt;0,"Contribution négative : vrai point dur.","Rentable. Point mort "&amp;TEXT($P15,"#,##0")&amp;" étudiants, marge de sécurité "&amp;TEXT($Q15,"0%")&amp;".")))))</f>
       </c>
     </row>
     <row r="16" ht="14.25" customHeight="1">
@@ -12099,16 +12099,16 @@
         <v>112</v>
       </c>
       <c r="S16" s="74">
-        <f>IF($R16="Fermer","",IF(SUMIFS($I$13:$I$72,$C$13:$C$72,$C16,$D$13:$D$72,$D16,$R$13:$R$72,"&lt;&gt;Fermer")=0,$M16,$M16+SUMIFS($M$13:$M$72,$C$13:$C$72,$C16,$D$13:$D$72,$D16,$R$13:$R$72,"Fermer")*$I16/SUMIFS($I$13:$I$72,$C$13:$C$72,$C16,$D$13:$D$72,$D16,$R$13:$R$72,"&lt;&gt;Fermer")))</f>
+        <f>IF(OR($C16="",COUNT($H16:$Q16)=0),"",IF($R16="Fermer","",IF(SUMIFS($I$13:$I$72,$C$13:$C$72,$C16,$D$13:$D$72,$D16,$R$13:$R$72,"&lt;&gt;Fermer")=0,$M16,$M16+SUMIFS($M$13:$M$72,$C$13:$C$72,$C16,$D$13:$D$72,$D16,$R$13:$R$72,"Fermer")*$I16/SUMIFS($I$13:$I$72,$C$13:$C$72,$C16,$D$13:$D$72,$D16,$R$13:$R$72,"&lt;&gt;Fermer"))))</f>
       </c>
       <c r="T16" s="75">
-        <f>IF($R16="Fermer","",$J16-$K16-$S16)</f>
+        <f>IF(OR($C16="",COUNT($H16:$Q16)=0),"",IF($R16="Fermer","",$J16-$K16-$S16))</f>
       </c>
       <c r="U16" s="74">
-        <f>IF($R16="Fermer",-$L16,0)</f>
+        <f>IF(OR($C16="",COUNT($H16:$Q16)=0),"",IF($R16="Fermer",-$L16,0))</f>
       </c>
       <c r="V16" s="76">
-        <f>IF($R16="Fermer","Fermer = perdre "&amp;TEXT($L16,"#,##0")&amp;" € de contribution. Le fixe, lui, reste.",IF(AND($O16&gt;=0,$T16&lt;0),"BASCULE : saine avant, en déficit à cause d'une fermeture voisine.",IF(AND($O16&lt;0,$L16&gt;0),"Déficit au coût complet mais contribution positive : ne pas fermer, c'est un artefact d'allocation.",IF($O16&lt;0,"Contribution négative : vrai point dur.","Rentable. Point mort "&amp;TEXT($P16,"#,##0")&amp;" étudiants, marge de sécurité "&amp;TEXT($Q16,"0%")&amp;"."))))</f>
+        <f>IF(OR($C16="",COUNT($H16:$Q16)=0),"",IF($R16="Fermer","Fermer = perdre "&amp;TEXT($L16,"#,##0")&amp;" € de contribution. Le fixe, lui, reste.",IF(AND($O16&gt;=0,$T16&lt;0),"BASCULE : saine avant, en déficit à cause d'une fermeture voisine.",IF(AND($O16&lt;0,$L16&gt;0),"Déficit au coût complet mais contribution positive : ne pas fermer, c'est un artefact d'allocation.",IF($O16&lt;0,"Contribution négative : vrai point dur.","Rentable. Point mort "&amp;TEXT($P16,"#,##0")&amp;" étudiants, marge de sécurité "&amp;TEXT($Q16,"0%")&amp;".")))))</f>
       </c>
     </row>
     <row r="17" ht="14.25" customHeight="1">
@@ -12161,16 +12161,16 @@
         <v>115</v>
       </c>
       <c r="S17" s="74">
-        <f>IF($R17="Fermer","",IF(SUMIFS($I$13:$I$72,$C$13:$C$72,$C17,$D$13:$D$72,$D17,$R$13:$R$72,"&lt;&gt;Fermer")=0,$M17,$M17+SUMIFS($M$13:$M$72,$C$13:$C$72,$C17,$D$13:$D$72,$D17,$R$13:$R$72,"Fermer")*$I17/SUMIFS($I$13:$I$72,$C$13:$C$72,$C17,$D$13:$D$72,$D17,$R$13:$R$72,"&lt;&gt;Fermer")))</f>
+        <f>IF(OR($C17="",COUNT($H17:$Q17)=0),"",IF($R17="Fermer","",IF(SUMIFS($I$13:$I$72,$C$13:$C$72,$C17,$D$13:$D$72,$D17,$R$13:$R$72,"&lt;&gt;Fermer")=0,$M17,$M17+SUMIFS($M$13:$M$72,$C$13:$C$72,$C17,$D$13:$D$72,$D17,$R$13:$R$72,"Fermer")*$I17/SUMIFS($I$13:$I$72,$C$13:$C$72,$C17,$D$13:$D$72,$D17,$R$13:$R$72,"&lt;&gt;Fermer"))))</f>
       </c>
       <c r="T17" s="75">
-        <f>IF($R17="Fermer","",$J17-$K17-$S17)</f>
+        <f>IF(OR($C17="",COUNT($H17:$Q17)=0),"",IF($R17="Fermer","",$J17-$K17-$S17))</f>
       </c>
       <c r="U17" s="74">
-        <f>IF($R17="Fermer",-$L17,0)</f>
+        <f>IF(OR($C17="",COUNT($H17:$Q17)=0),"",IF($R17="Fermer",-$L17,0))</f>
       </c>
       <c r="V17" s="76">
-        <f>IF($R17="Fermer","Fermer = perdre "&amp;TEXT($L17,"#,##0")&amp;" € de contribution. Le fixe, lui, reste.",IF(AND($O17&gt;=0,$T17&lt;0),"BASCULE : saine avant, en déficit à cause d'une fermeture voisine.",IF(AND($O17&lt;0,$L17&gt;0),"Déficit au coût complet mais contribution positive : ne pas fermer, c'est un artefact d'allocation.",IF($O17&lt;0,"Contribution négative : vrai point dur.","Rentable. Point mort "&amp;TEXT($P17,"#,##0")&amp;" étudiants, marge de sécurité "&amp;TEXT($Q17,"0%")&amp;"."))))</f>
+        <f>IF(OR($C17="",COUNT($H17:$Q17)=0),"",IF($R17="Fermer","Fermer = perdre "&amp;TEXT($L17,"#,##0")&amp;" € de contribution. Le fixe, lui, reste.",IF(AND($O17&gt;=0,$T17&lt;0),"BASCULE : saine avant, en déficit à cause d'une fermeture voisine.",IF(AND($O17&lt;0,$L17&gt;0),"Déficit au coût complet mais contribution positive : ne pas fermer, c'est un artefact d'allocation.",IF($O17&lt;0,"Contribution négative : vrai point dur.","Rentable. Point mort "&amp;TEXT($P17,"#,##0")&amp;" étudiants, marge de sécurité "&amp;TEXT($Q17,"0%")&amp;".")))))</f>
       </c>
     </row>
     <row r="18" ht="14.25" customHeight="1">
@@ -12223,16 +12223,16 @@
         <v>115</v>
       </c>
       <c r="S18" s="74">
-        <f>IF($R18="Fermer","",IF(SUMIFS($I$13:$I$72,$C$13:$C$72,$C18,$D$13:$D$72,$D18,$R$13:$R$72,"&lt;&gt;Fermer")=0,$M18,$M18+SUMIFS($M$13:$M$72,$C$13:$C$72,$C18,$D$13:$D$72,$D18,$R$13:$R$72,"Fermer")*$I18/SUMIFS($I$13:$I$72,$C$13:$C$72,$C18,$D$13:$D$72,$D18,$R$13:$R$72,"&lt;&gt;Fermer")))</f>
+        <f>IF(OR($C18="",COUNT($H18:$Q18)=0),"",IF($R18="Fermer","",IF(SUMIFS($I$13:$I$72,$C$13:$C$72,$C18,$D$13:$D$72,$D18,$R$13:$R$72,"&lt;&gt;Fermer")=0,$M18,$M18+SUMIFS($M$13:$M$72,$C$13:$C$72,$C18,$D$13:$D$72,$D18,$R$13:$R$72,"Fermer")*$I18/SUMIFS($I$13:$I$72,$C$13:$C$72,$C18,$D$13:$D$72,$D18,$R$13:$R$72,"&lt;&gt;Fermer"))))</f>
       </c>
       <c r="T18" s="75">
-        <f>IF($R18="Fermer","",$J18-$K18-$S18)</f>
+        <f>IF(OR($C18="",COUNT($H18:$Q18)=0),"",IF($R18="Fermer","",$J18-$K18-$S18))</f>
       </c>
       <c r="U18" s="74">
-        <f>IF($R18="Fermer",-$L18,0)</f>
+        <f>IF(OR($C18="",COUNT($H18:$Q18)=0),"",IF($R18="Fermer",-$L18,0))</f>
       </c>
       <c r="V18" s="76">
-        <f>IF($R18="Fermer","Fermer = perdre "&amp;TEXT($L18,"#,##0")&amp;" € de contribution. Le fixe, lui, reste.",IF(AND($O18&gt;=0,$T18&lt;0),"BASCULE : saine avant, en déficit à cause d'une fermeture voisine.",IF(AND($O18&lt;0,$L18&gt;0),"Déficit au coût complet mais contribution positive : ne pas fermer, c'est un artefact d'allocation.",IF($O18&lt;0,"Contribution négative : vrai point dur.","Rentable. Point mort "&amp;TEXT($P18,"#,##0")&amp;" étudiants, marge de sécurité "&amp;TEXT($Q18,"0%")&amp;"."))))</f>
+        <f>IF(OR($C18="",COUNT($H18:$Q18)=0),"",IF($R18="Fermer","Fermer = perdre "&amp;TEXT($L18,"#,##0")&amp;" € de contribution. Le fixe, lui, reste.",IF(AND($O18&gt;=0,$T18&lt;0),"BASCULE : saine avant, en déficit à cause d'une fermeture voisine.",IF(AND($O18&lt;0,$L18&gt;0),"Déficit au coût complet mais contribution positive : ne pas fermer, c'est un artefact d'allocation.",IF($O18&lt;0,"Contribution négative : vrai point dur.","Rentable. Point mort "&amp;TEXT($P18,"#,##0")&amp;" étudiants, marge de sécurité "&amp;TEXT($Q18,"0%")&amp;".")))))</f>
       </c>
     </row>
     <row r="19" ht="14.25" customHeight="1">
@@ -12285,16 +12285,16 @@
         <v>112</v>
       </c>
       <c r="S19" s="74">
-        <f>IF($R19="Fermer","",IF(SUMIFS($I$13:$I$72,$C$13:$C$72,$C19,$D$13:$D$72,$D19,$R$13:$R$72,"&lt;&gt;Fermer")=0,$M19,$M19+SUMIFS($M$13:$M$72,$C$13:$C$72,$C19,$D$13:$D$72,$D19,$R$13:$R$72,"Fermer")*$I19/SUMIFS($I$13:$I$72,$C$13:$C$72,$C19,$D$13:$D$72,$D19,$R$13:$R$72,"&lt;&gt;Fermer")))</f>
+        <f>IF(OR($C19="",COUNT($H19:$Q19)=0),"",IF($R19="Fermer","",IF(SUMIFS($I$13:$I$72,$C$13:$C$72,$C19,$D$13:$D$72,$D19,$R$13:$R$72,"&lt;&gt;Fermer")=0,$M19,$M19+SUMIFS($M$13:$M$72,$C$13:$C$72,$C19,$D$13:$D$72,$D19,$R$13:$R$72,"Fermer")*$I19/SUMIFS($I$13:$I$72,$C$13:$C$72,$C19,$D$13:$D$72,$D19,$R$13:$R$72,"&lt;&gt;Fermer"))))</f>
       </c>
       <c r="T19" s="75">
-        <f>IF($R19="Fermer","",$J19-$K19-$S19)</f>
+        <f>IF(OR($C19="",COUNT($H19:$Q19)=0),"",IF($R19="Fermer","",$J19-$K19-$S19))</f>
       </c>
       <c r="U19" s="74">
-        <f>IF($R19="Fermer",-$L19,0)</f>
+        <f>IF(OR($C19="",COUNT($H19:$Q19)=0),"",IF($R19="Fermer",-$L19,0))</f>
       </c>
       <c r="V19" s="76">
-        <f>IF($R19="Fermer","Fermer = perdre "&amp;TEXT($L19,"#,##0")&amp;" € de contribution. Le fixe, lui, reste.",IF(AND($O19&gt;=0,$T19&lt;0),"BASCULE : saine avant, en déficit à cause d'une fermeture voisine.",IF(AND($O19&lt;0,$L19&gt;0),"Déficit au coût complet mais contribution positive : ne pas fermer, c'est un artefact d'allocation.",IF($O19&lt;0,"Contribution négative : vrai point dur.","Rentable. Point mort "&amp;TEXT($P19,"#,##0")&amp;" étudiants, marge de sécurité "&amp;TEXT($Q19,"0%")&amp;"."))))</f>
+        <f>IF(OR($C19="",COUNT($H19:$Q19)=0),"",IF($R19="Fermer","Fermer = perdre "&amp;TEXT($L19,"#,##0")&amp;" € de contribution. Le fixe, lui, reste.",IF(AND($O19&gt;=0,$T19&lt;0),"BASCULE : saine avant, en déficit à cause d'une fermeture voisine.",IF(AND($O19&lt;0,$L19&gt;0),"Déficit au coût complet mais contribution positive : ne pas fermer, c'est un artefact d'allocation.",IF($O19&lt;0,"Contribution négative : vrai point dur.","Rentable. Point mort "&amp;TEXT($P19,"#,##0")&amp;" étudiants, marge de sécurité "&amp;TEXT($Q19,"0%")&amp;".")))))</f>
       </c>
     </row>
     <row r="20" ht="14.25" customHeight="1">
@@ -12347,16 +12347,16 @@
         <v>115</v>
       </c>
       <c r="S20" s="74">
-        <f>IF($R20="Fermer","",IF(SUMIFS($I$13:$I$72,$C$13:$C$72,$C20,$D$13:$D$72,$D20,$R$13:$R$72,"&lt;&gt;Fermer")=0,$M20,$M20+SUMIFS($M$13:$M$72,$C$13:$C$72,$C20,$D$13:$D$72,$D20,$R$13:$R$72,"Fermer")*$I20/SUMIFS($I$13:$I$72,$C$13:$C$72,$C20,$D$13:$D$72,$D20,$R$13:$R$72,"&lt;&gt;Fermer")))</f>
+        <f>IF(OR($C20="",COUNT($H20:$Q20)=0),"",IF($R20="Fermer","",IF(SUMIFS($I$13:$I$72,$C$13:$C$72,$C20,$D$13:$D$72,$D20,$R$13:$R$72,"&lt;&gt;Fermer")=0,$M20,$M20+SUMIFS($M$13:$M$72,$C$13:$C$72,$C20,$D$13:$D$72,$D20,$R$13:$R$72,"Fermer")*$I20/SUMIFS($I$13:$I$72,$C$13:$C$72,$C20,$D$13:$D$72,$D20,$R$13:$R$72,"&lt;&gt;Fermer"))))</f>
       </c>
       <c r="T20" s="75">
-        <f>IF($R20="Fermer","",$J20-$K20-$S20)</f>
+        <f>IF(OR($C20="",COUNT($H20:$Q20)=0),"",IF($R20="Fermer","",$J20-$K20-$S20))</f>
       </c>
       <c r="U20" s="74">
-        <f>IF($R20="Fermer",-$L20,0)</f>
+        <f>IF(OR($C20="",COUNT($H20:$Q20)=0),"",IF($R20="Fermer",-$L20,0))</f>
       </c>
       <c r="V20" s="76">
-        <f>IF($R20="Fermer","Fermer = perdre "&amp;TEXT($L20,"#,##0")&amp;" € de contribution. Le fixe, lui, reste.",IF(AND($O20&gt;=0,$T20&lt;0),"BASCULE : saine avant, en déficit à cause d'une fermeture voisine.",IF(AND($O20&lt;0,$L20&gt;0),"Déficit au coût complet mais contribution positive : ne pas fermer, c'est un artefact d'allocation.",IF($O20&lt;0,"Contribution négative : vrai point dur.","Rentable. Point mort "&amp;TEXT($P20,"#,##0")&amp;" étudiants, marge de sécurité "&amp;TEXT($Q20,"0%")&amp;"."))))</f>
+        <f>IF(OR($C20="",COUNT($H20:$Q20)=0),"",IF($R20="Fermer","Fermer = perdre "&amp;TEXT($L20,"#,##0")&amp;" € de contribution. Le fixe, lui, reste.",IF(AND($O20&gt;=0,$T20&lt;0),"BASCULE : saine avant, en déficit à cause d'une fermeture voisine.",IF(AND($O20&lt;0,$L20&gt;0),"Déficit au coût complet mais contribution positive : ne pas fermer, c'est un artefact d'allocation.",IF($O20&lt;0,"Contribution négative : vrai point dur.","Rentable. Point mort "&amp;TEXT($P20,"#,##0")&amp;" étudiants, marge de sécurité "&amp;TEXT($Q20,"0%")&amp;".")))))</f>
       </c>
     </row>
     <row r="21" ht="14.25" customHeight="1">
@@ -12409,16 +12409,16 @@
         <v>115</v>
       </c>
       <c r="S21" s="74">
-        <f>IF($R21="Fermer","",IF(SUMIFS($I$13:$I$72,$C$13:$C$72,$C21,$D$13:$D$72,$D21,$R$13:$R$72,"&lt;&gt;Fermer")=0,$M21,$M21+SUMIFS($M$13:$M$72,$C$13:$C$72,$C21,$D$13:$D$72,$D21,$R$13:$R$72,"Fermer")*$I21/SUMIFS($I$13:$I$72,$C$13:$C$72,$C21,$D$13:$D$72,$D21,$R$13:$R$72,"&lt;&gt;Fermer")))</f>
+        <f>IF(OR($C21="",COUNT($H21:$Q21)=0),"",IF($R21="Fermer","",IF(SUMIFS($I$13:$I$72,$C$13:$C$72,$C21,$D$13:$D$72,$D21,$R$13:$R$72,"&lt;&gt;Fermer")=0,$M21,$M21+SUMIFS($M$13:$M$72,$C$13:$C$72,$C21,$D$13:$D$72,$D21,$R$13:$R$72,"Fermer")*$I21/SUMIFS($I$13:$I$72,$C$13:$C$72,$C21,$D$13:$D$72,$D21,$R$13:$R$72,"&lt;&gt;Fermer"))))</f>
       </c>
       <c r="T21" s="75">
-        <f>IF($R21="Fermer","",$J21-$K21-$S21)</f>
+        <f>IF(OR($C21="",COUNT($H21:$Q21)=0),"",IF($R21="Fermer","",$J21-$K21-$S21))</f>
       </c>
       <c r="U21" s="74">
-        <f>IF($R21="Fermer",-$L21,0)</f>
+        <f>IF(OR($C21="",COUNT($H21:$Q21)=0),"",IF($R21="Fermer",-$L21,0))</f>
       </c>
       <c r="V21" s="76">
-        <f>IF($R21="Fermer","Fermer = perdre "&amp;TEXT($L21,"#,##0")&amp;" € de contribution. Le fixe, lui, reste.",IF(AND($O21&gt;=0,$T21&lt;0),"BASCULE : saine avant, en déficit à cause d'une fermeture voisine.",IF(AND($O21&lt;0,$L21&gt;0),"Déficit au coût complet mais contribution positive : ne pas fermer, c'est un artefact d'allocation.",IF($O21&lt;0,"Contribution négative : vrai point dur.","Rentable. Point mort "&amp;TEXT($P21,"#,##0")&amp;" étudiants, marge de sécurité "&amp;TEXT($Q21,"0%")&amp;"."))))</f>
+        <f>IF(OR($C21="",COUNT($H21:$Q21)=0),"",IF($R21="Fermer","Fermer = perdre "&amp;TEXT($L21,"#,##0")&amp;" € de contribution. Le fixe, lui, reste.",IF(AND($O21&gt;=0,$T21&lt;0),"BASCULE : saine avant, en déficit à cause d'une fermeture voisine.",IF(AND($O21&lt;0,$L21&gt;0),"Déficit au coût complet mais contribution positive : ne pas fermer, c'est un artefact d'allocation.",IF($O21&lt;0,"Contribution négative : vrai point dur.","Rentable. Point mort "&amp;TEXT($P21,"#,##0")&amp;" étudiants, marge de sécurité "&amp;TEXT($Q21,"0%")&amp;".")))))</f>
       </c>
     </row>
     <row r="22" ht="14.25" customHeight="1">
@@ -12471,16 +12471,16 @@
         <v>112</v>
       </c>
       <c r="S22" s="74">
-        <f>IF($R22="Fermer","",IF(SUMIFS($I$13:$I$72,$C$13:$C$72,$C22,$D$13:$D$72,$D22,$R$13:$R$72,"&lt;&gt;Fermer")=0,$M22,$M22+SUMIFS($M$13:$M$72,$C$13:$C$72,$C22,$D$13:$D$72,$D22,$R$13:$R$72,"Fermer")*$I22/SUMIFS($I$13:$I$72,$C$13:$C$72,$C22,$D$13:$D$72,$D22,$R$13:$R$72,"&lt;&gt;Fermer")))</f>
+        <f>IF(OR($C22="",COUNT($H22:$Q22)=0),"",IF($R22="Fermer","",IF(SUMIFS($I$13:$I$72,$C$13:$C$72,$C22,$D$13:$D$72,$D22,$R$13:$R$72,"&lt;&gt;Fermer")=0,$M22,$M22+SUMIFS($M$13:$M$72,$C$13:$C$72,$C22,$D$13:$D$72,$D22,$R$13:$R$72,"Fermer")*$I22/SUMIFS($I$13:$I$72,$C$13:$C$72,$C22,$D$13:$D$72,$D22,$R$13:$R$72,"&lt;&gt;Fermer"))))</f>
       </c>
       <c r="T22" s="75">
-        <f>IF($R22="Fermer","",$J22-$K22-$S22)</f>
+        <f>IF(OR($C22="",COUNT($H22:$Q22)=0),"",IF($R22="Fermer","",$J22-$K22-$S22))</f>
       </c>
       <c r="U22" s="74">
-        <f>IF($R22="Fermer",-$L22,0)</f>
+        <f>IF(OR($C22="",COUNT($H22:$Q22)=0),"",IF($R22="Fermer",-$L22,0))</f>
       </c>
       <c r="V22" s="76">
-        <f>IF($R22="Fermer","Fermer = perdre "&amp;TEXT($L22,"#,##0")&amp;" € de contribution. Le fixe, lui, reste.",IF(AND($O22&gt;=0,$T22&lt;0),"BASCULE : saine avant, en déficit à cause d'une fermeture voisine.",IF(AND($O22&lt;0,$L22&gt;0),"Déficit au coût complet mais contribution positive : ne pas fermer, c'est un artefact d'allocation.",IF($O22&lt;0,"Contribution négative : vrai point dur.","Rentable. Point mort "&amp;TEXT($P22,"#,##0")&amp;" étudiants, marge de sécurité "&amp;TEXT($Q22,"0%")&amp;"."))))</f>
+        <f>IF(OR($C22="",COUNT($H22:$Q22)=0),"",IF($R22="Fermer","Fermer = perdre "&amp;TEXT($L22,"#,##0")&amp;" € de contribution. Le fixe, lui, reste.",IF(AND($O22&gt;=0,$T22&lt;0),"BASCULE : saine avant, en déficit à cause d'une fermeture voisine.",IF(AND($O22&lt;0,$L22&gt;0),"Déficit au coût complet mais contribution positive : ne pas fermer, c'est un artefact d'allocation.",IF($O22&lt;0,"Contribution négative : vrai point dur.","Rentable. Point mort "&amp;TEXT($P22,"#,##0")&amp;" étudiants, marge de sécurité "&amp;TEXT($Q22,"0%")&amp;".")))))</f>
       </c>
     </row>
     <row r="23" ht="14.25" customHeight="1">
@@ -12533,16 +12533,16 @@
         <v>115</v>
       </c>
       <c r="S23" s="74">
-        <f>IF($R23="Fermer","",IF(SUMIFS($I$13:$I$72,$C$13:$C$72,$C23,$D$13:$D$72,$D23,$R$13:$R$72,"&lt;&gt;Fermer")=0,$M23,$M23+SUMIFS($M$13:$M$72,$C$13:$C$72,$C23,$D$13:$D$72,$D23,$R$13:$R$72,"Fermer")*$I23/SUMIFS($I$13:$I$72,$C$13:$C$72,$C23,$D$13:$D$72,$D23,$R$13:$R$72,"&lt;&gt;Fermer")))</f>
+        <f>IF(OR($C23="",COUNT($H23:$Q23)=0),"",IF($R23="Fermer","",IF(SUMIFS($I$13:$I$72,$C$13:$C$72,$C23,$D$13:$D$72,$D23,$R$13:$R$72,"&lt;&gt;Fermer")=0,$M23,$M23+SUMIFS($M$13:$M$72,$C$13:$C$72,$C23,$D$13:$D$72,$D23,$R$13:$R$72,"Fermer")*$I23/SUMIFS($I$13:$I$72,$C$13:$C$72,$C23,$D$13:$D$72,$D23,$R$13:$R$72,"&lt;&gt;Fermer"))))</f>
       </c>
       <c r="T23" s="75">
-        <f>IF($R23="Fermer","",$J23-$K23-$S23)</f>
+        <f>IF(OR($C23="",COUNT($H23:$Q23)=0),"",IF($R23="Fermer","",$J23-$K23-$S23))</f>
       </c>
       <c r="U23" s="74">
-        <f>IF($R23="Fermer",-$L23,0)</f>
+        <f>IF(OR($C23="",COUNT($H23:$Q23)=0),"",IF($R23="Fermer",-$L23,0))</f>
       </c>
       <c r="V23" s="76">
-        <f>IF($R23="Fermer","Fermer = perdre "&amp;TEXT($L23,"#,##0")&amp;" € de contribution. Le fixe, lui, reste.",IF(AND($O23&gt;=0,$T23&lt;0),"BASCULE : saine avant, en déficit à cause d'une fermeture voisine.",IF(AND($O23&lt;0,$L23&gt;0),"Déficit au coût complet mais contribution positive : ne pas fermer, c'est un artefact d'allocation.",IF($O23&lt;0,"Contribution négative : vrai point dur.","Rentable. Point mort "&amp;TEXT($P23,"#,##0")&amp;" étudiants, marge de sécurité "&amp;TEXT($Q23,"0%")&amp;"."))))</f>
+        <f>IF(OR($C23="",COUNT($H23:$Q23)=0),"",IF($R23="Fermer","Fermer = perdre "&amp;TEXT($L23,"#,##0")&amp;" € de contribution. Le fixe, lui, reste.",IF(AND($O23&gt;=0,$T23&lt;0),"BASCULE : saine avant, en déficit à cause d'une fermeture voisine.",IF(AND($O23&lt;0,$L23&gt;0),"Déficit au coût complet mais contribution positive : ne pas fermer, c'est un artefact d'allocation.",IF($O23&lt;0,"Contribution négative : vrai point dur.","Rentable. Point mort "&amp;TEXT($P23,"#,##0")&amp;" étudiants, marge de sécurité "&amp;TEXT($Q23,"0%")&amp;".")))))</f>
       </c>
     </row>
     <row r="24" ht="14.25" customHeight="1">
@@ -12595,16 +12595,16 @@
         <v>115</v>
       </c>
       <c r="S24" s="74">
-        <f>IF($R24="Fermer","",IF(SUMIFS($I$13:$I$72,$C$13:$C$72,$C24,$D$13:$D$72,$D24,$R$13:$R$72,"&lt;&gt;Fermer")=0,$M24,$M24+SUMIFS($M$13:$M$72,$C$13:$C$72,$C24,$D$13:$D$72,$D24,$R$13:$R$72,"Fermer")*$I24/SUMIFS($I$13:$I$72,$C$13:$C$72,$C24,$D$13:$D$72,$D24,$R$13:$R$72,"&lt;&gt;Fermer")))</f>
+        <f>IF(OR($C24="",COUNT($H24:$Q24)=0),"",IF($R24="Fermer","",IF(SUMIFS($I$13:$I$72,$C$13:$C$72,$C24,$D$13:$D$72,$D24,$R$13:$R$72,"&lt;&gt;Fermer")=0,$M24,$M24+SUMIFS($M$13:$M$72,$C$13:$C$72,$C24,$D$13:$D$72,$D24,$R$13:$R$72,"Fermer")*$I24/SUMIFS($I$13:$I$72,$C$13:$C$72,$C24,$D$13:$D$72,$D24,$R$13:$R$72,"&lt;&gt;Fermer"))))</f>
       </c>
       <c r="T24" s="75">
-        <f>IF($R24="Fermer","",$J24-$K24-$S24)</f>
+        <f>IF(OR($C24="",COUNT($H24:$Q24)=0),"",IF($R24="Fermer","",$J24-$K24-$S24))</f>
       </c>
       <c r="U24" s="74">
-        <f>IF($R24="Fermer",-$L24,0)</f>
+        <f>IF(OR($C24="",COUNT($H24:$Q24)=0),"",IF($R24="Fermer",-$L24,0))</f>
       </c>
       <c r="V24" s="76">
-        <f>IF($R24="Fermer","Fermer = perdre "&amp;TEXT($L24,"#,##0")&amp;" € de contribution. Le fixe, lui, reste.",IF(AND($O24&gt;=0,$T24&lt;0),"BASCULE : saine avant, en déficit à cause d'une fermeture voisine.",IF(AND($O24&lt;0,$L24&gt;0),"Déficit au coût complet mais contribution positive : ne pas fermer, c'est un artefact d'allocation.",IF($O24&lt;0,"Contribution négative : vrai point dur.","Rentable. Point mort "&amp;TEXT($P24,"#,##0")&amp;" étudiants, marge de sécurité "&amp;TEXT($Q24,"0%")&amp;"."))))</f>
+        <f>IF(OR($C24="",COUNT($H24:$Q24)=0),"",IF($R24="Fermer","Fermer = perdre "&amp;TEXT($L24,"#,##0")&amp;" € de contribution. Le fixe, lui, reste.",IF(AND($O24&gt;=0,$T24&lt;0),"BASCULE : saine avant, en déficit à cause d'une fermeture voisine.",IF(AND($O24&lt;0,$L24&gt;0),"Déficit au coût complet mais contribution positive : ne pas fermer, c'est un artefact d'allocation.",IF($O24&lt;0,"Contribution négative : vrai point dur.","Rentable. Point mort "&amp;TEXT($P24,"#,##0")&amp;" étudiants, marge de sécurité "&amp;TEXT($Q24,"0%")&amp;".")))))</f>
       </c>
     </row>
     <row r="25" ht="14.25" customHeight="1">
@@ -12657,16 +12657,16 @@
         <v>112</v>
       </c>
       <c r="S25" s="74">
-        <f>IF($R25="Fermer","",IF(SUMIFS($I$13:$I$72,$C$13:$C$72,$C25,$D$13:$D$72,$D25,$R$13:$R$72,"&lt;&gt;Fermer")=0,$M25,$M25+SUMIFS($M$13:$M$72,$C$13:$C$72,$C25,$D$13:$D$72,$D25,$R$13:$R$72,"Fermer")*$I25/SUMIFS($I$13:$I$72,$C$13:$C$72,$C25,$D$13:$D$72,$D25,$R$13:$R$72,"&lt;&gt;Fermer")))</f>
+        <f>IF(OR($C25="",COUNT($H25:$Q25)=0),"",IF($R25="Fermer","",IF(SUMIFS($I$13:$I$72,$C$13:$C$72,$C25,$D$13:$D$72,$D25,$R$13:$R$72,"&lt;&gt;Fermer")=0,$M25,$M25+SUMIFS($M$13:$M$72,$C$13:$C$72,$C25,$D$13:$D$72,$D25,$R$13:$R$72,"Fermer")*$I25/SUMIFS($I$13:$I$72,$C$13:$C$72,$C25,$D$13:$D$72,$D25,$R$13:$R$72,"&lt;&gt;Fermer"))))</f>
       </c>
       <c r="T25" s="75">
-        <f>IF($R25="Fermer","",$J25-$K25-$S25)</f>
+        <f>IF(OR($C25="",COUNT($H25:$Q25)=0),"",IF($R25="Fermer","",$J25-$K25-$S25))</f>
       </c>
       <c r="U25" s="74">
-        <f>IF($R25="Fermer",-$L25,0)</f>
+        <f>IF(OR($C25="",COUNT($H25:$Q25)=0),"",IF($R25="Fermer",-$L25,0))</f>
       </c>
       <c r="V25" s="76">
-        <f>IF($R25="Fermer","Fermer = perdre "&amp;TEXT($L25,"#,##0")&amp;" € de contribution. Le fixe, lui, reste.",IF(AND($O25&gt;=0,$T25&lt;0),"BASCULE : saine avant, en déficit à cause d'une fermeture voisine.",IF(AND($O25&lt;0,$L25&gt;0),"Déficit au coût complet mais contribution positive : ne pas fermer, c'est un artefact d'allocation.",IF($O25&lt;0,"Contribution négative : vrai point dur.","Rentable. Point mort "&amp;TEXT($P25,"#,##0")&amp;" étudiants, marge de sécurité "&amp;TEXT($Q25,"0%")&amp;"."))))</f>
+        <f>IF(OR($C25="",COUNT($H25:$Q25)=0),"",IF($R25="Fermer","Fermer = perdre "&amp;TEXT($L25,"#,##0")&amp;" € de contribution. Le fixe, lui, reste.",IF(AND($O25&gt;=0,$T25&lt;0),"BASCULE : saine avant, en déficit à cause d'une fermeture voisine.",IF(AND($O25&lt;0,$L25&gt;0),"Déficit au coût complet mais contribution positive : ne pas fermer, c'est un artefact d'allocation.",IF($O25&lt;0,"Contribution négative : vrai point dur.","Rentable. Point mort "&amp;TEXT($P25,"#,##0")&amp;" étudiants, marge de sécurité "&amp;TEXT($Q25,"0%")&amp;".")))))</f>
       </c>
     </row>
     <row r="26" ht="14.25" customHeight="1">
@@ -12719,16 +12719,16 @@
         <v>115</v>
       </c>
       <c r="S26" s="74">
-        <f>IF($R26="Fermer","",IF(SUMIFS($I$13:$I$72,$C$13:$C$72,$C26,$D$13:$D$72,$D26,$R$13:$R$72,"&lt;&gt;Fermer")=0,$M26,$M26+SUMIFS($M$13:$M$72,$C$13:$C$72,$C26,$D$13:$D$72,$D26,$R$13:$R$72,"Fermer")*$I26/SUMIFS($I$13:$I$72,$C$13:$C$72,$C26,$D$13:$D$72,$D26,$R$13:$R$72,"&lt;&gt;Fermer")))</f>
+        <f>IF(OR($C26="",COUNT($H26:$Q26)=0),"",IF($R26="Fermer","",IF(SUMIFS($I$13:$I$72,$C$13:$C$72,$C26,$D$13:$D$72,$D26,$R$13:$R$72,"&lt;&gt;Fermer")=0,$M26,$M26+SUMIFS($M$13:$M$72,$C$13:$C$72,$C26,$D$13:$D$72,$D26,$R$13:$R$72,"Fermer")*$I26/SUMIFS($I$13:$I$72,$C$13:$C$72,$C26,$D$13:$D$72,$D26,$R$13:$R$72,"&lt;&gt;Fermer"))))</f>
       </c>
       <c r="T26" s="75">
-        <f>IF($R26="Fermer","",$J26-$K26-$S26)</f>
+        <f>IF(OR($C26="",COUNT($H26:$Q26)=0),"",IF($R26="Fermer","",$J26-$K26-$S26))</f>
       </c>
       <c r="U26" s="74">
-        <f>IF($R26="Fermer",-$L26,0)</f>
+        <f>IF(OR($C26="",COUNT($H26:$Q26)=0),"",IF($R26="Fermer",-$L26,0))</f>
       </c>
       <c r="V26" s="76">
-        <f>IF($R26="Fermer","Fermer = perdre "&amp;TEXT($L26,"#,##0")&amp;" € de contribution. Le fixe, lui, reste.",IF(AND($O26&gt;=0,$T26&lt;0),"BASCULE : saine avant, en déficit à cause d'une fermeture voisine.",IF(AND($O26&lt;0,$L26&gt;0),"Déficit au coût complet mais contribution positive : ne pas fermer, c'est un artefact d'allocation.",IF($O26&lt;0,"Contribution négative : vrai point dur.","Rentable. Point mort "&amp;TEXT($P26,"#,##0")&amp;" étudiants, marge de sécurité "&amp;TEXT($Q26,"0%")&amp;"."))))</f>
+        <f>IF(OR($C26="",COUNT($H26:$Q26)=0),"",IF($R26="Fermer","Fermer = perdre "&amp;TEXT($L26,"#,##0")&amp;" € de contribution. Le fixe, lui, reste.",IF(AND($O26&gt;=0,$T26&lt;0),"BASCULE : saine avant, en déficit à cause d'une fermeture voisine.",IF(AND($O26&lt;0,$L26&gt;0),"Déficit au coût complet mais contribution positive : ne pas fermer, c'est un artefact d'allocation.",IF($O26&lt;0,"Contribution négative : vrai point dur.","Rentable. Point mort "&amp;TEXT($P26,"#,##0")&amp;" étudiants, marge de sécurité "&amp;TEXT($Q26,"0%")&amp;".")))))</f>
       </c>
     </row>
     <row r="27" ht="14.25" customHeight="1">
@@ -12781,16 +12781,16 @@
         <v>112</v>
       </c>
       <c r="S27" s="74">
-        <f>IF($R27="Fermer","",IF(SUMIFS($I$13:$I$72,$C$13:$C$72,$C27,$D$13:$D$72,$D27,$R$13:$R$72,"&lt;&gt;Fermer")=0,$M27,$M27+SUMIFS($M$13:$M$72,$C$13:$C$72,$C27,$D$13:$D$72,$D27,$R$13:$R$72,"Fermer")*$I27/SUMIFS($I$13:$I$72,$C$13:$C$72,$C27,$D$13:$D$72,$D27,$R$13:$R$72,"&lt;&gt;Fermer")))</f>
+        <f>IF(OR($C27="",COUNT($H27:$Q27)=0),"",IF($R27="Fermer","",IF(SUMIFS($I$13:$I$72,$C$13:$C$72,$C27,$D$13:$D$72,$D27,$R$13:$R$72,"&lt;&gt;Fermer")=0,$M27,$M27+SUMIFS($M$13:$M$72,$C$13:$C$72,$C27,$D$13:$D$72,$D27,$R$13:$R$72,"Fermer")*$I27/SUMIFS($I$13:$I$72,$C$13:$C$72,$C27,$D$13:$D$72,$D27,$R$13:$R$72,"&lt;&gt;Fermer"))))</f>
       </c>
       <c r="T27" s="75">
-        <f>IF($R27="Fermer","",$J27-$K27-$S27)</f>
+        <f>IF(OR($C27="",COUNT($H27:$Q27)=0),"",IF($R27="Fermer","",$J27-$K27-$S27))</f>
       </c>
       <c r="U27" s="74">
-        <f>IF($R27="Fermer",-$L27,0)</f>
+        <f>IF(OR($C27="",COUNT($H27:$Q27)=0),"",IF($R27="Fermer",-$L27,0))</f>
       </c>
       <c r="V27" s="76">
-        <f>IF($R27="Fermer","Fermer = perdre "&amp;TEXT($L27,"#,##0")&amp;" € de contribution. Le fixe, lui, reste.",IF(AND($O27&gt;=0,$T27&lt;0),"BASCULE : saine avant, en déficit à cause d'une fermeture voisine.",IF(AND($O27&lt;0,$L27&gt;0),"Déficit au coût complet mais contribution positive : ne pas fermer, c'est un artefact d'allocation.",IF($O27&lt;0,"Contribution négative : vrai point dur.","Rentable. Point mort "&amp;TEXT($P27,"#,##0")&amp;" étudiants, marge de sécurité "&amp;TEXT($Q27,"0%")&amp;"."))))</f>
+        <f>IF(OR($C27="",COUNT($H27:$Q27)=0),"",IF($R27="Fermer","Fermer = perdre "&amp;TEXT($L27,"#,##0")&amp;" € de contribution. Le fixe, lui, reste.",IF(AND($O27&gt;=0,$T27&lt;0),"BASCULE : saine avant, en déficit à cause d'une fermeture voisine.",IF(AND($O27&lt;0,$L27&gt;0),"Déficit au coût complet mais contribution positive : ne pas fermer, c'est un artefact d'allocation.",IF($O27&lt;0,"Contribution négative : vrai point dur.","Rentable. Point mort "&amp;TEXT($P27,"#,##0")&amp;" étudiants, marge de sécurité "&amp;TEXT($Q27,"0%")&amp;".")))))</f>
       </c>
     </row>
     <row r="28" ht="14.25" customHeight="1">
@@ -12843,16 +12843,16 @@
         <v>115</v>
       </c>
       <c r="S28" s="74">
-        <f>IF($R28="Fermer","",IF(SUMIFS($I$13:$I$72,$C$13:$C$72,$C28,$D$13:$D$72,$D28,$R$13:$R$72,"&lt;&gt;Fermer")=0,$M28,$M28+SUMIFS($M$13:$M$72,$C$13:$C$72,$C28,$D$13:$D$72,$D28,$R$13:$R$72,"Fermer")*$I28/SUMIFS($I$13:$I$72,$C$13:$C$72,$C28,$D$13:$D$72,$D28,$R$13:$R$72,"&lt;&gt;Fermer")))</f>
+        <f>IF(OR($C28="",COUNT($H28:$Q28)=0),"",IF($R28="Fermer","",IF(SUMIFS($I$13:$I$72,$C$13:$C$72,$C28,$D$13:$D$72,$D28,$R$13:$R$72,"&lt;&gt;Fermer")=0,$M28,$M28+SUMIFS($M$13:$M$72,$C$13:$C$72,$C28,$D$13:$D$72,$D28,$R$13:$R$72,"Fermer")*$I28/SUMIFS($I$13:$I$72,$C$13:$C$72,$C28,$D$13:$D$72,$D28,$R$13:$R$72,"&lt;&gt;Fermer"))))</f>
       </c>
       <c r="T28" s="75">
-        <f>IF($R28="Fermer","",$J28-$K28-$S28)</f>
+        <f>IF(OR($C28="",COUNT($H28:$Q28)=0),"",IF($R28="Fermer","",$J28-$K28-$S28))</f>
       </c>
       <c r="U28" s="74">
-        <f>IF($R28="Fermer",-$L28,0)</f>
+        <f>IF(OR($C28="",COUNT($H28:$Q28)=0),"",IF($R28="Fermer",-$L28,0))</f>
       </c>
       <c r="V28" s="76">
-        <f>IF($R28="Fermer","Fermer = perdre "&amp;TEXT($L28,"#,##0")&amp;" € de contribution. Le fixe, lui, reste.",IF(AND($O28&gt;=0,$T28&lt;0),"BASCULE : saine avant, en déficit à cause d'une fermeture voisine.",IF(AND($O28&lt;0,$L28&gt;0),"Déficit au coût complet mais contribution positive : ne pas fermer, c'est un artefact d'allocation.",IF($O28&lt;0,"Contribution négative : vrai point dur.","Rentable. Point mort "&amp;TEXT($P28,"#,##0")&amp;" étudiants, marge de sécurité "&amp;TEXT($Q28,"0%")&amp;"."))))</f>
+        <f>IF(OR($C28="",COUNT($H28:$Q28)=0),"",IF($R28="Fermer","Fermer = perdre "&amp;TEXT($L28,"#,##0")&amp;" € de contribution. Le fixe, lui, reste.",IF(AND($O28&gt;=0,$T28&lt;0),"BASCULE : saine avant, en déficit à cause d'une fermeture voisine.",IF(AND($O28&lt;0,$L28&gt;0),"Déficit au coût complet mais contribution positive : ne pas fermer, c'est un artefact d'allocation.",IF($O28&lt;0,"Contribution négative : vrai point dur.","Rentable. Point mort "&amp;TEXT($P28,"#,##0")&amp;" étudiants, marge de sécurité "&amp;TEXT($Q28,"0%")&amp;".")))))</f>
       </c>
     </row>
     <row r="29" ht="14.25" customHeight="1">
@@ -12905,16 +12905,16 @@
         <v>115</v>
       </c>
       <c r="S29" s="74">
-        <f>IF($R29="Fermer","",IF(SUMIFS($I$13:$I$72,$C$13:$C$72,$C29,$D$13:$D$72,$D29,$R$13:$R$72,"&lt;&gt;Fermer")=0,$M29,$M29+SUMIFS($M$13:$M$72,$C$13:$C$72,$C29,$D$13:$D$72,$D29,$R$13:$R$72,"Fermer")*$I29/SUMIFS($I$13:$I$72,$C$13:$C$72,$C29,$D$13:$D$72,$D29,$R$13:$R$72,"&lt;&gt;Fermer")))</f>
+        <f>IF(OR($C29="",COUNT($H29:$Q29)=0),"",IF($R29="Fermer","",IF(SUMIFS($I$13:$I$72,$C$13:$C$72,$C29,$D$13:$D$72,$D29,$R$13:$R$72,"&lt;&gt;Fermer")=0,$M29,$M29+SUMIFS($M$13:$M$72,$C$13:$C$72,$C29,$D$13:$D$72,$D29,$R$13:$R$72,"Fermer")*$I29/SUMIFS($I$13:$I$72,$C$13:$C$72,$C29,$D$13:$D$72,$D29,$R$13:$R$72,"&lt;&gt;Fermer"))))</f>
       </c>
       <c r="T29" s="75">
-        <f>IF($R29="Fermer","",$J29-$K29-$S29)</f>
+        <f>IF(OR($C29="",COUNT($H29:$Q29)=0),"",IF($R29="Fermer","",$J29-$K29-$S29))</f>
       </c>
       <c r="U29" s="74">
-        <f>IF($R29="Fermer",-$L29,0)</f>
+        <f>IF(OR($C29="",COUNT($H29:$Q29)=0),"",IF($R29="Fermer",-$L29,0))</f>
       </c>
       <c r="V29" s="76">
-        <f>IF($R29="Fermer","Fermer = perdre "&amp;TEXT($L29,"#,##0")&amp;" € de contribution. Le fixe, lui, reste.",IF(AND($O29&gt;=0,$T29&lt;0),"BASCULE : saine avant, en déficit à cause d'une fermeture voisine.",IF(AND($O29&lt;0,$L29&gt;0),"Déficit au coût complet mais contribution positive : ne pas fermer, c'est un artefact d'allocation.",IF($O29&lt;0,"Contribution négative : vrai point dur.","Rentable. Point mort "&amp;TEXT($P29,"#,##0")&amp;" étudiants, marge de sécurité "&amp;TEXT($Q29,"0%")&amp;"."))))</f>
+        <f>IF(OR($C29="",COUNT($H29:$Q29)=0),"",IF($R29="Fermer","Fermer = perdre "&amp;TEXT($L29,"#,##0")&amp;" € de contribution. Le fixe, lui, reste.",IF(AND($O29&gt;=0,$T29&lt;0),"BASCULE : saine avant, en déficit à cause d'une fermeture voisine.",IF(AND($O29&lt;0,$L29&gt;0),"Déficit au coût complet mais contribution positive : ne pas fermer, c'est un artefact d'allocation.",IF($O29&lt;0,"Contribution négative : vrai point dur.","Rentable. Point mort "&amp;TEXT($P29,"#,##0")&amp;" étudiants, marge de sécurité "&amp;TEXT($Q29,"0%")&amp;".")))))</f>
       </c>
     </row>
     <row r="30" ht="14.25" customHeight="1">
@@ -12967,16 +12967,16 @@
         <v>112</v>
       </c>
       <c r="S30" s="74">
-        <f>IF($R30="Fermer","",IF(SUMIFS($I$13:$I$72,$C$13:$C$72,$C30,$D$13:$D$72,$D30,$R$13:$R$72,"&lt;&gt;Fermer")=0,$M30,$M30+SUMIFS($M$13:$M$72,$C$13:$C$72,$C30,$D$13:$D$72,$D30,$R$13:$R$72,"Fermer")*$I30/SUMIFS($I$13:$I$72,$C$13:$C$72,$C30,$D$13:$D$72,$D30,$R$13:$R$72,"&lt;&gt;Fermer")))</f>
+        <f>IF(OR($C30="",COUNT($H30:$Q30)=0),"",IF($R30="Fermer","",IF(SUMIFS($I$13:$I$72,$C$13:$C$72,$C30,$D$13:$D$72,$D30,$R$13:$R$72,"&lt;&gt;Fermer")=0,$M30,$M30+SUMIFS($M$13:$M$72,$C$13:$C$72,$C30,$D$13:$D$72,$D30,$R$13:$R$72,"Fermer")*$I30/SUMIFS($I$13:$I$72,$C$13:$C$72,$C30,$D$13:$D$72,$D30,$R$13:$R$72,"&lt;&gt;Fermer"))))</f>
       </c>
       <c r="T30" s="75">
-        <f>IF($R30="Fermer","",$J30-$K30-$S30)</f>
+        <f>IF(OR($C30="",COUNT($H30:$Q30)=0),"",IF($R30="Fermer","",$J30-$K30-$S30))</f>
       </c>
       <c r="U30" s="74">
-        <f>IF($R30="Fermer",-$L30,0)</f>
+        <f>IF(OR($C30="",COUNT($H30:$Q30)=0),"",IF($R30="Fermer",-$L30,0))</f>
       </c>
       <c r="V30" s="76">
-        <f>IF($R30="Fermer","Fermer = perdre "&amp;TEXT($L30,"#,##0")&amp;" € de contribution. Le fixe, lui, reste.",IF(AND($O30&gt;=0,$T30&lt;0),"BASCULE : saine avant, en déficit à cause d'une fermeture voisine.",IF(AND($O30&lt;0,$L30&gt;0),"Déficit au coût complet mais contribution positive : ne pas fermer, c'est un artefact d'allocation.",IF($O30&lt;0,"Contribution négative : vrai point dur.","Rentable. Point mort "&amp;TEXT($P30,"#,##0")&amp;" étudiants, marge de sécurité "&amp;TEXT($Q30,"0%")&amp;"."))))</f>
+        <f>IF(OR($C30="",COUNT($H30:$Q30)=0),"",IF($R30="Fermer","Fermer = perdre "&amp;TEXT($L30,"#,##0")&amp;" € de contribution. Le fixe, lui, reste.",IF(AND($O30&gt;=0,$T30&lt;0),"BASCULE : saine avant, en déficit à cause d'une fermeture voisine.",IF(AND($O30&lt;0,$L30&gt;0),"Déficit au coût complet mais contribution positive : ne pas fermer, c'est un artefact d'allocation.",IF($O30&lt;0,"Contribution négative : vrai point dur.","Rentable. Point mort "&amp;TEXT($P30,"#,##0")&amp;" étudiants, marge de sécurité "&amp;TEXT($Q30,"0%")&amp;".")))))</f>
       </c>
     </row>
     <row r="31" ht="14.25" customHeight="1">
@@ -13029,16 +13029,16 @@
         <v>115</v>
       </c>
       <c r="S31" s="74">
-        <f>IF($R31="Fermer","",IF(SUMIFS($I$13:$I$72,$C$13:$C$72,$C31,$D$13:$D$72,$D31,$R$13:$R$72,"&lt;&gt;Fermer")=0,$M31,$M31+SUMIFS($M$13:$M$72,$C$13:$C$72,$C31,$D$13:$D$72,$D31,$R$13:$R$72,"Fermer")*$I31/SUMIFS($I$13:$I$72,$C$13:$C$72,$C31,$D$13:$D$72,$D31,$R$13:$R$72,"&lt;&gt;Fermer")))</f>
+        <f>IF(OR($C31="",COUNT($H31:$Q31)=0),"",IF($R31="Fermer","",IF(SUMIFS($I$13:$I$72,$C$13:$C$72,$C31,$D$13:$D$72,$D31,$R$13:$R$72,"&lt;&gt;Fermer")=0,$M31,$M31+SUMIFS($M$13:$M$72,$C$13:$C$72,$C31,$D$13:$D$72,$D31,$R$13:$R$72,"Fermer")*$I31/SUMIFS($I$13:$I$72,$C$13:$C$72,$C31,$D$13:$D$72,$D31,$R$13:$R$72,"&lt;&gt;Fermer"))))</f>
       </c>
       <c r="T31" s="75">
-        <f>IF($R31="Fermer","",$J31-$K31-$S31)</f>
+        <f>IF(OR($C31="",COUNT($H31:$Q31)=0),"",IF($R31="Fermer","",$J31-$K31-$S31))</f>
       </c>
       <c r="U31" s="74">
-        <f>IF($R31="Fermer",-$L31,0)</f>
+        <f>IF(OR($C31="",COUNT($H31:$Q31)=0),"",IF($R31="Fermer",-$L31,0))</f>
       </c>
       <c r="V31" s="76">
-        <f>IF($R31="Fermer","Fermer = perdre "&amp;TEXT($L31,"#,##0")&amp;" € de contribution. Le fixe, lui, reste.",IF(AND($O31&gt;=0,$T31&lt;0),"BASCULE : saine avant, en déficit à cause d'une fermeture voisine.",IF(AND($O31&lt;0,$L31&gt;0),"Déficit au coût complet mais contribution positive : ne pas fermer, c'est un artefact d'allocation.",IF($O31&lt;0,"Contribution négative : vrai point dur.","Rentable. Point mort "&amp;TEXT($P31,"#,##0")&amp;" étudiants, marge de sécurité "&amp;TEXT($Q31,"0%")&amp;"."))))</f>
+        <f>IF(OR($C31="",COUNT($H31:$Q31)=0),"",IF($R31="Fermer","Fermer = perdre "&amp;TEXT($L31,"#,##0")&amp;" € de contribution. Le fixe, lui, reste.",IF(AND($O31&gt;=0,$T31&lt;0),"BASCULE : saine avant, en déficit à cause d'une fermeture voisine.",IF(AND($O31&lt;0,$L31&gt;0),"Déficit au coût complet mais contribution positive : ne pas fermer, c'est un artefact d'allocation.",IF($O31&lt;0,"Contribution négative : vrai point dur.","Rentable. Point mort "&amp;TEXT($P31,"#,##0")&amp;" étudiants, marge de sécurité "&amp;TEXT($Q31,"0%")&amp;".")))))</f>
       </c>
     </row>
     <row r="32" ht="14.25" customHeight="1">
@@ -13091,16 +13091,16 @@
         <v>112</v>
       </c>
       <c r="S32" s="74">
-        <f>IF($R32="Fermer","",IF(SUMIFS($I$13:$I$72,$C$13:$C$72,$C32,$D$13:$D$72,$D32,$R$13:$R$72,"&lt;&gt;Fermer")=0,$M32,$M32+SUMIFS($M$13:$M$72,$C$13:$C$72,$C32,$D$13:$D$72,$D32,$R$13:$R$72,"Fermer")*$I32/SUMIFS($I$13:$I$72,$C$13:$C$72,$C32,$D$13:$D$72,$D32,$R$13:$R$72,"&lt;&gt;Fermer")))</f>
+        <f>IF(OR($C32="",COUNT($H32:$Q32)=0),"",IF($R32="Fermer","",IF(SUMIFS($I$13:$I$72,$C$13:$C$72,$C32,$D$13:$D$72,$D32,$R$13:$R$72,"&lt;&gt;Fermer")=0,$M32,$M32+SUMIFS($M$13:$M$72,$C$13:$C$72,$C32,$D$13:$D$72,$D32,$R$13:$R$72,"Fermer")*$I32/SUMIFS($I$13:$I$72,$C$13:$C$72,$C32,$D$13:$D$72,$D32,$R$13:$R$72,"&lt;&gt;Fermer"))))</f>
       </c>
       <c r="T32" s="75">
-        <f>IF($R32="Fermer","",$J32-$K32-$S32)</f>
+        <f>IF(OR($C32="",COUNT($H32:$Q32)=0),"",IF($R32="Fermer","",$J32-$K32-$S32))</f>
       </c>
       <c r="U32" s="74">
-        <f>IF($R32="Fermer",-$L32,0)</f>
+        <f>IF(OR($C32="",COUNT($H32:$Q32)=0),"",IF($R32="Fermer",-$L32,0))</f>
       </c>
       <c r="V32" s="76">
-        <f>IF($R32="Fermer","Fermer = perdre "&amp;TEXT($L32,"#,##0")&amp;" € de contribution. Le fixe, lui, reste.",IF(AND($O32&gt;=0,$T32&lt;0),"BASCULE : saine avant, en déficit à cause d'une fermeture voisine.",IF(AND($O32&lt;0,$L32&gt;0),"Déficit au coût complet mais contribution positive : ne pas fermer, c'est un artefact d'allocation.",IF($O32&lt;0,"Contribution négative : vrai point dur.","Rentable. Point mort "&amp;TEXT($P32,"#,##0")&amp;" étudiants, marge de sécurité "&amp;TEXT($Q32,"0%")&amp;"."))))</f>
+        <f>IF(OR($C32="",COUNT($H32:$Q32)=0),"",IF($R32="Fermer","Fermer = perdre "&amp;TEXT($L32,"#,##0")&amp;" € de contribution. Le fixe, lui, reste.",IF(AND($O32&gt;=0,$T32&lt;0),"BASCULE : saine avant, en déficit à cause d'une fermeture voisine.",IF(AND($O32&lt;0,$L32&gt;0),"Déficit au coût complet mais contribution positive : ne pas fermer, c'est un artefact d'allocation.",IF($O32&lt;0,"Contribution négative : vrai point dur.","Rentable. Point mort "&amp;TEXT($P32,"#,##0")&amp;" étudiants, marge de sécurité "&amp;TEXT($Q32,"0%")&amp;".")))))</f>
       </c>
     </row>
     <row r="33" ht="14.25" customHeight="1">
@@ -13153,16 +13153,16 @@
         <v>115</v>
       </c>
       <c r="S33" s="74">
-        <f>IF($R33="Fermer","",IF(SUMIFS($I$13:$I$72,$C$13:$C$72,$C33,$D$13:$D$72,$D33,$R$13:$R$72,"&lt;&gt;Fermer")=0,$M33,$M33+SUMIFS($M$13:$M$72,$C$13:$C$72,$C33,$D$13:$D$72,$D33,$R$13:$R$72,"Fermer")*$I33/SUMIFS($I$13:$I$72,$C$13:$C$72,$C33,$D$13:$D$72,$D33,$R$13:$R$72,"&lt;&gt;Fermer")))</f>
+        <f>IF(OR($C33="",COUNT($H33:$Q33)=0),"",IF($R33="Fermer","",IF(SUMIFS($I$13:$I$72,$C$13:$C$72,$C33,$D$13:$D$72,$D33,$R$13:$R$72,"&lt;&gt;Fermer")=0,$M33,$M33+SUMIFS($M$13:$M$72,$C$13:$C$72,$C33,$D$13:$D$72,$D33,$R$13:$R$72,"Fermer")*$I33/SUMIFS($I$13:$I$72,$C$13:$C$72,$C33,$D$13:$D$72,$D33,$R$13:$R$72,"&lt;&gt;Fermer"))))</f>
       </c>
       <c r="T33" s="75">
-        <f>IF($R33="Fermer","",$J33-$K33-$S33)</f>
+        <f>IF(OR($C33="",COUNT($H33:$Q33)=0),"",IF($R33="Fermer","",$J33-$K33-$S33))</f>
       </c>
       <c r="U33" s="74">
-        <f>IF($R33="Fermer",-$L33,0)</f>
+        <f>IF(OR($C33="",COUNT($H33:$Q33)=0),"",IF($R33="Fermer",-$L33,0))</f>
       </c>
       <c r="V33" s="76">
-        <f>IF($R33="Fermer","Fermer = perdre "&amp;TEXT($L33,"#,##0")&amp;" € de contribution. Le fixe, lui, reste.",IF(AND($O33&gt;=0,$T33&lt;0),"BASCULE : saine avant, en déficit à cause d'une fermeture voisine.",IF(AND($O33&lt;0,$L33&gt;0),"Déficit au coût complet mais contribution positive : ne pas fermer, c'est un artefact d'allocation.",IF($O33&lt;0,"Contribution négative : vrai point dur.","Rentable. Point mort "&amp;TEXT($P33,"#,##0")&amp;" étudiants, marge de sécurité "&amp;TEXT($Q33,"0%")&amp;"."))))</f>
+        <f>IF(OR($C33="",COUNT($H33:$Q33)=0),"",IF($R33="Fermer","Fermer = perdre "&amp;TEXT($L33,"#,##0")&amp;" € de contribution. Le fixe, lui, reste.",IF(AND($O33&gt;=0,$T33&lt;0),"BASCULE : saine avant, en déficit à cause d'une fermeture voisine.",IF(AND($O33&lt;0,$L33&gt;0),"Déficit au coût complet mais contribution positive : ne pas fermer, c'est un artefact d'allocation.",IF($O33&lt;0,"Contribution négative : vrai point dur.","Rentable. Point mort "&amp;TEXT($P33,"#,##0")&amp;" étudiants, marge de sécurité "&amp;TEXT($Q33,"0%")&amp;".")))))</f>
       </c>
     </row>
     <row r="34" ht="14.25" customHeight="1">
@@ -13215,16 +13215,16 @@
         <v>115</v>
       </c>
       <c r="S34" s="74">
-        <f>IF($R34="Fermer","",IF(SUMIFS($I$13:$I$72,$C$13:$C$72,$C34,$D$13:$D$72,$D34,$R$13:$R$72,"&lt;&gt;Fermer")=0,$M34,$M34+SUMIFS($M$13:$M$72,$C$13:$C$72,$C34,$D$13:$D$72,$D34,$R$13:$R$72,"Fermer")*$I34/SUMIFS($I$13:$I$72,$C$13:$C$72,$C34,$D$13:$D$72,$D34,$R$13:$R$72,"&lt;&gt;Fermer")))</f>
+        <f>IF(OR($C34="",COUNT($H34:$Q34)=0),"",IF($R34="Fermer","",IF(SUMIFS($I$13:$I$72,$C$13:$C$72,$C34,$D$13:$D$72,$D34,$R$13:$R$72,"&lt;&gt;Fermer")=0,$M34,$M34+SUMIFS($M$13:$M$72,$C$13:$C$72,$C34,$D$13:$D$72,$D34,$R$13:$R$72,"Fermer")*$I34/SUMIFS($I$13:$I$72,$C$13:$C$72,$C34,$D$13:$D$72,$D34,$R$13:$R$72,"&lt;&gt;Fermer"))))</f>
       </c>
       <c r="T34" s="75">
-        <f>IF($R34="Fermer","",$J34-$K34-$S34)</f>
+        <f>IF(OR($C34="",COUNT($H34:$Q34)=0),"",IF($R34="Fermer","",$J34-$K34-$S34))</f>
       </c>
       <c r="U34" s="74">
-        <f>IF($R34="Fermer",-$L34,0)</f>
+        <f>IF(OR($C34="",COUNT($H34:$Q34)=0),"",IF($R34="Fermer",-$L34,0))</f>
       </c>
       <c r="V34" s="76">
-        <f>IF($R34="Fermer","Fermer = perdre "&amp;TEXT($L34,"#,##0")&amp;" € de contribution. Le fixe, lui, reste.",IF(AND($O34&gt;=0,$T34&lt;0),"BASCULE : saine avant, en déficit à cause d'une fermeture voisine.",IF(AND($O34&lt;0,$L34&gt;0),"Déficit au coût complet mais contribution positive : ne pas fermer, c'est un artefact d'allocation.",IF($O34&lt;0,"Contribution négative : vrai point dur.","Rentable. Point mort "&amp;TEXT($P34,"#,##0")&amp;" étudiants, marge de sécurité "&amp;TEXT($Q34,"0%")&amp;"."))))</f>
+        <f>IF(OR($C34="",COUNT($H34:$Q34)=0),"",IF($R34="Fermer","Fermer = perdre "&amp;TEXT($L34,"#,##0")&amp;" € de contribution. Le fixe, lui, reste.",IF(AND($O34&gt;=0,$T34&lt;0),"BASCULE : saine avant, en déficit à cause d'une fermeture voisine.",IF(AND($O34&lt;0,$L34&gt;0),"Déficit au coût complet mais contribution positive : ne pas fermer, c'est un artefact d'allocation.",IF($O34&lt;0,"Contribution négative : vrai point dur.","Rentable. Point mort "&amp;TEXT($P34,"#,##0")&amp;" étudiants, marge de sécurité "&amp;TEXT($Q34,"0%")&amp;".")))))</f>
       </c>
     </row>
     <row r="35" ht="14.25" customHeight="1">
@@ -13277,16 +13277,16 @@
         <v>112</v>
       </c>
       <c r="S35" s="74">
-        <f>IF($R35="Fermer","",IF(SUMIFS($I$13:$I$72,$C$13:$C$72,$C35,$D$13:$D$72,$D35,$R$13:$R$72,"&lt;&gt;Fermer")=0,$M35,$M35+SUMIFS($M$13:$M$72,$C$13:$C$72,$C35,$D$13:$D$72,$D35,$R$13:$R$72,"Fermer")*$I35/SUMIFS($I$13:$I$72,$C$13:$C$72,$C35,$D$13:$D$72,$D35,$R$13:$R$72,"&lt;&gt;Fermer")))</f>
+        <f>IF(OR($C35="",COUNT($H35:$Q35)=0),"",IF($R35="Fermer","",IF(SUMIFS($I$13:$I$72,$C$13:$C$72,$C35,$D$13:$D$72,$D35,$R$13:$R$72,"&lt;&gt;Fermer")=0,$M35,$M35+SUMIFS($M$13:$M$72,$C$13:$C$72,$C35,$D$13:$D$72,$D35,$R$13:$R$72,"Fermer")*$I35/SUMIFS($I$13:$I$72,$C$13:$C$72,$C35,$D$13:$D$72,$D35,$R$13:$R$72,"&lt;&gt;Fermer"))))</f>
       </c>
       <c r="T35" s="75">
-        <f>IF($R35="Fermer","",$J35-$K35-$S35)</f>
+        <f>IF(OR($C35="",COUNT($H35:$Q35)=0),"",IF($R35="Fermer","",$J35-$K35-$S35))</f>
       </c>
       <c r="U35" s="74">
-        <f>IF($R35="Fermer",-$L35,0)</f>
+        <f>IF(OR($C35="",COUNT($H35:$Q35)=0),"",IF($R35="Fermer",-$L35,0))</f>
       </c>
       <c r="V35" s="76">
-        <f>IF($R35="Fermer","Fermer = perdre "&amp;TEXT($L35,"#,##0")&amp;" € de contribution. Le fixe, lui, reste.",IF(AND($O35&gt;=0,$T35&lt;0),"BASCULE : saine avant, en déficit à cause d'une fermeture voisine.",IF(AND($O35&lt;0,$L35&gt;0),"Déficit au coût complet mais contribution positive : ne pas fermer, c'est un artefact d'allocation.",IF($O35&lt;0,"Contribution négative : vrai point dur.","Rentable. Point mort "&amp;TEXT($P35,"#,##0")&amp;" étudiants, marge de sécurité "&amp;TEXT($Q35,"0%")&amp;"."))))</f>
+        <f>IF(OR($C35="",COUNT($H35:$Q35)=0),"",IF($R35="Fermer","Fermer = perdre "&amp;TEXT($L35,"#,##0")&amp;" € de contribution. Le fixe, lui, reste.",IF(AND($O35&gt;=0,$T35&lt;0),"BASCULE : saine avant, en déficit à cause d'une fermeture voisine.",IF(AND($O35&lt;0,$L35&gt;0),"Déficit au coût complet mais contribution positive : ne pas fermer, c'est un artefact d'allocation.",IF($O35&lt;0,"Contribution négative : vrai point dur.","Rentable. Point mort "&amp;TEXT($P35,"#,##0")&amp;" étudiants, marge de sécurité "&amp;TEXT($Q35,"0%")&amp;".")))))</f>
       </c>
     </row>
     <row r="36" ht="14.25" customHeight="1">
@@ -13339,16 +13339,16 @@
         <v>115</v>
       </c>
       <c r="S36" s="74">
-        <f>IF($R36="Fermer","",IF(SUMIFS($I$13:$I$72,$C$13:$C$72,$C36,$D$13:$D$72,$D36,$R$13:$R$72,"&lt;&gt;Fermer")=0,$M36,$M36+SUMIFS($M$13:$M$72,$C$13:$C$72,$C36,$D$13:$D$72,$D36,$R$13:$R$72,"Fermer")*$I36/SUMIFS($I$13:$I$72,$C$13:$C$72,$C36,$D$13:$D$72,$D36,$R$13:$R$72,"&lt;&gt;Fermer")))</f>
+        <f>IF(OR($C36="",COUNT($H36:$Q36)=0),"",IF($R36="Fermer","",IF(SUMIFS($I$13:$I$72,$C$13:$C$72,$C36,$D$13:$D$72,$D36,$R$13:$R$72,"&lt;&gt;Fermer")=0,$M36,$M36+SUMIFS($M$13:$M$72,$C$13:$C$72,$C36,$D$13:$D$72,$D36,$R$13:$R$72,"Fermer")*$I36/SUMIFS($I$13:$I$72,$C$13:$C$72,$C36,$D$13:$D$72,$D36,$R$13:$R$72,"&lt;&gt;Fermer"))))</f>
       </c>
       <c r="T36" s="75">
-        <f>IF($R36="Fermer","",$J36-$K36-$S36)</f>
+        <f>IF(OR($C36="",COUNT($H36:$Q36)=0),"",IF($R36="Fermer","",$J36-$K36-$S36))</f>
       </c>
       <c r="U36" s="74">
-        <f>IF($R36="Fermer",-$L36,0)</f>
+        <f>IF(OR($C36="",COUNT($H36:$Q36)=0),"",IF($R36="Fermer",-$L36,0))</f>
       </c>
       <c r="V36" s="76">
-        <f>IF($R36="Fermer","Fermer = perdre "&amp;TEXT($L36,"#,##0")&amp;" € de contribution. Le fixe, lui, reste.",IF(AND($O36&gt;=0,$T36&lt;0),"BASCULE : saine avant, en déficit à cause d'une fermeture voisine.",IF(AND($O36&lt;0,$L36&gt;0),"Déficit au coût complet mais contribution positive : ne pas fermer, c'est un artefact d'allocation.",IF($O36&lt;0,"Contribution négative : vrai point dur.","Rentable. Point mort "&amp;TEXT($P36,"#,##0")&amp;" étudiants, marge de sécurité "&amp;TEXT($Q36,"0%")&amp;"."))))</f>
+        <f>IF(OR($C36="",COUNT($H36:$Q36)=0),"",IF($R36="Fermer","Fermer = perdre "&amp;TEXT($L36,"#,##0")&amp;" € de contribution. Le fixe, lui, reste.",IF(AND($O36&gt;=0,$T36&lt;0),"BASCULE : saine avant, en déficit à cause d'une fermeture voisine.",IF(AND($O36&lt;0,$L36&gt;0),"Déficit au coût complet mais contribution positive : ne pas fermer, c'est un artefact d'allocation.",IF($O36&lt;0,"Contribution négative : vrai point dur.","Rentable. Point mort "&amp;TEXT($P36,"#,##0")&amp;" étudiants, marge de sécurité "&amp;TEXT($Q36,"0%")&amp;".")))))</f>
       </c>
     </row>
     <row r="37" ht="14.25" customHeight="1">
@@ -13401,16 +13401,16 @@
         <v>112</v>
       </c>
       <c r="S37" s="74">
-        <f>IF($R37="Fermer","",IF(SUMIFS($I$13:$I$72,$C$13:$C$72,$C37,$D$13:$D$72,$D37,$R$13:$R$72,"&lt;&gt;Fermer")=0,$M37,$M37+SUMIFS($M$13:$M$72,$C$13:$C$72,$C37,$D$13:$D$72,$D37,$R$13:$R$72,"Fermer")*$I37/SUMIFS($I$13:$I$72,$C$13:$C$72,$C37,$D$13:$D$72,$D37,$R$13:$R$72,"&lt;&gt;Fermer")))</f>
+        <f>IF(OR($C37="",COUNT($H37:$Q37)=0),"",IF($R37="Fermer","",IF(SUMIFS($I$13:$I$72,$C$13:$C$72,$C37,$D$13:$D$72,$D37,$R$13:$R$72,"&lt;&gt;Fermer")=0,$M37,$M37+SUMIFS($M$13:$M$72,$C$13:$C$72,$C37,$D$13:$D$72,$D37,$R$13:$R$72,"Fermer")*$I37/SUMIFS($I$13:$I$72,$C$13:$C$72,$C37,$D$13:$D$72,$D37,$R$13:$R$72,"&lt;&gt;Fermer"))))</f>
       </c>
       <c r="T37" s="75">
-        <f>IF($R37="Fermer","",$J37-$K37-$S37)</f>
+        <f>IF(OR($C37="",COUNT($H37:$Q37)=0),"",IF($R37="Fermer","",$J37-$K37-$S37))</f>
       </c>
       <c r="U37" s="74">
-        <f>IF($R37="Fermer",-$L37,0)</f>
+        <f>IF(OR($C37="",COUNT($H37:$Q37)=0),"",IF($R37="Fermer",-$L37,0))</f>
       </c>
       <c r="V37" s="76">
-        <f>IF($R37="Fermer","Fermer = perdre "&amp;TEXT($L37,"#,##0")&amp;" € de contribution. Le fixe, lui, reste.",IF(AND($O37&gt;=0,$T37&lt;0),"BASCULE : saine avant, en déficit à cause d'une fermeture voisine.",IF(AND($O37&lt;0,$L37&gt;0),"Déficit au coût complet mais contribution positive : ne pas fermer, c'est un artefact d'allocation.",IF($O37&lt;0,"Contribution négative : vrai point dur.","Rentable. Point mort "&amp;TEXT($P37,"#,##0")&amp;" étudiants, marge de sécurité "&amp;TEXT($Q37,"0%")&amp;"."))))</f>
+        <f>IF(OR($C37="",COUNT($H37:$Q37)=0),"",IF($R37="Fermer","Fermer = perdre "&amp;TEXT($L37,"#,##0")&amp;" € de contribution. Le fixe, lui, reste.",IF(AND($O37&gt;=0,$T37&lt;0),"BASCULE : saine avant, en déficit à cause d'une fermeture voisine.",IF(AND($O37&lt;0,$L37&gt;0),"Déficit au coût complet mais contribution positive : ne pas fermer, c'est un artefact d'allocation.",IF($O37&lt;0,"Contribution négative : vrai point dur.","Rentable. Point mort "&amp;TEXT($P37,"#,##0")&amp;" étudiants, marge de sécurité "&amp;TEXT($Q37,"0%")&amp;".")))))</f>
       </c>
     </row>
     <row r="38" ht="14.25" customHeight="1">
@@ -13464,16 +13464,16 @@
         <v>115</v>
       </c>
       <c r="S38" s="74">
-        <f>IF($R38="Fermer","",IF(SUMIFS($I$13:$I$72,$C$13:$C$72,$C38,$D$13:$D$72,$D38,$R$13:$R$72,"&lt;&gt;Fermer")=0,$M38,$M38+SUMIFS($M$13:$M$72,$C$13:$C$72,$C38,$D$13:$D$72,$D38,$R$13:$R$72,"Fermer")*$I38/SUMIFS($I$13:$I$72,$C$13:$C$72,$C38,$D$13:$D$72,$D38,$R$13:$R$72,"&lt;&gt;Fermer")))</f>
+        <f>IF(OR($C38="",COUNT($H38:$Q38)=0),"",IF($R38="Fermer","",IF(SUMIFS($I$13:$I$72,$C$13:$C$72,$C38,$D$13:$D$72,$D38,$R$13:$R$72,"&lt;&gt;Fermer")=0,$M38,$M38+SUMIFS($M$13:$M$72,$C$13:$C$72,$C38,$D$13:$D$72,$D38,$R$13:$R$72,"Fermer")*$I38/SUMIFS($I$13:$I$72,$C$13:$C$72,$C38,$D$13:$D$72,$D38,$R$13:$R$72,"&lt;&gt;Fermer"))))</f>
       </c>
       <c r="T38" s="75">
-        <f>IF($R38="Fermer","",$J38-$K38-$S38)</f>
+        <f>IF(OR($C38="",COUNT($H38:$Q38)=0),"",IF($R38="Fermer","",$J38-$K38-$S38))</f>
       </c>
       <c r="U38" s="74">
-        <f>IF($R38="Fermer",-$L38,0)</f>
+        <f>IF(OR($C38="",COUNT($H38:$Q38)=0),"",IF($R38="Fermer",-$L38,0))</f>
       </c>
       <c r="V38" s="76">
-        <f>IF($R38="Fermer","Fermer = perdre "&amp;TEXT($L38,"#,##0")&amp;" € de contribution. Le fixe, lui, reste.",IF(AND($O38&gt;=0,$T38&lt;0),"BASCULE : saine avant, en déficit à cause d'une fermeture voisine.",IF(AND($O38&lt;0,$L38&gt;0),"Déficit au coût complet mais contribution positive : ne pas fermer, c'est un artefact d'allocation.",IF($O38&lt;0,"Contribution négative : vrai point dur.","Rentable. Point mort "&amp;TEXT($P38,"#,##0")&amp;" étudiants, marge de sécurité "&amp;TEXT($Q38,"0%")&amp;"."))))</f>
+        <f>IF(OR($C38="",COUNT($H38:$Q38)=0),"",IF($R38="Fermer","Fermer = perdre "&amp;TEXT($L38,"#,##0")&amp;" € de contribution. Le fixe, lui, reste.",IF(AND($O38&gt;=0,$T38&lt;0),"BASCULE : saine avant, en déficit à cause d'une fermeture voisine.",IF(AND($O38&lt;0,$L38&gt;0),"Déficit au coût complet mais contribution positive : ne pas fermer, c'est un artefact d'allocation.",IF($O38&lt;0,"Contribution négative : vrai point dur.","Rentable. Point mort "&amp;TEXT($P38,"#,##0")&amp;" étudiants, marge de sécurité "&amp;TEXT($Q38,"0%")&amp;".")))))</f>
       </c>
       <c r="W38" s="47"/>
       <c r="X38" s="47"/>
@@ -13536,16 +13536,16 @@
         <v>115</v>
       </c>
       <c r="S39" s="74">
-        <f>IF($R39="Fermer","",IF(SUMIFS($I$13:$I$72,$C$13:$C$72,$C39,$D$13:$D$72,$D39,$R$13:$R$72,"&lt;&gt;Fermer")=0,$M39,$M39+SUMIFS($M$13:$M$72,$C$13:$C$72,$C39,$D$13:$D$72,$D39,$R$13:$R$72,"Fermer")*$I39/SUMIFS($I$13:$I$72,$C$13:$C$72,$C39,$D$13:$D$72,$D39,$R$13:$R$72,"&lt;&gt;Fermer")))</f>
+        <f>IF(OR($C39="",COUNT($H39:$Q39)=0),"",IF($R39="Fermer","",IF(SUMIFS($I$13:$I$72,$C$13:$C$72,$C39,$D$13:$D$72,$D39,$R$13:$R$72,"&lt;&gt;Fermer")=0,$M39,$M39+SUMIFS($M$13:$M$72,$C$13:$C$72,$C39,$D$13:$D$72,$D39,$R$13:$R$72,"Fermer")*$I39/SUMIFS($I$13:$I$72,$C$13:$C$72,$C39,$D$13:$D$72,$D39,$R$13:$R$72,"&lt;&gt;Fermer"))))</f>
       </c>
       <c r="T39" s="75">
-        <f>IF($R39="Fermer","",$J39-$K39-$S39)</f>
+        <f>IF(OR($C39="",COUNT($H39:$Q39)=0),"",IF($R39="Fermer","",$J39-$K39-$S39))</f>
       </c>
       <c r="U39" s="74">
-        <f>IF($R39="Fermer",-$L39,0)</f>
+        <f>IF(OR($C39="",COUNT($H39:$Q39)=0),"",IF($R39="Fermer",-$L39,0))</f>
       </c>
       <c r="V39" s="76">
-        <f>IF($R39="Fermer","Fermer = perdre "&amp;TEXT($L39,"#,##0")&amp;" € de contribution. Le fixe, lui, reste.",IF(AND($O39&gt;=0,$T39&lt;0),"BASCULE : saine avant, en déficit à cause d'une fermeture voisine.",IF(AND($O39&lt;0,$L39&gt;0),"Déficit au coût complet mais contribution positive : ne pas fermer, c'est un artefact d'allocation.",IF($O39&lt;0,"Contribution négative : vrai point dur.","Rentable. Point mort "&amp;TEXT($P39,"#,##0")&amp;" étudiants, marge de sécurité "&amp;TEXT($Q39,"0%")&amp;"."))))</f>
+        <f>IF(OR($C39="",COUNT($H39:$Q39)=0),"",IF($R39="Fermer","Fermer = perdre "&amp;TEXT($L39,"#,##0")&amp;" € de contribution. Le fixe, lui, reste.",IF(AND($O39&gt;=0,$T39&lt;0),"BASCULE : saine avant, en déficit à cause d'une fermeture voisine.",IF(AND($O39&lt;0,$L39&gt;0),"Déficit au coût complet mais contribution positive : ne pas fermer, c'est un artefact d'allocation.",IF($O39&lt;0,"Contribution négative : vrai point dur.","Rentable. Point mort "&amp;TEXT($P39,"#,##0")&amp;" étudiants, marge de sécurité "&amp;TEXT($Q39,"0%")&amp;".")))))</f>
       </c>
       <c r="W39" s="47"/>
       <c r="X39" s="47"/>
@@ -13608,16 +13608,16 @@
         <v>112</v>
       </c>
       <c r="S40" s="74">
-        <f>IF($R40="Fermer","",IF(SUMIFS($I$13:$I$72,$C$13:$C$72,$C40,$D$13:$D$72,$D40,$R$13:$R$72,"&lt;&gt;Fermer")=0,$M40,$M40+SUMIFS($M$13:$M$72,$C$13:$C$72,$C40,$D$13:$D$72,$D40,$R$13:$R$72,"Fermer")*$I40/SUMIFS($I$13:$I$72,$C$13:$C$72,$C40,$D$13:$D$72,$D40,$R$13:$R$72,"&lt;&gt;Fermer")))</f>
+        <f>IF(OR($C40="",COUNT($H40:$Q40)=0),"",IF($R40="Fermer","",IF(SUMIFS($I$13:$I$72,$C$13:$C$72,$C40,$D$13:$D$72,$D40,$R$13:$R$72,"&lt;&gt;Fermer")=0,$M40,$M40+SUMIFS($M$13:$M$72,$C$13:$C$72,$C40,$D$13:$D$72,$D40,$R$13:$R$72,"Fermer")*$I40/SUMIFS($I$13:$I$72,$C$13:$C$72,$C40,$D$13:$D$72,$D40,$R$13:$R$72,"&lt;&gt;Fermer"))))</f>
       </c>
       <c r="T40" s="75">
-        <f>IF($R40="Fermer","",$J40-$K40-$S40)</f>
+        <f>IF(OR($C40="",COUNT($H40:$Q40)=0),"",IF($R40="Fermer","",$J40-$K40-$S40))</f>
       </c>
       <c r="U40" s="74">
-        <f>IF($R40="Fermer",-$L40,0)</f>
+        <f>IF(OR($C40="",COUNT($H40:$Q40)=0),"",IF($R40="Fermer",-$L40,0))</f>
       </c>
       <c r="V40" s="76">
-        <f>IF($R40="Fermer","Fermer = perdre "&amp;TEXT($L40,"#,##0")&amp;" € de contribution. Le fixe, lui, reste.",IF(AND($O40&gt;=0,$T40&lt;0),"BASCULE : saine avant, en déficit à cause d'une fermeture voisine.",IF(AND($O40&lt;0,$L40&gt;0),"Déficit au coût complet mais contribution positive : ne pas fermer, c'est un artefact d'allocation.",IF($O40&lt;0,"Contribution négative : vrai point dur.","Rentable. Point mort "&amp;TEXT($P40,"#,##0")&amp;" étudiants, marge de sécurité "&amp;TEXT($Q40,"0%")&amp;"."))))</f>
+        <f>IF(OR($C40="",COUNT($H40:$Q40)=0),"",IF($R40="Fermer","Fermer = perdre "&amp;TEXT($L40,"#,##0")&amp;" € de contribution. Le fixe, lui, reste.",IF(AND($O40&gt;=0,$T40&lt;0),"BASCULE : saine avant, en déficit à cause d'une fermeture voisine.",IF(AND($O40&lt;0,$L40&gt;0),"Déficit au coût complet mais contribution positive : ne pas fermer, c'est un artefact d'allocation.",IF($O40&lt;0,"Contribution négative : vrai point dur.","Rentable. Point mort "&amp;TEXT($P40,"#,##0")&amp;" étudiants, marge de sécurité "&amp;TEXT($Q40,"0%")&amp;".")))))</f>
       </c>
       <c r="W40" s="47"/>
       <c r="X40" s="47"/>
@@ -13680,16 +13680,16 @@
         <v>115</v>
       </c>
       <c r="S41" s="74">
-        <f>IF($R41="Fermer","",IF(SUMIFS($I$13:$I$72,$C$13:$C$72,$C41,$D$13:$D$72,$D41,$R$13:$R$72,"&lt;&gt;Fermer")=0,$M41,$M41+SUMIFS($M$13:$M$72,$C$13:$C$72,$C41,$D$13:$D$72,$D41,$R$13:$R$72,"Fermer")*$I41/SUMIFS($I$13:$I$72,$C$13:$C$72,$C41,$D$13:$D$72,$D41,$R$13:$R$72,"&lt;&gt;Fermer")))</f>
+        <f>IF(OR($C41="",COUNT($H41:$Q41)=0),"",IF($R41="Fermer","",IF(SUMIFS($I$13:$I$72,$C$13:$C$72,$C41,$D$13:$D$72,$D41,$R$13:$R$72,"&lt;&gt;Fermer")=0,$M41,$M41+SUMIFS($M$13:$M$72,$C$13:$C$72,$C41,$D$13:$D$72,$D41,$R$13:$R$72,"Fermer")*$I41/SUMIFS($I$13:$I$72,$C$13:$C$72,$C41,$D$13:$D$72,$D41,$R$13:$R$72,"&lt;&gt;Fermer"))))</f>
       </c>
       <c r="T41" s="75">
-        <f>IF($R41="Fermer","",$J41-$K41-$S41)</f>
+        <f>IF(OR($C41="",COUNT($H41:$Q41)=0),"",IF($R41="Fermer","",$J41-$K41-$S41))</f>
       </c>
       <c r="U41" s="74">
-        <f>IF($R41="Fermer",-$L41,0)</f>
+        <f>IF(OR($C41="",COUNT($H41:$Q41)=0),"",IF($R41="Fermer",-$L41,0))</f>
       </c>
       <c r="V41" s="76">
-        <f>IF($R41="Fermer","Fermer = perdre "&amp;TEXT($L41,"#,##0")&amp;" € de contribution. Le fixe, lui, reste.",IF(AND($O41&gt;=0,$T41&lt;0),"BASCULE : saine avant, en déficit à cause d'une fermeture voisine.",IF(AND($O41&lt;0,$L41&gt;0),"Déficit au coût complet mais contribution positive : ne pas fermer, c'est un artefact d'allocation.",IF($O41&lt;0,"Contribution négative : vrai point dur.","Rentable. Point mort "&amp;TEXT($P41,"#,##0")&amp;" étudiants, marge de sécurité "&amp;TEXT($Q41,"0%")&amp;"."))))</f>
+        <f>IF(OR($C41="",COUNT($H41:$Q41)=0),"",IF($R41="Fermer","Fermer = perdre "&amp;TEXT($L41,"#,##0")&amp;" € de contribution. Le fixe, lui, reste.",IF(AND($O41&gt;=0,$T41&lt;0),"BASCULE : saine avant, en déficit à cause d'une fermeture voisine.",IF(AND($O41&lt;0,$L41&gt;0),"Déficit au coût complet mais contribution positive : ne pas fermer, c'est un artefact d'allocation.",IF($O41&lt;0,"Contribution négative : vrai point dur.","Rentable. Point mort "&amp;TEXT($P41,"#,##0")&amp;" étudiants, marge de sécurité "&amp;TEXT($Q41,"0%")&amp;".")))))</f>
       </c>
       <c r="W41" s="47"/>
       <c r="X41" s="47"/>
@@ -13752,16 +13752,16 @@
         <v>112</v>
       </c>
       <c r="S42" s="74">
-        <f>IF($R42="Fermer","",IF(SUMIFS($I$13:$I$72,$C$13:$C$72,$C42,$D$13:$D$72,$D42,$R$13:$R$72,"&lt;&gt;Fermer")=0,$M42,$M42+SUMIFS($M$13:$M$72,$C$13:$C$72,$C42,$D$13:$D$72,$D42,$R$13:$R$72,"Fermer")*$I42/SUMIFS($I$13:$I$72,$C$13:$C$72,$C42,$D$13:$D$72,$D42,$R$13:$R$72,"&lt;&gt;Fermer")))</f>
+        <f>IF(OR($C42="",COUNT($H42:$Q42)=0),"",IF($R42="Fermer","",IF(SUMIFS($I$13:$I$72,$C$13:$C$72,$C42,$D$13:$D$72,$D42,$R$13:$R$72,"&lt;&gt;Fermer")=0,$M42,$M42+SUMIFS($M$13:$M$72,$C$13:$C$72,$C42,$D$13:$D$72,$D42,$R$13:$R$72,"Fermer")*$I42/SUMIFS($I$13:$I$72,$C$13:$C$72,$C42,$D$13:$D$72,$D42,$R$13:$R$72,"&lt;&gt;Fermer"))))</f>
       </c>
       <c r="T42" s="75">
-        <f>IF($R42="Fermer","",$J42-$K42-$S42)</f>
+        <f>IF(OR($C42="",COUNT($H42:$Q42)=0),"",IF($R42="Fermer","",$J42-$K42-$S42))</f>
       </c>
       <c r="U42" s="74">
-        <f>IF($R42="Fermer",-$L42,0)</f>
+        <f>IF(OR($C42="",COUNT($H42:$Q42)=0),"",IF($R42="Fermer",-$L42,0))</f>
       </c>
       <c r="V42" s="76">
-        <f>IF($R42="Fermer","Fermer = perdre "&amp;TEXT($L42,"#,##0")&amp;" € de contribution. Le fixe, lui, reste.",IF(AND($O42&gt;=0,$T42&lt;0),"BASCULE : saine avant, en déficit à cause d'une fermeture voisine.",IF(AND($O42&lt;0,$L42&gt;0),"Déficit au coût complet mais contribution positive : ne pas fermer, c'est un artefact d'allocation.",IF($O42&lt;0,"Contribution négative : vrai point dur.","Rentable. Point mort "&amp;TEXT($P42,"#,##0")&amp;" étudiants, marge de sécurité "&amp;TEXT($Q42,"0%")&amp;"."))))</f>
+        <f>IF(OR($C42="",COUNT($H42:$Q42)=0),"",IF($R42="Fermer","Fermer = perdre "&amp;TEXT($L42,"#,##0")&amp;" € de contribution. Le fixe, lui, reste.",IF(AND($O42&gt;=0,$T42&lt;0),"BASCULE : saine avant, en déficit à cause d'une fermeture voisine.",IF(AND($O42&lt;0,$L42&gt;0),"Déficit au coût complet mais contribution positive : ne pas fermer, c'est un artefact d'allocation.",IF($O42&lt;0,"Contribution négative : vrai point dur.","Rentable. Point mort "&amp;TEXT($P42,"#,##0")&amp;" étudiants, marge de sécurité "&amp;TEXT($Q42,"0%")&amp;".")))))</f>
       </c>
       <c r="W42" s="47"/>
       <c r="X42" s="47"/>
@@ -13824,16 +13824,16 @@
         <v>115</v>
       </c>
       <c r="S43" s="74">
-        <f>IF($R43="Fermer","",IF(SUMIFS($I$13:$I$72,$C$13:$C$72,$C43,$D$13:$D$72,$D43,$R$13:$R$72,"&lt;&gt;Fermer")=0,$M43,$M43+SUMIFS($M$13:$M$72,$C$13:$C$72,$C43,$D$13:$D$72,$D43,$R$13:$R$72,"Fermer")*$I43/SUMIFS($I$13:$I$72,$C$13:$C$72,$C43,$D$13:$D$72,$D43,$R$13:$R$72,"&lt;&gt;Fermer")))</f>
+        <f>IF(OR($C43="",COUNT($H43:$Q43)=0),"",IF($R43="Fermer","",IF(SUMIFS($I$13:$I$72,$C$13:$C$72,$C43,$D$13:$D$72,$D43,$R$13:$R$72,"&lt;&gt;Fermer")=0,$M43,$M43+SUMIFS($M$13:$M$72,$C$13:$C$72,$C43,$D$13:$D$72,$D43,$R$13:$R$72,"Fermer")*$I43/SUMIFS($I$13:$I$72,$C$13:$C$72,$C43,$D$13:$D$72,$D43,$R$13:$R$72,"&lt;&gt;Fermer"))))</f>
       </c>
       <c r="T43" s="75">
-        <f>IF($R43="Fermer","",$J43-$K43-$S43)</f>
+        <f>IF(OR($C43="",COUNT($H43:$Q43)=0),"",IF($R43="Fermer","",$J43-$K43-$S43))</f>
       </c>
       <c r="U43" s="74">
-        <f>IF($R43="Fermer",-$L43,0)</f>
+        <f>IF(OR($C43="",COUNT($H43:$Q43)=0),"",IF($R43="Fermer",-$L43,0))</f>
       </c>
       <c r="V43" s="76">
-        <f>IF($R43="Fermer","Fermer = perdre "&amp;TEXT($L43,"#,##0")&amp;" € de contribution. Le fixe, lui, reste.",IF(AND($O43&gt;=0,$T43&lt;0),"BASCULE : saine avant, en déficit à cause d'une fermeture voisine.",IF(AND($O43&lt;0,$L43&gt;0),"Déficit au coût complet mais contribution positive : ne pas fermer, c'est un artefact d'allocation.",IF($O43&lt;0,"Contribution négative : vrai point dur.","Rentable. Point mort "&amp;TEXT($P43,"#,##0")&amp;" étudiants, marge de sécurité "&amp;TEXT($Q43,"0%")&amp;"."))))</f>
+        <f>IF(OR($C43="",COUNT($H43:$Q43)=0),"",IF($R43="Fermer","Fermer = perdre "&amp;TEXT($L43,"#,##0")&amp;" € de contribution. Le fixe, lui, reste.",IF(AND($O43&gt;=0,$T43&lt;0),"BASCULE : saine avant, en déficit à cause d'une fermeture voisine.",IF(AND($O43&lt;0,$L43&gt;0),"Déficit au coût complet mais contribution positive : ne pas fermer, c'est un artefact d'allocation.",IF($O43&lt;0,"Contribution négative : vrai point dur.","Rentable. Point mort "&amp;TEXT($P43,"#,##0")&amp;" étudiants, marge de sécurité "&amp;TEXT($Q43,"0%")&amp;".")))))</f>
       </c>
       <c r="W43" s="47"/>
       <c r="X43" s="47"/>
@@ -13896,16 +13896,16 @@
         <v>115</v>
       </c>
       <c r="S44" s="74">
-        <f>IF($R44="Fermer","",IF(SUMIFS($I$13:$I$72,$C$13:$C$72,$C44,$D$13:$D$72,$D44,$R$13:$R$72,"&lt;&gt;Fermer")=0,$M44,$M44+SUMIFS($M$13:$M$72,$C$13:$C$72,$C44,$D$13:$D$72,$D44,$R$13:$R$72,"Fermer")*$I44/SUMIFS($I$13:$I$72,$C$13:$C$72,$C44,$D$13:$D$72,$D44,$R$13:$R$72,"&lt;&gt;Fermer")))</f>
+        <f>IF(OR($C44="",COUNT($H44:$Q44)=0),"",IF($R44="Fermer","",IF(SUMIFS($I$13:$I$72,$C$13:$C$72,$C44,$D$13:$D$72,$D44,$R$13:$R$72,"&lt;&gt;Fermer")=0,$M44,$M44+SUMIFS($M$13:$M$72,$C$13:$C$72,$C44,$D$13:$D$72,$D44,$R$13:$R$72,"Fermer")*$I44/SUMIFS($I$13:$I$72,$C$13:$C$72,$C44,$D$13:$D$72,$D44,$R$13:$R$72,"&lt;&gt;Fermer"))))</f>
       </c>
       <c r="T44" s="75">
-        <f>IF($R44="Fermer","",$J44-$K44-$S44)</f>
+        <f>IF(OR($C44="",COUNT($H44:$Q44)=0),"",IF($R44="Fermer","",$J44-$K44-$S44))</f>
       </c>
       <c r="U44" s="74">
-        <f>IF($R44="Fermer",-$L44,0)</f>
+        <f>IF(OR($C44="",COUNT($H44:$Q44)=0),"",IF($R44="Fermer",-$L44,0))</f>
       </c>
       <c r="V44" s="76">
-        <f>IF($R44="Fermer","Fermer = perdre "&amp;TEXT($L44,"#,##0")&amp;" € de contribution. Le fixe, lui, reste.",IF(AND($O44&gt;=0,$T44&lt;0),"BASCULE : saine avant, en déficit à cause d'une fermeture voisine.",IF(AND($O44&lt;0,$L44&gt;0),"Déficit au coût complet mais contribution positive : ne pas fermer, c'est un artefact d'allocation.",IF($O44&lt;0,"Contribution négative : vrai point dur.","Rentable. Point mort "&amp;TEXT($P44,"#,##0")&amp;" étudiants, marge de sécurité "&amp;TEXT($Q44,"0%")&amp;"."))))</f>
+        <f>IF(OR($C44="",COUNT($H44:$Q44)=0),"",IF($R44="Fermer","Fermer = perdre "&amp;TEXT($L44,"#,##0")&amp;" € de contribution. Le fixe, lui, reste.",IF(AND($O44&gt;=0,$T44&lt;0),"BASCULE : saine avant, en déficit à cause d'une fermeture voisine.",IF(AND($O44&lt;0,$L44&gt;0),"Déficit au coût complet mais contribution positive : ne pas fermer, c'est un artefact d'allocation.",IF($O44&lt;0,"Contribution négative : vrai point dur.","Rentable. Point mort "&amp;TEXT($P44,"#,##0")&amp;" étudiants, marge de sécurité "&amp;TEXT($Q44,"0%")&amp;".")))))</f>
       </c>
       <c r="W44" s="47"/>
       <c r="X44" s="47"/>
@@ -13968,16 +13968,16 @@
         <v>112</v>
       </c>
       <c r="S45" s="74">
-        <f>IF($R45="Fermer","",IF(SUMIFS($I$13:$I$72,$C$13:$C$72,$C45,$D$13:$D$72,$D45,$R$13:$R$72,"&lt;&gt;Fermer")=0,$M45,$M45+SUMIFS($M$13:$M$72,$C$13:$C$72,$C45,$D$13:$D$72,$D45,$R$13:$R$72,"Fermer")*$I45/SUMIFS($I$13:$I$72,$C$13:$C$72,$C45,$D$13:$D$72,$D45,$R$13:$R$72,"&lt;&gt;Fermer")))</f>
+        <f>IF(OR($C45="",COUNT($H45:$Q45)=0),"",IF($R45="Fermer","",IF(SUMIFS($I$13:$I$72,$C$13:$C$72,$C45,$D$13:$D$72,$D45,$R$13:$R$72,"&lt;&gt;Fermer")=0,$M45,$M45+SUMIFS($M$13:$M$72,$C$13:$C$72,$C45,$D$13:$D$72,$D45,$R$13:$R$72,"Fermer")*$I45/SUMIFS($I$13:$I$72,$C$13:$C$72,$C45,$D$13:$D$72,$D45,$R$13:$R$72,"&lt;&gt;Fermer"))))</f>
       </c>
       <c r="T45" s="75">
-        <f>IF($R45="Fermer","",$J45-$K45-$S45)</f>
+        <f>IF(OR($C45="",COUNT($H45:$Q45)=0),"",IF($R45="Fermer","",$J45-$K45-$S45))</f>
       </c>
       <c r="U45" s="74">
-        <f>IF($R45="Fermer",-$L45,0)</f>
+        <f>IF(OR($C45="",COUNT($H45:$Q45)=0),"",IF($R45="Fermer",-$L45,0))</f>
       </c>
       <c r="V45" s="76">
-        <f>IF($R45="Fermer","Fermer = perdre "&amp;TEXT($L45,"#,##0")&amp;" € de contribution. Le fixe, lui, reste.",IF(AND($O45&gt;=0,$T45&lt;0),"BASCULE : saine avant, en déficit à cause d'une fermeture voisine.",IF(AND($O45&lt;0,$L45&gt;0),"Déficit au coût complet mais contribution positive : ne pas fermer, c'est un artefact d'allocation.",IF($O45&lt;0,"Contribution négative : vrai point dur.","Rentable. Point mort "&amp;TEXT($P45,"#,##0")&amp;" étudiants, marge de sécurité "&amp;TEXT($Q45,"0%")&amp;"."))))</f>
+        <f>IF(OR($C45="",COUNT($H45:$Q45)=0),"",IF($R45="Fermer","Fermer = perdre "&amp;TEXT($L45,"#,##0")&amp;" € de contribution. Le fixe, lui, reste.",IF(AND($O45&gt;=0,$T45&lt;0),"BASCULE : saine avant, en déficit à cause d'une fermeture voisine.",IF(AND($O45&lt;0,$L45&gt;0),"Déficit au coût complet mais contribution positive : ne pas fermer, c'est un artefact d'allocation.",IF($O45&lt;0,"Contribution négative : vrai point dur.","Rentable. Point mort "&amp;TEXT($P45,"#,##0")&amp;" étudiants, marge de sécurité "&amp;TEXT($Q45,"0%")&amp;".")))))</f>
       </c>
       <c r="W45" s="47"/>
       <c r="X45" s="47"/>
@@ -14040,16 +14040,16 @@
         <v>115</v>
       </c>
       <c r="S46" s="74">
-        <f>IF($R46="Fermer","",IF(SUMIFS($I$13:$I$72,$C$13:$C$72,$C46,$D$13:$D$72,$D46,$R$13:$R$72,"&lt;&gt;Fermer")=0,$M46,$M46+SUMIFS($M$13:$M$72,$C$13:$C$72,$C46,$D$13:$D$72,$D46,$R$13:$R$72,"Fermer")*$I46/SUMIFS($I$13:$I$72,$C$13:$C$72,$C46,$D$13:$D$72,$D46,$R$13:$R$72,"&lt;&gt;Fermer")))</f>
+        <f>IF(OR($C46="",COUNT($H46:$Q46)=0),"",IF($R46="Fermer","",IF(SUMIFS($I$13:$I$72,$C$13:$C$72,$C46,$D$13:$D$72,$D46,$R$13:$R$72,"&lt;&gt;Fermer")=0,$M46,$M46+SUMIFS($M$13:$M$72,$C$13:$C$72,$C46,$D$13:$D$72,$D46,$R$13:$R$72,"Fermer")*$I46/SUMIFS($I$13:$I$72,$C$13:$C$72,$C46,$D$13:$D$72,$D46,$R$13:$R$72,"&lt;&gt;Fermer"))))</f>
       </c>
       <c r="T46" s="75">
-        <f>IF($R46="Fermer","",$J46-$K46-$S46)</f>
+        <f>IF(OR($C46="",COUNT($H46:$Q46)=0),"",IF($R46="Fermer","",$J46-$K46-$S46))</f>
       </c>
       <c r="U46" s="74">
-        <f>IF($R46="Fermer",-$L46,0)</f>
+        <f>IF(OR($C46="",COUNT($H46:$Q46)=0),"",IF($R46="Fermer",-$L46,0))</f>
       </c>
       <c r="V46" s="76">
-        <f>IF($R46="Fermer","Fermer = perdre "&amp;TEXT($L46,"#,##0")&amp;" € de contribution. Le fixe, lui, reste.",IF(AND($O46&gt;=0,$T46&lt;0),"BASCULE : saine avant, en déficit à cause d'une fermeture voisine.",IF(AND($O46&lt;0,$L46&gt;0),"Déficit au coût complet mais contribution positive : ne pas fermer, c'est un artefact d'allocation.",IF($O46&lt;0,"Contribution négative : vrai point dur.","Rentable. Point mort "&amp;TEXT($P46,"#,##0")&amp;" étudiants, marge de sécurité "&amp;TEXT($Q46,"0%")&amp;"."))))</f>
+        <f>IF(OR($C46="",COUNT($H46:$Q46)=0),"",IF($R46="Fermer","Fermer = perdre "&amp;TEXT($L46,"#,##0")&amp;" € de contribution. Le fixe, lui, reste.",IF(AND($O46&gt;=0,$T46&lt;0),"BASCULE : saine avant, en déficit à cause d'une fermeture voisine.",IF(AND($O46&lt;0,$L46&gt;0),"Déficit au coût complet mais contribution positive : ne pas fermer, c'est un artefact d'allocation.",IF($O46&lt;0,"Contribution négative : vrai point dur.","Rentable. Point mort "&amp;TEXT($P46,"#,##0")&amp;" étudiants, marge de sécurité "&amp;TEXT($Q46,"0%")&amp;".")))))</f>
       </c>
       <c r="W46" s="47"/>
       <c r="X46" s="47"/>
@@ -14112,16 +14112,16 @@
         <v>112</v>
       </c>
       <c r="S47" s="74">
-        <f>IF($R47="Fermer","",IF(SUMIFS($I$13:$I$72,$C$13:$C$72,$C47,$D$13:$D$72,$D47,$R$13:$R$72,"&lt;&gt;Fermer")=0,$M47,$M47+SUMIFS($M$13:$M$72,$C$13:$C$72,$C47,$D$13:$D$72,$D47,$R$13:$R$72,"Fermer")*$I47/SUMIFS($I$13:$I$72,$C$13:$C$72,$C47,$D$13:$D$72,$D47,$R$13:$R$72,"&lt;&gt;Fermer")))</f>
+        <f>IF(OR($C47="",COUNT($H47:$Q47)=0),"",IF($R47="Fermer","",IF(SUMIFS($I$13:$I$72,$C$13:$C$72,$C47,$D$13:$D$72,$D47,$R$13:$R$72,"&lt;&gt;Fermer")=0,$M47,$M47+SUMIFS($M$13:$M$72,$C$13:$C$72,$C47,$D$13:$D$72,$D47,$R$13:$R$72,"Fermer")*$I47/SUMIFS($I$13:$I$72,$C$13:$C$72,$C47,$D$13:$D$72,$D47,$R$13:$R$72,"&lt;&gt;Fermer"))))</f>
       </c>
       <c r="T47" s="75">
-        <f>IF($R47="Fermer","",$J47-$K47-$S47)</f>
+        <f>IF(OR($C47="",COUNT($H47:$Q47)=0),"",IF($R47="Fermer","",$J47-$K47-$S47))</f>
       </c>
       <c r="U47" s="74">
-        <f>IF($R47="Fermer",-$L47,0)</f>
+        <f>IF(OR($C47="",COUNT($H47:$Q47)=0),"",IF($R47="Fermer",-$L47,0))</f>
       </c>
       <c r="V47" s="76">
-        <f>IF($R47="Fermer","Fermer = perdre "&amp;TEXT($L47,"#,##0")&amp;" € de contribution. Le fixe, lui, reste.",IF(AND($O47&gt;=0,$T47&lt;0),"BASCULE : saine avant, en déficit à cause d'une fermeture voisine.",IF(AND($O47&lt;0,$L47&gt;0),"Déficit au coût complet mais contribution positive : ne pas fermer, c'est un artefact d'allocation.",IF($O47&lt;0,"Contribution négative : vrai point dur.","Rentable. Point mort "&amp;TEXT($P47,"#,##0")&amp;" étudiants, marge de sécurité "&amp;TEXT($Q47,"0%")&amp;"."))))</f>
+        <f>IF(OR($C47="",COUNT($H47:$Q47)=0),"",IF($R47="Fermer","Fermer = perdre "&amp;TEXT($L47,"#,##0")&amp;" € de contribution. Le fixe, lui, reste.",IF(AND($O47&gt;=0,$T47&lt;0),"BASCULE : saine avant, en déficit à cause d'une fermeture voisine.",IF(AND($O47&lt;0,$L47&gt;0),"Déficit au coût complet mais contribution positive : ne pas fermer, c'est un artefact d'allocation.",IF($O47&lt;0,"Contribution négative : vrai point dur.","Rentable. Point mort "&amp;TEXT($P47,"#,##0")&amp;" étudiants, marge de sécurité "&amp;TEXT($Q47,"0%")&amp;".")))))</f>
       </c>
       <c r="W47" s="47"/>
       <c r="X47" s="47"/>
@@ -14184,16 +14184,16 @@
         <v>115</v>
       </c>
       <c r="S48" s="74">
-        <f>IF($R48="Fermer","",IF(SUMIFS($I$13:$I$72,$C$13:$C$72,$C48,$D$13:$D$72,$D48,$R$13:$R$72,"&lt;&gt;Fermer")=0,$M48,$M48+SUMIFS($M$13:$M$72,$C$13:$C$72,$C48,$D$13:$D$72,$D48,$R$13:$R$72,"Fermer")*$I48/SUMIFS($I$13:$I$72,$C$13:$C$72,$C48,$D$13:$D$72,$D48,$R$13:$R$72,"&lt;&gt;Fermer")))</f>
+        <f>IF(OR($C48="",COUNT($H48:$Q48)=0),"",IF($R48="Fermer","",IF(SUMIFS($I$13:$I$72,$C$13:$C$72,$C48,$D$13:$D$72,$D48,$R$13:$R$72,"&lt;&gt;Fermer")=0,$M48,$M48+SUMIFS($M$13:$M$72,$C$13:$C$72,$C48,$D$13:$D$72,$D48,$R$13:$R$72,"Fermer")*$I48/SUMIFS($I$13:$I$72,$C$13:$C$72,$C48,$D$13:$D$72,$D48,$R$13:$R$72,"&lt;&gt;Fermer"))))</f>
       </c>
       <c r="T48" s="75">
-        <f>IF($R48="Fermer","",$J48-$K48-$S48)</f>
+        <f>IF(OR($C48="",COUNT($H48:$Q48)=0),"",IF($R48="Fermer","",$J48-$K48-$S48))</f>
       </c>
       <c r="U48" s="74">
-        <f>IF($R48="Fermer",-$L48,0)</f>
+        <f>IF(OR($C48="",COUNT($H48:$Q48)=0),"",IF($R48="Fermer",-$L48,0))</f>
       </c>
       <c r="V48" s="76">
-        <f>IF($R48="Fermer","Fermer = perdre "&amp;TEXT($L48,"#,##0")&amp;" € de contribution. Le fixe, lui, reste.",IF(AND($O48&gt;=0,$T48&lt;0),"BASCULE : saine avant, en déficit à cause d'une fermeture voisine.",IF(AND($O48&lt;0,$L48&gt;0),"Déficit au coût complet mais contribution positive : ne pas fermer, c'est un artefact d'allocation.",IF($O48&lt;0,"Contribution négative : vrai point dur.","Rentable. Point mort "&amp;TEXT($P48,"#,##0")&amp;" étudiants, marge de sécurité "&amp;TEXT($Q48,"0%")&amp;"."))))</f>
+        <f>IF(OR($C48="",COUNT($H48:$Q48)=0),"",IF($R48="Fermer","Fermer = perdre "&amp;TEXT($L48,"#,##0")&amp;" € de contribution. Le fixe, lui, reste.",IF(AND($O48&gt;=0,$T48&lt;0),"BASCULE : saine avant, en déficit à cause d'une fermeture voisine.",IF(AND($O48&lt;0,$L48&gt;0),"Déficit au coût complet mais contribution positive : ne pas fermer, c'est un artefact d'allocation.",IF($O48&lt;0,"Contribution négative : vrai point dur.","Rentable. Point mort "&amp;TEXT($P48,"#,##0")&amp;" étudiants, marge de sécurité "&amp;TEXT($Q48,"0%")&amp;".")))))</f>
       </c>
       <c r="W48" s="47"/>
       <c r="X48" s="47"/>
@@ -14256,16 +14256,16 @@
         <v>115</v>
       </c>
       <c r="S49" s="74">
-        <f>IF($R49="Fermer","",IF(SUMIFS($I$13:$I$72,$C$13:$C$72,$C49,$D$13:$D$72,$D49,$R$13:$R$72,"&lt;&gt;Fermer")=0,$M49,$M49+SUMIFS($M$13:$M$72,$C$13:$C$72,$C49,$D$13:$D$72,$D49,$R$13:$R$72,"Fermer")*$I49/SUMIFS($I$13:$I$72,$C$13:$C$72,$C49,$D$13:$D$72,$D49,$R$13:$R$72,"&lt;&gt;Fermer")))</f>
+        <f>IF(OR($C49="",COUNT($H49:$Q49)=0),"",IF($R49="Fermer","",IF(SUMIFS($I$13:$I$72,$C$13:$C$72,$C49,$D$13:$D$72,$D49,$R$13:$R$72,"&lt;&gt;Fermer")=0,$M49,$M49+SUMIFS($M$13:$M$72,$C$13:$C$72,$C49,$D$13:$D$72,$D49,$R$13:$R$72,"Fermer")*$I49/SUMIFS($I$13:$I$72,$C$13:$C$72,$C49,$D$13:$D$72,$D49,$R$13:$R$72,"&lt;&gt;Fermer"))))</f>
       </c>
       <c r="T49" s="75">
-        <f>IF($R49="Fermer","",$J49-$K49-$S49)</f>
+        <f>IF(OR($C49="",COUNT($H49:$Q49)=0),"",IF($R49="Fermer","",$J49-$K49-$S49))</f>
       </c>
       <c r="U49" s="74">
-        <f>IF($R49="Fermer",-$L49,0)</f>
+        <f>IF(OR($C49="",COUNT($H49:$Q49)=0),"",IF($R49="Fermer",-$L49,0))</f>
       </c>
       <c r="V49" s="76">
-        <f>IF($R49="Fermer","Fermer = perdre "&amp;TEXT($L49,"#,##0")&amp;" € de contribution. Le fixe, lui, reste.",IF(AND($O49&gt;=0,$T49&lt;0),"BASCULE : saine avant, en déficit à cause d'une fermeture voisine.",IF(AND($O49&lt;0,$L49&gt;0),"Déficit au coût complet mais contribution positive : ne pas fermer, c'est un artefact d'allocation.",IF($O49&lt;0,"Contribution négative : vrai point dur.","Rentable. Point mort "&amp;TEXT($P49,"#,##0")&amp;" étudiants, marge de sécurité "&amp;TEXT($Q49,"0%")&amp;"."))))</f>
+        <f>IF(OR($C49="",COUNT($H49:$Q49)=0),"",IF($R49="Fermer","Fermer = perdre "&amp;TEXT($L49,"#,##0")&amp;" € de contribution. Le fixe, lui, reste.",IF(AND($O49&gt;=0,$T49&lt;0),"BASCULE : saine avant, en déficit à cause d'une fermeture voisine.",IF(AND($O49&lt;0,$L49&gt;0),"Déficit au coût complet mais contribution positive : ne pas fermer, c'est un artefact d'allocation.",IF($O49&lt;0,"Contribution négative : vrai point dur.","Rentable. Point mort "&amp;TEXT($P49,"#,##0")&amp;" étudiants, marge de sécurité "&amp;TEXT($Q49,"0%")&amp;".")))))</f>
       </c>
       <c r="W49" s="47"/>
       <c r="X49" s="47"/>
@@ -14328,16 +14328,16 @@
         <v>112</v>
       </c>
       <c r="S50" s="74">
-        <f>IF($R50="Fermer","",IF(SUMIFS($I$13:$I$72,$C$13:$C$72,$C50,$D$13:$D$72,$D50,$R$13:$R$72,"&lt;&gt;Fermer")=0,$M50,$M50+SUMIFS($M$13:$M$72,$C$13:$C$72,$C50,$D$13:$D$72,$D50,$R$13:$R$72,"Fermer")*$I50/SUMIFS($I$13:$I$72,$C$13:$C$72,$C50,$D$13:$D$72,$D50,$R$13:$R$72,"&lt;&gt;Fermer")))</f>
+        <f>IF(OR($C50="",COUNT($H50:$Q50)=0),"",IF($R50="Fermer","",IF(SUMIFS($I$13:$I$72,$C$13:$C$72,$C50,$D$13:$D$72,$D50,$R$13:$R$72,"&lt;&gt;Fermer")=0,$M50,$M50+SUMIFS($M$13:$M$72,$C$13:$C$72,$C50,$D$13:$D$72,$D50,$R$13:$R$72,"Fermer")*$I50/SUMIFS($I$13:$I$72,$C$13:$C$72,$C50,$D$13:$D$72,$D50,$R$13:$R$72,"&lt;&gt;Fermer"))))</f>
       </c>
       <c r="T50" s="75">
-        <f>IF($R50="Fermer","",$J50-$K50-$S50)</f>
+        <f>IF(OR($C50="",COUNT($H50:$Q50)=0),"",IF($R50="Fermer","",$J50-$K50-$S50))</f>
       </c>
       <c r="U50" s="74">
-        <f>IF($R50="Fermer",-$L50,0)</f>
+        <f>IF(OR($C50="",COUNT($H50:$Q50)=0),"",IF($R50="Fermer",-$L50,0))</f>
       </c>
       <c r="V50" s="76">
-        <f>IF($R50="Fermer","Fermer = perdre "&amp;TEXT($L50,"#,##0")&amp;" € de contribution. Le fixe, lui, reste.",IF(AND($O50&gt;=0,$T50&lt;0),"BASCULE : saine avant, en déficit à cause d'une fermeture voisine.",IF(AND($O50&lt;0,$L50&gt;0),"Déficit au coût complet mais contribution positive : ne pas fermer, c'est un artefact d'allocation.",IF($O50&lt;0,"Contribution négative : vrai point dur.","Rentable. Point mort "&amp;TEXT($P50,"#,##0")&amp;" étudiants, marge de sécurité "&amp;TEXT($Q50,"0%")&amp;"."))))</f>
+        <f>IF(OR($C50="",COUNT($H50:$Q50)=0),"",IF($R50="Fermer","Fermer = perdre "&amp;TEXT($L50,"#,##0")&amp;" € de contribution. Le fixe, lui, reste.",IF(AND($O50&gt;=0,$T50&lt;0),"BASCULE : saine avant, en déficit à cause d'une fermeture voisine.",IF(AND($O50&lt;0,$L50&gt;0),"Déficit au coût complet mais contribution positive : ne pas fermer, c'est un artefact d'allocation.",IF($O50&lt;0,"Contribution négative : vrai point dur.","Rentable. Point mort "&amp;TEXT($P50,"#,##0")&amp;" étudiants, marge de sécurité "&amp;TEXT($Q50,"0%")&amp;".")))))</f>
       </c>
       <c r="W50" s="47"/>
       <c r="X50" s="47"/>
@@ -14400,16 +14400,16 @@
         <v>115</v>
       </c>
       <c r="S51" s="74">
-        <f>IF($R51="Fermer","",IF(SUMIFS($I$13:$I$72,$C$13:$C$72,$C51,$D$13:$D$72,$D51,$R$13:$R$72,"&lt;&gt;Fermer")=0,$M51,$M51+SUMIFS($M$13:$M$72,$C$13:$C$72,$C51,$D$13:$D$72,$D51,$R$13:$R$72,"Fermer")*$I51/SUMIFS($I$13:$I$72,$C$13:$C$72,$C51,$D$13:$D$72,$D51,$R$13:$R$72,"&lt;&gt;Fermer")))</f>
+        <f>IF(OR($C51="",COUNT($H51:$Q51)=0),"",IF($R51="Fermer","",IF(SUMIFS($I$13:$I$72,$C$13:$C$72,$C51,$D$13:$D$72,$D51,$R$13:$R$72,"&lt;&gt;Fermer")=0,$M51,$M51+SUMIFS($M$13:$M$72,$C$13:$C$72,$C51,$D$13:$D$72,$D51,$R$13:$R$72,"Fermer")*$I51/SUMIFS($I$13:$I$72,$C$13:$C$72,$C51,$D$13:$D$72,$D51,$R$13:$R$72,"&lt;&gt;Fermer"))))</f>
       </c>
       <c r="T51" s="75">
-        <f>IF($R51="Fermer","",$J51-$K51-$S51)</f>
+        <f>IF(OR($C51="",COUNT($H51:$Q51)=0),"",IF($R51="Fermer","",$J51-$K51-$S51))</f>
       </c>
       <c r="U51" s="74">
-        <f>IF($R51="Fermer",-$L51,0)</f>
+        <f>IF(OR($C51="",COUNT($H51:$Q51)=0),"",IF($R51="Fermer",-$L51,0))</f>
       </c>
       <c r="V51" s="76">
-        <f>IF($R51="Fermer","Fermer = perdre "&amp;TEXT($L51,"#,##0")&amp;" € de contribution. Le fixe, lui, reste.",IF(AND($O51&gt;=0,$T51&lt;0),"BASCULE : saine avant, en déficit à cause d'une fermeture voisine.",IF(AND($O51&lt;0,$L51&gt;0),"Déficit au coût complet mais contribution positive : ne pas fermer, c'est un artefact d'allocation.",IF($O51&lt;0,"Contribution négative : vrai point dur.","Rentable. Point mort "&amp;TEXT($P51,"#,##0")&amp;" étudiants, marge de sécurité "&amp;TEXT($Q51,"0%")&amp;"."))))</f>
+        <f>IF(OR($C51="",COUNT($H51:$Q51)=0),"",IF($R51="Fermer","Fermer = perdre "&amp;TEXT($L51,"#,##0")&amp;" € de contribution. Le fixe, lui, reste.",IF(AND($O51&gt;=0,$T51&lt;0),"BASCULE : saine avant, en déficit à cause d'une fermeture voisine.",IF(AND($O51&lt;0,$L51&gt;0),"Déficit au coût complet mais contribution positive : ne pas fermer, c'est un artefact d'allocation.",IF($O51&lt;0,"Contribution négative : vrai point dur.","Rentable. Point mort "&amp;TEXT($P51,"#,##0")&amp;" étudiants, marge de sécurité "&amp;TEXT($Q51,"0%")&amp;".")))))</f>
       </c>
       <c r="W51" s="47"/>
       <c r="X51" s="47"/>
@@ -14472,16 +14472,16 @@
         <v>112</v>
       </c>
       <c r="S52" s="74">
-        <f>IF($R52="Fermer","",IF(SUMIFS($I$13:$I$72,$C$13:$C$72,$C52,$D$13:$D$72,$D52,$R$13:$R$72,"&lt;&gt;Fermer")=0,$M52,$M52+SUMIFS($M$13:$M$72,$C$13:$C$72,$C52,$D$13:$D$72,$D52,$R$13:$R$72,"Fermer")*$I52/SUMIFS($I$13:$I$72,$C$13:$C$72,$C52,$D$13:$D$72,$D52,$R$13:$R$72,"&lt;&gt;Fermer")))</f>
+        <f>IF(OR($C52="",COUNT($H52:$Q52)=0),"",IF($R52="Fermer","",IF(SUMIFS($I$13:$I$72,$C$13:$C$72,$C52,$D$13:$D$72,$D52,$R$13:$R$72,"&lt;&gt;Fermer")=0,$M52,$M52+SUMIFS($M$13:$M$72,$C$13:$C$72,$C52,$D$13:$D$72,$D52,$R$13:$R$72,"Fermer")*$I52/SUMIFS($I$13:$I$72,$C$13:$C$72,$C52,$D$13:$D$72,$D52,$R$13:$R$72,"&lt;&gt;Fermer"))))</f>
       </c>
       <c r="T52" s="75">
-        <f>IF($R52="Fermer","",$J52-$K52-$S52)</f>
+        <f>IF(OR($C52="",COUNT($H52:$Q52)=0),"",IF($R52="Fermer","",$J52-$K52-$S52))</f>
       </c>
       <c r="U52" s="74">
-        <f>IF($R52="Fermer",-$L52,0)</f>
+        <f>IF(OR($C52="",COUNT($H52:$Q52)=0),"",IF($R52="Fermer",-$L52,0))</f>
       </c>
       <c r="V52" s="76">
-        <f>IF($R52="Fermer","Fermer = perdre "&amp;TEXT($L52,"#,##0")&amp;" € de contribution. Le fixe, lui, reste.",IF(AND($O52&gt;=0,$T52&lt;0),"BASCULE : saine avant, en déficit à cause d'une fermeture voisine.",IF(AND($O52&lt;0,$L52&gt;0),"Déficit au coût complet mais contribution positive : ne pas fermer, c'est un artefact d'allocation.",IF($O52&lt;0,"Contribution négative : vrai point dur.","Rentable. Point mort "&amp;TEXT($P52,"#,##0")&amp;" étudiants, marge de sécurité "&amp;TEXT($Q52,"0%")&amp;"."))))</f>
+        <f>IF(OR($C52="",COUNT($H52:$Q52)=0),"",IF($R52="Fermer","Fermer = perdre "&amp;TEXT($L52,"#,##0")&amp;" € de contribution. Le fixe, lui, reste.",IF(AND($O52&gt;=0,$T52&lt;0),"BASCULE : saine avant, en déficit à cause d'une fermeture voisine.",IF(AND($O52&lt;0,$L52&gt;0),"Déficit au coût complet mais contribution positive : ne pas fermer, c'est un artefact d'allocation.",IF($O52&lt;0,"Contribution négative : vrai point dur.","Rentable. Point mort "&amp;TEXT($P52,"#,##0")&amp;" étudiants, marge de sécurité "&amp;TEXT($Q52,"0%")&amp;".")))))</f>
       </c>
       <c r="W52" s="47"/>
       <c r="X52" s="47"/>
@@ -14544,16 +14544,16 @@
         <v>115</v>
       </c>
       <c r="S53" s="74">
-        <f>IF($R53="Fermer","",IF(SUMIFS($I$13:$I$72,$C$13:$C$72,$C53,$D$13:$D$72,$D53,$R$13:$R$72,"&lt;&gt;Fermer")=0,$M53,$M53+SUMIFS($M$13:$M$72,$C$13:$C$72,$C53,$D$13:$D$72,$D53,$R$13:$R$72,"Fermer")*$I53/SUMIFS($I$13:$I$72,$C$13:$C$72,$C53,$D$13:$D$72,$D53,$R$13:$R$72,"&lt;&gt;Fermer")))</f>
+        <f>IF(OR($C53="",COUNT($H53:$Q53)=0),"",IF($R53="Fermer","",IF(SUMIFS($I$13:$I$72,$C$13:$C$72,$C53,$D$13:$D$72,$D53,$R$13:$R$72,"&lt;&gt;Fermer")=0,$M53,$M53+SUMIFS($M$13:$M$72,$C$13:$C$72,$C53,$D$13:$D$72,$D53,$R$13:$R$72,"Fermer")*$I53/SUMIFS($I$13:$I$72,$C$13:$C$72,$C53,$D$13:$D$72,$D53,$R$13:$R$72,"&lt;&gt;Fermer"))))</f>
       </c>
       <c r="T53" s="75">
-        <f>IF($R53="Fermer","",$J53-$K53-$S53)</f>
+        <f>IF(OR($C53="",COUNT($H53:$Q53)=0),"",IF($R53="Fermer","",$J53-$K53-$S53))</f>
       </c>
       <c r="U53" s="74">
-        <f>IF($R53="Fermer",-$L53,0)</f>
+        <f>IF(OR($C53="",COUNT($H53:$Q53)=0),"",IF($R53="Fermer",-$L53,0))</f>
       </c>
       <c r="V53" s="76">
-        <f>IF($R53="Fermer","Fermer = perdre "&amp;TEXT($L53,"#,##0")&amp;" € de contribution. Le fixe, lui, reste.",IF(AND($O53&gt;=0,$T53&lt;0),"BASCULE : saine avant, en déficit à cause d'une fermeture voisine.",IF(AND($O53&lt;0,$L53&gt;0),"Déficit au coût complet mais contribution positive : ne pas fermer, c'est un artefact d'allocation.",IF($O53&lt;0,"Contribution négative : vrai point dur.","Rentable. Point mort "&amp;TEXT($P53,"#,##0")&amp;" étudiants, marge de sécurité "&amp;TEXT($Q53,"0%")&amp;"."))))</f>
+        <f>IF(OR($C53="",COUNT($H53:$Q53)=0),"",IF($R53="Fermer","Fermer = perdre "&amp;TEXT($L53,"#,##0")&amp;" € de contribution. Le fixe, lui, reste.",IF(AND($O53&gt;=0,$T53&lt;0),"BASCULE : saine avant, en déficit à cause d'une fermeture voisine.",IF(AND($O53&lt;0,$L53&gt;0),"Déficit au coût complet mais contribution positive : ne pas fermer, c'est un artefact d'allocation.",IF($O53&lt;0,"Contribution négative : vrai point dur.","Rentable. Point mort "&amp;TEXT($P53,"#,##0")&amp;" étudiants, marge de sécurité "&amp;TEXT($Q53,"0%")&amp;".")))))</f>
       </c>
       <c r="W53" s="47"/>
       <c r="X53" s="47"/>
@@ -14616,16 +14616,16 @@
         <v>115</v>
       </c>
       <c r="S54" s="74">
-        <f>IF($R54="Fermer","",IF(SUMIFS($I$13:$I$72,$C$13:$C$72,$C54,$D$13:$D$72,$D54,$R$13:$R$72,"&lt;&gt;Fermer")=0,$M54,$M54+SUMIFS($M$13:$M$72,$C$13:$C$72,$C54,$D$13:$D$72,$D54,$R$13:$R$72,"Fermer")*$I54/SUMIFS($I$13:$I$72,$C$13:$C$72,$C54,$D$13:$D$72,$D54,$R$13:$R$72,"&lt;&gt;Fermer")))</f>
+        <f>IF(OR($C54="",COUNT($H54:$Q54)=0),"",IF($R54="Fermer","",IF(SUMIFS($I$13:$I$72,$C$13:$C$72,$C54,$D$13:$D$72,$D54,$R$13:$R$72,"&lt;&gt;Fermer")=0,$M54,$M54+SUMIFS($M$13:$M$72,$C$13:$C$72,$C54,$D$13:$D$72,$D54,$R$13:$R$72,"Fermer")*$I54/SUMIFS($I$13:$I$72,$C$13:$C$72,$C54,$D$13:$D$72,$D54,$R$13:$R$72,"&lt;&gt;Fermer"))))</f>
       </c>
       <c r="T54" s="75">
-        <f>IF($R54="Fermer","",$J54-$K54-$S54)</f>
+        <f>IF(OR($C54="",COUNT($H54:$Q54)=0),"",IF($R54="Fermer","",$J54-$K54-$S54))</f>
       </c>
       <c r="U54" s="74">
-        <f>IF($R54="Fermer",-$L54,0)</f>
+        <f>IF(OR($C54="",COUNT($H54:$Q54)=0),"",IF($R54="Fermer",-$L54,0))</f>
       </c>
       <c r="V54" s="76">
-        <f>IF($R54="Fermer","Fermer = perdre "&amp;TEXT($L54,"#,##0")&amp;" € de contribution. Le fixe, lui, reste.",IF(AND($O54&gt;=0,$T54&lt;0),"BASCULE : saine avant, en déficit à cause d'une fermeture voisine.",IF(AND($O54&lt;0,$L54&gt;0),"Déficit au coût complet mais contribution positive : ne pas fermer, c'est un artefact d'allocation.",IF($O54&lt;0,"Contribution négative : vrai point dur.","Rentable. Point mort "&amp;TEXT($P54,"#,##0")&amp;" étudiants, marge de sécurité "&amp;TEXT($Q54,"0%")&amp;"."))))</f>
+        <f>IF(OR($C54="",COUNT($H54:$Q54)=0),"",IF($R54="Fermer","Fermer = perdre "&amp;TEXT($L54,"#,##0")&amp;" € de contribution. Le fixe, lui, reste.",IF(AND($O54&gt;=0,$T54&lt;0),"BASCULE : saine avant, en déficit à cause d'une fermeture voisine.",IF(AND($O54&lt;0,$L54&gt;0),"Déficit au coût complet mais contribution positive : ne pas fermer, c'est un artefact d'allocation.",IF($O54&lt;0,"Contribution négative : vrai point dur.","Rentable. Point mort "&amp;TEXT($P54,"#,##0")&amp;" étudiants, marge de sécurité "&amp;TEXT($Q54,"0%")&amp;".")))))</f>
       </c>
       <c r="W54" s="47"/>
       <c r="X54" s="47"/>
@@ -14688,16 +14688,16 @@
         <v>112</v>
       </c>
       <c r="S55" s="74">
-        <f>IF($R55="Fermer","",IF(SUMIFS($I$13:$I$72,$C$13:$C$72,$C55,$D$13:$D$72,$D55,$R$13:$R$72,"&lt;&gt;Fermer")=0,$M55,$M55+SUMIFS($M$13:$M$72,$C$13:$C$72,$C55,$D$13:$D$72,$D55,$R$13:$R$72,"Fermer")*$I55/SUMIFS($I$13:$I$72,$C$13:$C$72,$C55,$D$13:$D$72,$D55,$R$13:$R$72,"&lt;&gt;Fermer")))</f>
+        <f>IF(OR($C55="",COUNT($H55:$Q55)=0),"",IF($R55="Fermer","",IF(SUMIFS($I$13:$I$72,$C$13:$C$72,$C55,$D$13:$D$72,$D55,$R$13:$R$72,"&lt;&gt;Fermer")=0,$M55,$M55+SUMIFS($M$13:$M$72,$C$13:$C$72,$C55,$D$13:$D$72,$D55,$R$13:$R$72,"Fermer")*$I55/SUMIFS($I$13:$I$72,$C$13:$C$72,$C55,$D$13:$D$72,$D55,$R$13:$R$72,"&lt;&gt;Fermer"))))</f>
       </c>
       <c r="T55" s="75">
-        <f>IF($R55="Fermer","",$J55-$K55-$S55)</f>
+        <f>IF(OR($C55="",COUNT($H55:$Q55)=0),"",IF($R55="Fermer","",$J55-$K55-$S55))</f>
       </c>
       <c r="U55" s="74">
-        <f>IF($R55="Fermer",-$L55,0)</f>
+        <f>IF(OR($C55="",COUNT($H55:$Q55)=0),"",IF($R55="Fermer",-$L55,0))</f>
       </c>
       <c r="V55" s="76">
-        <f>IF($R55="Fermer","Fermer = perdre "&amp;TEXT($L55,"#,##0")&amp;" € de contribution. Le fixe, lui, reste.",IF(AND($O55&gt;=0,$T55&lt;0),"BASCULE : saine avant, en déficit à cause d'une fermeture voisine.",IF(AND($O55&lt;0,$L55&gt;0),"Déficit au coût complet mais contribution positive : ne pas fermer, c'est un artefact d'allocation.",IF($O55&lt;0,"Contribution négative : vrai point dur.","Rentable. Point mort "&amp;TEXT($P55,"#,##0")&amp;" étudiants, marge de sécurité "&amp;TEXT($Q55,"0%")&amp;"."))))</f>
+        <f>IF(OR($C55="",COUNT($H55:$Q55)=0),"",IF($R55="Fermer","Fermer = perdre "&amp;TEXT($L55,"#,##0")&amp;" € de contribution. Le fixe, lui, reste.",IF(AND($O55&gt;=0,$T55&lt;0),"BASCULE : saine avant, en déficit à cause d'une fermeture voisine.",IF(AND($O55&lt;0,$L55&gt;0),"Déficit au coût complet mais contribution positive : ne pas fermer, c'est un artefact d'allocation.",IF($O55&lt;0,"Contribution négative : vrai point dur.","Rentable. Point mort "&amp;TEXT($P55,"#,##0")&amp;" étudiants, marge de sécurité "&amp;TEXT($Q55,"0%")&amp;".")))))</f>
       </c>
       <c r="W55" s="47"/>
       <c r="X55" s="47"/>
@@ -14760,16 +14760,16 @@
         <v>115</v>
       </c>
       <c r="S56" s="74">
-        <f>IF($R56="Fermer","",IF(SUMIFS($I$13:$I$72,$C$13:$C$72,$C56,$D$13:$D$72,$D56,$R$13:$R$72,"&lt;&gt;Fermer")=0,$M56,$M56+SUMIFS($M$13:$M$72,$C$13:$C$72,$C56,$D$13:$D$72,$D56,$R$13:$R$72,"Fermer")*$I56/SUMIFS($I$13:$I$72,$C$13:$C$72,$C56,$D$13:$D$72,$D56,$R$13:$R$72,"&lt;&gt;Fermer")))</f>
+        <f>IF(OR($C56="",COUNT($H56:$Q56)=0),"",IF($R56="Fermer","",IF(SUMIFS($I$13:$I$72,$C$13:$C$72,$C56,$D$13:$D$72,$D56,$R$13:$R$72,"&lt;&gt;Fermer")=0,$M56,$M56+SUMIFS($M$13:$M$72,$C$13:$C$72,$C56,$D$13:$D$72,$D56,$R$13:$R$72,"Fermer")*$I56/SUMIFS($I$13:$I$72,$C$13:$C$72,$C56,$D$13:$D$72,$D56,$R$13:$R$72,"&lt;&gt;Fermer"))))</f>
       </c>
       <c r="T56" s="75">
-        <f>IF($R56="Fermer","",$J56-$K56-$S56)</f>
+        <f>IF(OR($C56="",COUNT($H56:$Q56)=0),"",IF($R56="Fermer","",$J56-$K56-$S56))</f>
       </c>
       <c r="U56" s="74">
-        <f>IF($R56="Fermer",-$L56,0)</f>
+        <f>IF(OR($C56="",COUNT($H56:$Q56)=0),"",IF($R56="Fermer",-$L56,0))</f>
       </c>
       <c r="V56" s="76">
-        <f>IF($R56="Fermer","Fermer = perdre "&amp;TEXT($L56,"#,##0")&amp;" € de contribution. Le fixe, lui, reste.",IF(AND($O56&gt;=0,$T56&lt;0),"BASCULE : saine avant, en déficit à cause d'une fermeture voisine.",IF(AND($O56&lt;0,$L56&gt;0),"Déficit au coût complet mais contribution positive : ne pas fermer, c'est un artefact d'allocation.",IF($O56&lt;0,"Contribution négative : vrai point dur.","Rentable. Point mort "&amp;TEXT($P56,"#,##0")&amp;" étudiants, marge de sécurité "&amp;TEXT($Q56,"0%")&amp;"."))))</f>
+        <f>IF(OR($C56="",COUNT($H56:$Q56)=0),"",IF($R56="Fermer","Fermer = perdre "&amp;TEXT($L56,"#,##0")&amp;" € de contribution. Le fixe, lui, reste.",IF(AND($O56&gt;=0,$T56&lt;0),"BASCULE : saine avant, en déficit à cause d'une fermeture voisine.",IF(AND($O56&lt;0,$L56&gt;0),"Déficit au coût complet mais contribution positive : ne pas fermer, c'est un artefact d'allocation.",IF($O56&lt;0,"Contribution négative : vrai point dur.","Rentable. Point mort "&amp;TEXT($P56,"#,##0")&amp;" étudiants, marge de sécurité "&amp;TEXT($Q56,"0%")&amp;".")))))</f>
       </c>
       <c r="W56" s="47"/>
       <c r="X56" s="47"/>
@@ -14832,16 +14832,16 @@
         <v>112</v>
       </c>
       <c r="S57" s="74">
-        <f>IF($R57="Fermer","",IF(SUMIFS($I$13:$I$72,$C$13:$C$72,$C57,$D$13:$D$72,$D57,$R$13:$R$72,"&lt;&gt;Fermer")=0,$M57,$M57+SUMIFS($M$13:$M$72,$C$13:$C$72,$C57,$D$13:$D$72,$D57,$R$13:$R$72,"Fermer")*$I57/SUMIFS($I$13:$I$72,$C$13:$C$72,$C57,$D$13:$D$72,$D57,$R$13:$R$72,"&lt;&gt;Fermer")))</f>
+        <f>IF(OR($C57="",COUNT($H57:$Q57)=0),"",IF($R57="Fermer","",IF(SUMIFS($I$13:$I$72,$C$13:$C$72,$C57,$D$13:$D$72,$D57,$R$13:$R$72,"&lt;&gt;Fermer")=0,$M57,$M57+SUMIFS($M$13:$M$72,$C$13:$C$72,$C57,$D$13:$D$72,$D57,$R$13:$R$72,"Fermer")*$I57/SUMIFS($I$13:$I$72,$C$13:$C$72,$C57,$D$13:$D$72,$D57,$R$13:$R$72,"&lt;&gt;Fermer"))))</f>
       </c>
       <c r="T57" s="75">
-        <f>IF($R57="Fermer","",$J57-$K57-$S57)</f>
+        <f>IF(OR($C57="",COUNT($H57:$Q57)=0),"",IF($R57="Fermer","",$J57-$K57-$S57))</f>
       </c>
       <c r="U57" s="74">
-        <f>IF($R57="Fermer",-$L57,0)</f>
+        <f>IF(OR($C57="",COUNT($H57:$Q57)=0),"",IF($R57="Fermer",-$L57,0))</f>
       </c>
       <c r="V57" s="76">
-        <f>IF($R57="Fermer","Fermer = perdre "&amp;TEXT($L57,"#,##0")&amp;" € de contribution. Le fixe, lui, reste.",IF(AND($O57&gt;=0,$T57&lt;0),"BASCULE : saine avant, en déficit à cause d'une fermeture voisine.",IF(AND($O57&lt;0,$L57&gt;0),"Déficit au coût complet mais contribution positive : ne pas fermer, c'est un artefact d'allocation.",IF($O57&lt;0,"Contribution négative : vrai point dur.","Rentable. Point mort "&amp;TEXT($P57,"#,##0")&amp;" étudiants, marge de sécurité "&amp;TEXT($Q57,"0%")&amp;"."))))</f>
+        <f>IF(OR($C57="",COUNT($H57:$Q57)=0),"",IF($R57="Fermer","Fermer = perdre "&amp;TEXT($L57,"#,##0")&amp;" € de contribution. Le fixe, lui, reste.",IF(AND($O57&gt;=0,$T57&lt;0),"BASCULE : saine avant, en déficit à cause d'une fermeture voisine.",IF(AND($O57&lt;0,$L57&gt;0),"Déficit au coût complet mais contribution positive : ne pas fermer, c'est un artefact d'allocation.",IF($O57&lt;0,"Contribution négative : vrai point dur.","Rentable. Point mort "&amp;TEXT($P57,"#,##0")&amp;" étudiants, marge de sécurité "&amp;TEXT($Q57,"0%")&amp;".")))))</f>
       </c>
       <c r="W57" s="47"/>
       <c r="X57" s="47"/>
@@ -14904,16 +14904,16 @@
         <v>115</v>
       </c>
       <c r="S58" s="74">
-        <f>IF($R58="Fermer","",IF(SUMIFS($I$13:$I$72,$C$13:$C$72,$C58,$D$13:$D$72,$D58,$R$13:$R$72,"&lt;&gt;Fermer")=0,$M58,$M58+SUMIFS($M$13:$M$72,$C$13:$C$72,$C58,$D$13:$D$72,$D58,$R$13:$R$72,"Fermer")*$I58/SUMIFS($I$13:$I$72,$C$13:$C$72,$C58,$D$13:$D$72,$D58,$R$13:$R$72,"&lt;&gt;Fermer")))</f>
+        <f>IF(OR($C58="",COUNT($H58:$Q58)=0),"",IF($R58="Fermer","",IF(SUMIFS($I$13:$I$72,$C$13:$C$72,$C58,$D$13:$D$72,$D58,$R$13:$R$72,"&lt;&gt;Fermer")=0,$M58,$M58+SUMIFS($M$13:$M$72,$C$13:$C$72,$C58,$D$13:$D$72,$D58,$R$13:$R$72,"Fermer")*$I58/SUMIFS($I$13:$I$72,$C$13:$C$72,$C58,$D$13:$D$72,$D58,$R$13:$R$72,"&lt;&gt;Fermer"))))</f>
       </c>
       <c r="T58" s="75">
-        <f>IF($R58="Fermer","",$J58-$K58-$S58)</f>
+        <f>IF(OR($C58="",COUNT($H58:$Q58)=0),"",IF($R58="Fermer","",$J58-$K58-$S58))</f>
       </c>
       <c r="U58" s="74">
-        <f>IF($R58="Fermer",-$L58,0)</f>
+        <f>IF(OR($C58="",COUNT($H58:$Q58)=0),"",IF($R58="Fermer",-$L58,0))</f>
       </c>
       <c r="V58" s="76">
-        <f>IF($R58="Fermer","Fermer = perdre "&amp;TEXT($L58,"#,##0")&amp;" € de contribution. Le fixe, lui, reste.",IF(AND($O58&gt;=0,$T58&lt;0),"BASCULE : saine avant, en déficit à cause d'une fermeture voisine.",IF(AND($O58&lt;0,$L58&gt;0),"Déficit au coût complet mais contribution positive : ne pas fermer, c'est un artefact d'allocation.",IF($O58&lt;0,"Contribution négative : vrai point dur.","Rentable. Point mort "&amp;TEXT($P58,"#,##0")&amp;" étudiants, marge de sécurité "&amp;TEXT($Q58,"0%")&amp;"."))))</f>
+        <f>IF(OR($C58="",COUNT($H58:$Q58)=0),"",IF($R58="Fermer","Fermer = perdre "&amp;TEXT($L58,"#,##0")&amp;" € de contribution. Le fixe, lui, reste.",IF(AND($O58&gt;=0,$T58&lt;0),"BASCULE : saine avant, en déficit à cause d'une fermeture voisine.",IF(AND($O58&lt;0,$L58&gt;0),"Déficit au coût complet mais contribution positive : ne pas fermer, c'est un artefact d'allocation.",IF($O58&lt;0,"Contribution négative : vrai point dur.","Rentable. Point mort "&amp;TEXT($P58,"#,##0")&amp;" étudiants, marge de sécurité "&amp;TEXT($Q58,"0%")&amp;".")))))</f>
       </c>
       <c r="W58" s="47"/>
       <c r="X58" s="47"/>
@@ -14976,16 +14976,16 @@
         <v>112</v>
       </c>
       <c r="S59" s="74">
-        <f>IF($R59="Fermer","",IF(SUMIFS($I$13:$I$72,$C$13:$C$72,$C59,$D$13:$D$72,$D59,$R$13:$R$72,"&lt;&gt;Fermer")=0,$M59,$M59+SUMIFS($M$13:$M$72,$C$13:$C$72,$C59,$D$13:$D$72,$D59,$R$13:$R$72,"Fermer")*$I59/SUMIFS($I$13:$I$72,$C$13:$C$72,$C59,$D$13:$D$72,$D59,$R$13:$R$72,"&lt;&gt;Fermer")))</f>
+        <f>IF(OR($C59="",COUNT($H59:$Q59)=0),"",IF($R59="Fermer","",IF(SUMIFS($I$13:$I$72,$C$13:$C$72,$C59,$D$13:$D$72,$D59,$R$13:$R$72,"&lt;&gt;Fermer")=0,$M59,$M59+SUMIFS($M$13:$M$72,$C$13:$C$72,$C59,$D$13:$D$72,$D59,$R$13:$R$72,"Fermer")*$I59/SUMIFS($I$13:$I$72,$C$13:$C$72,$C59,$D$13:$D$72,$D59,$R$13:$R$72,"&lt;&gt;Fermer"))))</f>
       </c>
       <c r="T59" s="75">
-        <f>IF($R59="Fermer","",$J59-$K59-$S59)</f>
+        <f>IF(OR($C59="",COUNT($H59:$Q59)=0),"",IF($R59="Fermer","",$J59-$K59-$S59))</f>
       </c>
       <c r="U59" s="74">
-        <f>IF($R59="Fermer",-$L59,0)</f>
+        <f>IF(OR($C59="",COUNT($H59:$Q59)=0),"",IF($R59="Fermer",-$L59,0))</f>
       </c>
       <c r="V59" s="76">
-        <f>IF($R59="Fermer","Fermer = perdre "&amp;TEXT($L59,"#,##0")&amp;" € de contribution. Le fixe, lui, reste.",IF(AND($O59&gt;=0,$T59&lt;0),"BASCULE : saine avant, en déficit à cause d'une fermeture voisine.",IF(AND($O59&lt;0,$L59&gt;0),"Déficit au coût complet mais contribution positive : ne pas fermer, c'est un artefact d'allocation.",IF($O59&lt;0,"Contribution négative : vrai point dur.","Rentable. Point mort "&amp;TEXT($P59,"#,##0")&amp;" étudiants, marge de sécurité "&amp;TEXT($Q59,"0%")&amp;"."))))</f>
+        <f>IF(OR($C59="",COUNT($H59:$Q59)=0),"",IF($R59="Fermer","Fermer = perdre "&amp;TEXT($L59,"#,##0")&amp;" € de contribution. Le fixe, lui, reste.",IF(AND($O59&gt;=0,$T59&lt;0),"BASCULE : saine avant, en déficit à cause d'une fermeture voisine.",IF(AND($O59&lt;0,$L59&gt;0),"Déficit au coût complet mais contribution positive : ne pas fermer, c'est un artefact d'allocation.",IF($O59&lt;0,"Contribution négative : vrai point dur.","Rentable. Point mort "&amp;TEXT($P59,"#,##0")&amp;" étudiants, marge de sécurité "&amp;TEXT($Q59,"0%")&amp;".")))))</f>
       </c>
       <c r="W59" s="47"/>
       <c r="X59" s="47"/>
@@ -15048,16 +15048,16 @@
         <v>115</v>
       </c>
       <c r="S60" s="74">
-        <f>IF($R60="Fermer","",IF(SUMIFS($I$13:$I$72,$C$13:$C$72,$C60,$D$13:$D$72,$D60,$R$13:$R$72,"&lt;&gt;Fermer")=0,$M60,$M60+SUMIFS($M$13:$M$72,$C$13:$C$72,$C60,$D$13:$D$72,$D60,$R$13:$R$72,"Fermer")*$I60/SUMIFS($I$13:$I$72,$C$13:$C$72,$C60,$D$13:$D$72,$D60,$R$13:$R$72,"&lt;&gt;Fermer")))</f>
+        <f>IF(OR($C60="",COUNT($H60:$Q60)=0),"",IF($R60="Fermer","",IF(SUMIFS($I$13:$I$72,$C$13:$C$72,$C60,$D$13:$D$72,$D60,$R$13:$R$72,"&lt;&gt;Fermer")=0,$M60,$M60+SUMIFS($M$13:$M$72,$C$13:$C$72,$C60,$D$13:$D$72,$D60,$R$13:$R$72,"Fermer")*$I60/SUMIFS($I$13:$I$72,$C$13:$C$72,$C60,$D$13:$D$72,$D60,$R$13:$R$72,"&lt;&gt;Fermer"))))</f>
       </c>
       <c r="T60" s="75">
-        <f>IF($R60="Fermer","",$J60-$K60-$S60)</f>
+        <f>IF(OR($C60="",COUNT($H60:$Q60)=0),"",IF($R60="Fermer","",$J60-$K60-$S60))</f>
       </c>
       <c r="U60" s="74">
-        <f>IF($R60="Fermer",-$L60,0)</f>
+        <f>IF(OR($C60="",COUNT($H60:$Q60)=0),"",IF($R60="Fermer",-$L60,0))</f>
       </c>
       <c r="V60" s="76">
-        <f>IF($R60="Fermer","Fermer = perdre "&amp;TEXT($L60,"#,##0")&amp;" € de contribution. Le fixe, lui, reste.",IF(AND($O60&gt;=0,$T60&lt;0),"BASCULE : saine avant, en déficit à cause d'une fermeture voisine.",IF(AND($O60&lt;0,$L60&gt;0),"Déficit au coût complet mais contribution positive : ne pas fermer, c'est un artefact d'allocation.",IF($O60&lt;0,"Contribution négative : vrai point dur.","Rentable. Point mort "&amp;TEXT($P60,"#,##0")&amp;" étudiants, marge de sécurité "&amp;TEXT($Q60,"0%")&amp;"."))))</f>
+        <f>IF(OR($C60="",COUNT($H60:$Q60)=0),"",IF($R60="Fermer","Fermer = perdre "&amp;TEXT($L60,"#,##0")&amp;" € de contribution. Le fixe, lui, reste.",IF(AND($O60&gt;=0,$T60&lt;0),"BASCULE : saine avant, en déficit à cause d'une fermeture voisine.",IF(AND($O60&lt;0,$L60&gt;0),"Déficit au coût complet mais contribution positive : ne pas fermer, c'est un artefact d'allocation.",IF($O60&lt;0,"Contribution négative : vrai point dur.","Rentable. Point mort "&amp;TEXT($P60,"#,##0")&amp;" étudiants, marge de sécurité "&amp;TEXT($Q60,"0%")&amp;".")))))</f>
       </c>
     </row>
     <row r="61" ht="14.25" customHeight="1">
@@ -15111,16 +15111,16 @@
         <v>115</v>
       </c>
       <c r="S61" s="74">
-        <f>IF($R61="Fermer","",IF(SUMIFS($I$13:$I$72,$C$13:$C$72,$C61,$D$13:$D$72,$D61,$R$13:$R$72,"&lt;&gt;Fermer")=0,$M61,$M61+SUMIFS($M$13:$M$72,$C$13:$C$72,$C61,$D$13:$D$72,$D61,$R$13:$R$72,"Fermer")*$I61/SUMIFS($I$13:$I$72,$C$13:$C$72,$C61,$D$13:$D$72,$D61,$R$13:$R$72,"&lt;&gt;Fermer")))</f>
+        <f>IF(OR($C61="",COUNT($H61:$Q61)=0),"",IF($R61="Fermer","",IF(SUMIFS($I$13:$I$72,$C$13:$C$72,$C61,$D$13:$D$72,$D61,$R$13:$R$72,"&lt;&gt;Fermer")=0,$M61,$M61+SUMIFS($M$13:$M$72,$C$13:$C$72,$C61,$D$13:$D$72,$D61,$R$13:$R$72,"Fermer")*$I61/SUMIFS($I$13:$I$72,$C$13:$C$72,$C61,$D$13:$D$72,$D61,$R$13:$R$72,"&lt;&gt;Fermer"))))</f>
       </c>
       <c r="T61" s="75">
-        <f>IF($R61="Fermer","",$J61-$K61-$S61)</f>
+        <f>IF(OR($C61="",COUNT($H61:$Q61)=0),"",IF($R61="Fermer","",$J61-$K61-$S61))</f>
       </c>
       <c r="U61" s="74">
-        <f>IF($R61="Fermer",-$L61,0)</f>
+        <f>IF(OR($C61="",COUNT($H61:$Q61)=0),"",IF($R61="Fermer",-$L61,0))</f>
       </c>
       <c r="V61" s="76">
-        <f>IF($R61="Fermer","Fermer = perdre "&amp;TEXT($L61,"#,##0")&amp;" € de contribution. Le fixe, lui, reste.",IF(AND($O61&gt;=0,$T61&lt;0),"BASCULE : saine avant, en déficit à cause d'une fermeture voisine.",IF(AND($O61&lt;0,$L61&gt;0),"Déficit au coût complet mais contribution positive : ne pas fermer, c'est un artefact d'allocation.",IF($O61&lt;0,"Contribution négative : vrai point dur.","Rentable. Point mort "&amp;TEXT($P61,"#,##0")&amp;" étudiants, marge de sécurité "&amp;TEXT($Q61,"0%")&amp;"."))))</f>
+        <f>IF(OR($C61="",COUNT($H61:$Q61)=0),"",IF($R61="Fermer","Fermer = perdre "&amp;TEXT($L61,"#,##0")&amp;" € de contribution. Le fixe, lui, reste.",IF(AND($O61&gt;=0,$T61&lt;0),"BASCULE : saine avant, en déficit à cause d'une fermeture voisine.",IF(AND($O61&lt;0,$L61&gt;0),"Déficit au coût complet mais contribution positive : ne pas fermer, c'est un artefact d'allocation.",IF($O61&lt;0,"Contribution négative : vrai point dur.","Rentable. Point mort "&amp;TEXT($P61,"#,##0")&amp;" étudiants, marge de sécurité "&amp;TEXT($Q61,"0%")&amp;".")))))</f>
       </c>
     </row>
     <row r="62" ht="14.25" customHeight="1">
@@ -15174,16 +15174,16 @@
         <v>115</v>
       </c>
       <c r="S62" s="74">
-        <f>IF($R62="Fermer","",IF(SUMIFS($I$13:$I$72,$C$13:$C$72,$C62,$D$13:$D$72,$D62,$R$13:$R$72,"&lt;&gt;Fermer")=0,$M62,$M62+SUMIFS($M$13:$M$72,$C$13:$C$72,$C62,$D$13:$D$72,$D62,$R$13:$R$72,"Fermer")*$I62/SUMIFS($I$13:$I$72,$C$13:$C$72,$C62,$D$13:$D$72,$D62,$R$13:$R$72,"&lt;&gt;Fermer")))</f>
+        <f>IF(OR($C62="",COUNT($H62:$Q62)=0),"",IF($R62="Fermer","",IF(SUMIFS($I$13:$I$72,$C$13:$C$72,$C62,$D$13:$D$72,$D62,$R$13:$R$72,"&lt;&gt;Fermer")=0,$M62,$M62+SUMIFS($M$13:$M$72,$C$13:$C$72,$C62,$D$13:$D$72,$D62,$R$13:$R$72,"Fermer")*$I62/SUMIFS($I$13:$I$72,$C$13:$C$72,$C62,$D$13:$D$72,$D62,$R$13:$R$72,"&lt;&gt;Fermer"))))</f>
       </c>
       <c r="T62" s="75">
-        <f>IF($R62="Fermer","",$J62-$K62-$S62)</f>
+        <f>IF(OR($C62="",COUNT($H62:$Q62)=0),"",IF($R62="Fermer","",$J62-$K62-$S62))</f>
       </c>
       <c r="U62" s="74">
-        <f>IF($R62="Fermer",-$L62,0)</f>
+        <f>IF(OR($C62="",COUNT($H62:$Q62)=0),"",IF($R62="Fermer",-$L62,0))</f>
       </c>
       <c r="V62" s="76">
-        <f>IF($R62="Fermer","Fermer = perdre "&amp;TEXT($L62,"#,##0")&amp;" € de contribution. Le fixe, lui, reste.",IF(AND($O62&gt;=0,$T62&lt;0),"BASCULE : saine avant, en déficit à cause d'une fermeture voisine.",IF(AND($O62&lt;0,$L62&gt;0),"Déficit au coût complet mais contribution positive : ne pas fermer, c'est un artefact d'allocation.",IF($O62&lt;0,"Contribution négative : vrai point dur.","Rentable. Point mort "&amp;TEXT($P62,"#,##0")&amp;" étudiants, marge de sécurité "&amp;TEXT($Q62,"0%")&amp;"."))))</f>
+        <f>IF(OR($C62="",COUNT($H62:$Q62)=0),"",IF($R62="Fermer","Fermer = perdre "&amp;TEXT($L62,"#,##0")&amp;" € de contribution. Le fixe, lui, reste.",IF(AND($O62&gt;=0,$T62&lt;0),"BASCULE : saine avant, en déficit à cause d'une fermeture voisine.",IF(AND($O62&lt;0,$L62&gt;0),"Déficit au coût complet mais contribution positive : ne pas fermer, c'est un artefact d'allocation.",IF($O62&lt;0,"Contribution négative : vrai point dur.","Rentable. Point mort "&amp;TEXT($P62,"#,##0")&amp;" étudiants, marge de sécurité "&amp;TEXT($Q62,"0%")&amp;".")))))</f>
       </c>
     </row>
     <row r="63" ht="14.25" customHeight="1">
@@ -15237,16 +15237,16 @@
         <v>115</v>
       </c>
       <c r="S63" s="74">
-        <f>IF($R63="Fermer","",IF(SUMIFS($I$13:$I$72,$C$13:$C$72,$C63,$D$13:$D$72,$D63,$R$13:$R$72,"&lt;&gt;Fermer")=0,$M63,$M63+SUMIFS($M$13:$M$72,$C$13:$C$72,$C63,$D$13:$D$72,$D63,$R$13:$R$72,"Fermer")*$I63/SUMIFS($I$13:$I$72,$C$13:$C$72,$C63,$D$13:$D$72,$D63,$R$13:$R$72,"&lt;&gt;Fermer")))</f>
+        <f>IF(OR($C63="",COUNT($H63:$Q63)=0),"",IF($R63="Fermer","",IF(SUMIFS($I$13:$I$72,$C$13:$C$72,$C63,$D$13:$D$72,$D63,$R$13:$R$72,"&lt;&gt;Fermer")=0,$M63,$M63+SUMIFS($M$13:$M$72,$C$13:$C$72,$C63,$D$13:$D$72,$D63,$R$13:$R$72,"Fermer")*$I63/SUMIFS($I$13:$I$72,$C$13:$C$72,$C63,$D$13:$D$72,$D63,$R$13:$R$72,"&lt;&gt;Fermer"))))</f>
       </c>
       <c r="T63" s="75">
-        <f>IF($R63="Fermer","",$J63-$K63-$S63)</f>
+        <f>IF(OR($C63="",COUNT($H63:$Q63)=0),"",IF($R63="Fermer","",$J63-$K63-$S63))</f>
       </c>
       <c r="U63" s="74">
-        <f>IF($R63="Fermer",-$L63,0)</f>
+        <f>IF(OR($C63="",COUNT($H63:$Q63)=0),"",IF($R63="Fermer",-$L63,0))</f>
       </c>
       <c r="V63" s="76">
-        <f>IF($R63="Fermer","Fermer = perdre "&amp;TEXT($L63,"#,##0")&amp;" € de contribution. Le fixe, lui, reste.",IF(AND($O63&gt;=0,$T63&lt;0),"BASCULE : saine avant, en déficit à cause d'une fermeture voisine.",IF(AND($O63&lt;0,$L63&gt;0),"Déficit au coût complet mais contribution positive : ne pas fermer, c'est un artefact d'allocation.",IF($O63&lt;0,"Contribution négative : vrai point dur.","Rentable. Point mort "&amp;TEXT($P63,"#,##0")&amp;" étudiants, marge de sécurité "&amp;TEXT($Q63,"0%")&amp;"."))))</f>
+        <f>IF(OR($C63="",COUNT($H63:$Q63)=0),"",IF($R63="Fermer","Fermer = perdre "&amp;TEXT($L63,"#,##0")&amp;" € de contribution. Le fixe, lui, reste.",IF(AND($O63&gt;=0,$T63&lt;0),"BASCULE : saine avant, en déficit à cause d'une fermeture voisine.",IF(AND($O63&lt;0,$L63&gt;0),"Déficit au coût complet mais contribution positive : ne pas fermer, c'est un artefact d'allocation.",IF($O63&lt;0,"Contribution négative : vrai point dur.","Rentable. Point mort "&amp;TEXT($P63,"#,##0")&amp;" étudiants, marge de sécurité "&amp;TEXT($Q63,"0%")&amp;".")))))</f>
       </c>
     </row>
     <row r="64" ht="14.25" customHeight="1">
@@ -15300,16 +15300,16 @@
         <v>112</v>
       </c>
       <c r="S64" s="74">
-        <f>IF($R64="Fermer","",IF(SUMIFS($I$13:$I$72,$C$13:$C$72,$C64,$D$13:$D$72,$D64,$R$13:$R$72,"&lt;&gt;Fermer")=0,$M64,$M64+SUMIFS($M$13:$M$72,$C$13:$C$72,$C64,$D$13:$D$72,$D64,$R$13:$R$72,"Fermer")*$I64/SUMIFS($I$13:$I$72,$C$13:$C$72,$C64,$D$13:$D$72,$D64,$R$13:$R$72,"&lt;&gt;Fermer")))</f>
+        <f>IF(OR($C64="",COUNT($H64:$Q64)=0),"",IF($R64="Fermer","",IF(SUMIFS($I$13:$I$72,$C$13:$C$72,$C64,$D$13:$D$72,$D64,$R$13:$R$72,"&lt;&gt;Fermer")=0,$M64,$M64+SUMIFS($M$13:$M$72,$C$13:$C$72,$C64,$D$13:$D$72,$D64,$R$13:$R$72,"Fermer")*$I64/SUMIFS($I$13:$I$72,$C$13:$C$72,$C64,$D$13:$D$72,$D64,$R$13:$R$72,"&lt;&gt;Fermer"))))</f>
       </c>
       <c r="T64" s="75">
-        <f>IF($R64="Fermer","",$J64-$K64-$S64)</f>
+        <f>IF(OR($C64="",COUNT($H64:$Q64)=0),"",IF($R64="Fermer","",$J64-$K64-$S64))</f>
       </c>
       <c r="U64" s="74">
-        <f>IF($R64="Fermer",-$L64,0)</f>
+        <f>IF(OR($C64="",COUNT($H64:$Q64)=0),"",IF($R64="Fermer",-$L64,0))</f>
       </c>
       <c r="V64" s="76">
-        <f>IF($R64="Fermer","Fermer = perdre "&amp;TEXT($L64,"#,##0")&amp;" € de contribution. Le fixe, lui, reste.",IF(AND($O64&gt;=0,$T64&lt;0),"BASCULE : saine avant, en déficit à cause d'une fermeture voisine.",IF(AND($O64&lt;0,$L64&gt;0),"Déficit au coût complet mais contribution positive : ne pas fermer, c'est un artefact d'allocation.",IF($O64&lt;0,"Contribution négative : vrai point dur.","Rentable. Point mort "&amp;TEXT($P64,"#,##0")&amp;" étudiants, marge de sécurité "&amp;TEXT($Q64,"0%")&amp;"."))))</f>
+        <f>IF(OR($C64="",COUNT($H64:$Q64)=0),"",IF($R64="Fermer","Fermer = perdre "&amp;TEXT($L64,"#,##0")&amp;" € de contribution. Le fixe, lui, reste.",IF(AND($O64&gt;=0,$T64&lt;0),"BASCULE : saine avant, en déficit à cause d'une fermeture voisine.",IF(AND($O64&lt;0,$L64&gt;0),"Déficit au coût complet mais contribution positive : ne pas fermer, c'est un artefact d'allocation.",IF($O64&lt;0,"Contribution négative : vrai point dur.","Rentable. Point mort "&amp;TEXT($P64,"#,##0")&amp;" étudiants, marge de sécurité "&amp;TEXT($Q64,"0%")&amp;".")))))</f>
       </c>
     </row>
     <row r="65" ht="14.25" customHeight="1">
@@ -15363,16 +15363,16 @@
         <v>115</v>
       </c>
       <c r="S65" s="74">
-        <f>IF($R65="Fermer","",IF(SUMIFS($I$13:$I$72,$C$13:$C$72,$C65,$D$13:$D$72,$D65,$R$13:$R$72,"&lt;&gt;Fermer")=0,$M65,$M65+SUMIFS($M$13:$M$72,$C$13:$C$72,$C65,$D$13:$D$72,$D65,$R$13:$R$72,"Fermer")*$I65/SUMIFS($I$13:$I$72,$C$13:$C$72,$C65,$D$13:$D$72,$D65,$R$13:$R$72,"&lt;&gt;Fermer")))</f>
+        <f>IF(OR($C65="",COUNT($H65:$Q65)=0),"",IF($R65="Fermer","",IF(SUMIFS($I$13:$I$72,$C$13:$C$72,$C65,$D$13:$D$72,$D65,$R$13:$R$72,"&lt;&gt;Fermer")=0,$M65,$M65+SUMIFS($M$13:$M$72,$C$13:$C$72,$C65,$D$13:$D$72,$D65,$R$13:$R$72,"Fermer")*$I65/SUMIFS($I$13:$I$72,$C$13:$C$72,$C65,$D$13:$D$72,$D65,$R$13:$R$72,"&lt;&gt;Fermer"))))</f>
       </c>
       <c r="T65" s="75">
-        <f>IF($R65="Fermer","",$J65-$K65-$S65)</f>
+        <f>IF(OR($C65="",COUNT($H65:$Q65)=0),"",IF($R65="Fermer","",$J65-$K65-$S65))</f>
       </c>
       <c r="U65" s="74">
-        <f>IF($R65="Fermer",-$L65,0)</f>
+        <f>IF(OR($C65="",COUNT($H65:$Q65)=0),"",IF($R65="Fermer",-$L65,0))</f>
       </c>
       <c r="V65" s="76">
-        <f>IF($R65="Fermer","Fermer = perdre "&amp;TEXT($L65,"#,##0")&amp;" € de contribution. Le fixe, lui, reste.",IF(AND($O65&gt;=0,$T65&lt;0),"BASCULE : saine avant, en déficit à cause d'une fermeture voisine.",IF(AND($O65&lt;0,$L65&gt;0),"Déficit au coût complet mais contribution positive : ne pas fermer, c'est un artefact d'allocation.",IF($O65&lt;0,"Contribution négative : vrai point dur.","Rentable. Point mort "&amp;TEXT($P65,"#,##0")&amp;" étudiants, marge de sécurité "&amp;TEXT($Q65,"0%")&amp;"."))))</f>
+        <f>IF(OR($C65="",COUNT($H65:$Q65)=0),"",IF($R65="Fermer","Fermer = perdre "&amp;TEXT($L65,"#,##0")&amp;" € de contribution. Le fixe, lui, reste.",IF(AND($O65&gt;=0,$T65&lt;0),"BASCULE : saine avant, en déficit à cause d'une fermeture voisine.",IF(AND($O65&lt;0,$L65&gt;0),"Déficit au coût complet mais contribution positive : ne pas fermer, c'est un artefact d'allocation.",IF($O65&lt;0,"Contribution négative : vrai point dur.","Rentable. Point mort "&amp;TEXT($P65,"#,##0")&amp;" étudiants, marge de sécurité "&amp;TEXT($Q65,"0%")&amp;".")))))</f>
       </c>
     </row>
     <row r="66" ht="14.25" customHeight="1">
@@ -15426,16 +15426,16 @@
         <v>112</v>
       </c>
       <c r="S66" s="74">
-        <f>IF($R66="Fermer","",IF(SUMIFS($I$13:$I$72,$C$13:$C$72,$C66,$D$13:$D$72,$D66,$R$13:$R$72,"&lt;&gt;Fermer")=0,$M66,$M66+SUMIFS($M$13:$M$72,$C$13:$C$72,$C66,$D$13:$D$72,$D66,$R$13:$R$72,"Fermer")*$I66/SUMIFS($I$13:$I$72,$C$13:$C$72,$C66,$D$13:$D$72,$D66,$R$13:$R$72,"&lt;&gt;Fermer")))</f>
+        <f>IF(OR($C66="",COUNT($H66:$Q66)=0),"",IF($R66="Fermer","",IF(SUMIFS($I$13:$I$72,$C$13:$C$72,$C66,$D$13:$D$72,$D66,$R$13:$R$72,"&lt;&gt;Fermer")=0,$M66,$M66+SUMIFS($M$13:$M$72,$C$13:$C$72,$C66,$D$13:$D$72,$D66,$R$13:$R$72,"Fermer")*$I66/SUMIFS($I$13:$I$72,$C$13:$C$72,$C66,$D$13:$D$72,$D66,$R$13:$R$72,"&lt;&gt;Fermer"))))</f>
       </c>
       <c r="T66" s="75">
-        <f>IF($R66="Fermer","",$J66-$K66-$S66)</f>
+        <f>IF(OR($C66="",COUNT($H66:$Q66)=0),"",IF($R66="Fermer","",$J66-$K66-$S66))</f>
       </c>
       <c r="U66" s="74">
-        <f>IF($R66="Fermer",-$L66,0)</f>
+        <f>IF(OR($C66="",COUNT($H66:$Q66)=0),"",IF($R66="Fermer",-$L66,0))</f>
       </c>
       <c r="V66" s="76">
-        <f>IF($R66="Fermer","Fermer = perdre "&amp;TEXT($L66,"#,##0")&amp;" € de contribution. Le fixe, lui, reste.",IF(AND($O66&gt;=0,$T66&lt;0),"BASCULE : saine avant, en déficit à cause d'une fermeture voisine.",IF(AND($O66&lt;0,$L66&gt;0),"Déficit au coût complet mais contribution positive : ne pas fermer, c'est un artefact d'allocation.",IF($O66&lt;0,"Contribution négative : vrai point dur.","Rentable. Point mort "&amp;TEXT($P66,"#,##0")&amp;" étudiants, marge de sécurité "&amp;TEXT($Q66,"0%")&amp;"."))))</f>
+        <f>IF(OR($C66="",COUNT($H66:$Q66)=0),"",IF($R66="Fermer","Fermer = perdre "&amp;TEXT($L66,"#,##0")&amp;" € de contribution. Le fixe, lui, reste.",IF(AND($O66&gt;=0,$T66&lt;0),"BASCULE : saine avant, en déficit à cause d'une fermeture voisine.",IF(AND($O66&lt;0,$L66&gt;0),"Déficit au coût complet mais contribution positive : ne pas fermer, c'est un artefact d'allocation.",IF($O66&lt;0,"Contribution négative : vrai point dur.","Rentable. Point mort "&amp;TEXT($P66,"#,##0")&amp;" étudiants, marge de sécurité "&amp;TEXT($Q66,"0%")&amp;".")))))</f>
       </c>
     </row>
     <row r="67" ht="14.25" customHeight="1">
@@ -15489,16 +15489,16 @@
         <v>112</v>
       </c>
       <c r="S67" s="74">
-        <f>IF($R67="Fermer","",IF(SUMIFS($I$13:$I$72,$C$13:$C$72,$C67,$D$13:$D$72,$D67,$R$13:$R$72,"&lt;&gt;Fermer")=0,$M67,$M67+SUMIFS($M$13:$M$72,$C$13:$C$72,$C67,$D$13:$D$72,$D67,$R$13:$R$72,"Fermer")*$I67/SUMIFS($I$13:$I$72,$C$13:$C$72,$C67,$D$13:$D$72,$D67,$R$13:$R$72,"&lt;&gt;Fermer")))</f>
+        <f>IF(OR($C67="",COUNT($H67:$Q67)=0),"",IF($R67="Fermer","",IF(SUMIFS($I$13:$I$72,$C$13:$C$72,$C67,$D$13:$D$72,$D67,$R$13:$R$72,"&lt;&gt;Fermer")=0,$M67,$M67+SUMIFS($M$13:$M$72,$C$13:$C$72,$C67,$D$13:$D$72,$D67,$R$13:$R$72,"Fermer")*$I67/SUMIFS($I$13:$I$72,$C$13:$C$72,$C67,$D$13:$D$72,$D67,$R$13:$R$72,"&lt;&gt;Fermer"))))</f>
       </c>
       <c r="T67" s="75">
-        <f>IF($R67="Fermer","",$J67-$K67-$S67)</f>
+        <f>IF(OR($C67="",COUNT($H67:$Q67)=0),"",IF($R67="Fermer","",$J67-$K67-$S67))</f>
       </c>
       <c r="U67" s="74">
-        <f>IF($R67="Fermer",-$L67,0)</f>
+        <f>IF(OR($C67="",COUNT($H67:$Q67)=0),"",IF($R67="Fermer",-$L67,0))</f>
       </c>
       <c r="V67" s="76">
-        <f>IF($R67="Fermer","Fermer = perdre "&amp;TEXT($L67,"#,##0")&amp;" € de contribution. Le fixe, lui, reste.",IF(AND($O67&gt;=0,$T67&lt;0),"BASCULE : saine avant, en déficit à cause d'une fermeture voisine.",IF(AND($O67&lt;0,$L67&gt;0),"Déficit au coût complet mais contribution positive : ne pas fermer, c'est un artefact d'allocation.",IF($O67&lt;0,"Contribution négative : vrai point dur.","Rentable. Point mort "&amp;TEXT($P67,"#,##0")&amp;" étudiants, marge de sécurité "&amp;TEXT($Q67,"0%")&amp;"."))))</f>
+        <f>IF(OR($C67="",COUNT($H67:$Q67)=0),"",IF($R67="Fermer","Fermer = perdre "&amp;TEXT($L67,"#,##0")&amp;" € de contribution. Le fixe, lui, reste.",IF(AND($O67&gt;=0,$T67&lt;0),"BASCULE : saine avant, en déficit à cause d'une fermeture voisine.",IF(AND($O67&lt;0,$L67&gt;0),"Déficit au coût complet mais contribution positive : ne pas fermer, c'est un artefact d'allocation.",IF($O67&lt;0,"Contribution négative : vrai point dur.","Rentable. Point mort "&amp;TEXT($P67,"#,##0")&amp;" étudiants, marge de sécurité "&amp;TEXT($Q67,"0%")&amp;".")))))</f>
       </c>
     </row>
     <row r="68" ht="14.25" customHeight="1">
@@ -15552,16 +15552,16 @@
         <v>115</v>
       </c>
       <c r="S68" s="74">
-        <f>IF($R68="Fermer","",IF(SUMIFS($I$13:$I$72,$C$13:$C$72,$C68,$D$13:$D$72,$D68,$R$13:$R$72,"&lt;&gt;Fermer")=0,$M68,$M68+SUMIFS($M$13:$M$72,$C$13:$C$72,$C68,$D$13:$D$72,$D68,$R$13:$R$72,"Fermer")*$I68/SUMIFS($I$13:$I$72,$C$13:$C$72,$C68,$D$13:$D$72,$D68,$R$13:$R$72,"&lt;&gt;Fermer")))</f>
+        <f>IF(OR($C68="",COUNT($H68:$Q68)=0),"",IF($R68="Fermer","",IF(SUMIFS($I$13:$I$72,$C$13:$C$72,$C68,$D$13:$D$72,$D68,$R$13:$R$72,"&lt;&gt;Fermer")=0,$M68,$M68+SUMIFS($M$13:$M$72,$C$13:$C$72,$C68,$D$13:$D$72,$D68,$R$13:$R$72,"Fermer")*$I68/SUMIFS($I$13:$I$72,$C$13:$C$72,$C68,$D$13:$D$72,$D68,$R$13:$R$72,"&lt;&gt;Fermer"))))</f>
       </c>
       <c r="T68" s="75">
-        <f>IF($R68="Fermer","",$J68-$K68-$S68)</f>
+        <f>IF(OR($C68="",COUNT($H68:$Q68)=0),"",IF($R68="Fermer","",$J68-$K68-$S68))</f>
       </c>
       <c r="U68" s="74">
-        <f>IF($R68="Fermer",-$L68,0)</f>
+        <f>IF(OR($C68="",COUNT($H68:$Q68)=0),"",IF($R68="Fermer",-$L68,0))</f>
       </c>
       <c r="V68" s="76">
-        <f>IF($R68="Fermer","Fermer = perdre "&amp;TEXT($L68,"#,##0")&amp;" € de contribution. Le fixe, lui, reste.",IF(AND($O68&gt;=0,$T68&lt;0),"BASCULE : saine avant, en déficit à cause d'une fermeture voisine.",IF(AND($O68&lt;0,$L68&gt;0),"Déficit au coût complet mais contribution positive : ne pas fermer, c'est un artefact d'allocation.",IF($O68&lt;0,"Contribution négative : vrai point dur.","Rentable. Point mort "&amp;TEXT($P68,"#,##0")&amp;" étudiants, marge de sécurité "&amp;TEXT($Q68,"0%")&amp;"."))))</f>
+        <f>IF(OR($C68="",COUNT($H68:$Q68)=0),"",IF($R68="Fermer","Fermer = perdre "&amp;TEXT($L68,"#,##0")&amp;" € de contribution. Le fixe, lui, reste.",IF(AND($O68&gt;=0,$T68&lt;0),"BASCULE : saine avant, en déficit à cause d'une fermeture voisine.",IF(AND($O68&lt;0,$L68&gt;0),"Déficit au coût complet mais contribution positive : ne pas fermer, c'est un artefact d'allocation.",IF($O68&lt;0,"Contribution négative : vrai point dur.","Rentable. Point mort "&amp;TEXT($P68,"#,##0")&amp;" étudiants, marge de sécurité "&amp;TEXT($Q68,"0%")&amp;".")))))</f>
       </c>
     </row>
     <row r="69" ht="14.25" customHeight="1">
@@ -15615,16 +15615,16 @@
         <v>115</v>
       </c>
       <c r="S69" s="74">
-        <f>IF($R69="Fermer","",IF(SUMIFS($I$13:$I$72,$C$13:$C$72,$C69,$D$13:$D$72,$D69,$R$13:$R$72,"&lt;&gt;Fermer")=0,$M69,$M69+SUMIFS($M$13:$M$72,$C$13:$C$72,$C69,$D$13:$D$72,$D69,$R$13:$R$72,"Fermer")*$I69/SUMIFS($I$13:$I$72,$C$13:$C$72,$C69,$D$13:$D$72,$D69,$R$13:$R$72,"&lt;&gt;Fermer")))</f>
+        <f>IF(OR($C69="",COUNT($H69:$Q69)=0),"",IF($R69="Fermer","",IF(SUMIFS($I$13:$I$72,$C$13:$C$72,$C69,$D$13:$D$72,$D69,$R$13:$R$72,"&lt;&gt;Fermer")=0,$M69,$M69+SUMIFS($M$13:$M$72,$C$13:$C$72,$C69,$D$13:$D$72,$D69,$R$13:$R$72,"Fermer")*$I69/SUMIFS($I$13:$I$72,$C$13:$C$72,$C69,$D$13:$D$72,$D69,$R$13:$R$72,"&lt;&gt;Fermer"))))</f>
       </c>
       <c r="T69" s="75">
-        <f>IF($R69="Fermer","",$J69-$K69-$S69)</f>
+        <f>IF(OR($C69="",COUNT($H69:$Q69)=0),"",IF($R69="Fermer","",$J69-$K69-$S69))</f>
       </c>
       <c r="U69" s="74">
-        <f>IF($R69="Fermer",-$L69,0)</f>
+        <f>IF(OR($C69="",COUNT($H69:$Q69)=0),"",IF($R69="Fermer",-$L69,0))</f>
       </c>
       <c r="V69" s="76">
-        <f>IF($R69="Fermer","Fermer = perdre "&amp;TEXT($L69,"#,##0")&amp;" € de contribution. Le fixe, lui, reste.",IF(AND($O69&gt;=0,$T69&lt;0),"BASCULE : saine avant, en déficit à cause d'une fermeture voisine.",IF(AND($O69&lt;0,$L69&gt;0),"Déficit au coût complet mais contribution positive : ne pas fermer, c'est un artefact d'allocation.",IF($O69&lt;0,"Contribution négative : vrai point dur.","Rentable. Point mort "&amp;TEXT($P69,"#,##0")&amp;" étudiants, marge de sécurité "&amp;TEXT($Q69,"0%")&amp;"."))))</f>
+        <f>IF(OR($C69="",COUNT($H69:$Q69)=0),"",IF($R69="Fermer","Fermer = perdre "&amp;TEXT($L69,"#,##0")&amp;" € de contribution. Le fixe, lui, reste.",IF(AND($O69&gt;=0,$T69&lt;0),"BASCULE : saine avant, en déficit à cause d'une fermeture voisine.",IF(AND($O69&lt;0,$L69&gt;0),"Déficit au coût complet mais contribution positive : ne pas fermer, c'est un artefact d'allocation.",IF($O69&lt;0,"Contribution négative : vrai point dur.","Rentable. Point mort "&amp;TEXT($P69,"#,##0")&amp;" étudiants, marge de sécurité "&amp;TEXT($Q69,"0%")&amp;".")))))</f>
       </c>
     </row>
     <row r="70" ht="14.25" customHeight="1">
@@ -15678,16 +15678,16 @@
         <v>112</v>
       </c>
       <c r="S70" s="74">
-        <f>IF($R70="Fermer","",IF(SUMIFS($I$13:$I$72,$C$13:$C$72,$C70,$D$13:$D$72,$D70,$R$13:$R$72,"&lt;&gt;Fermer")=0,$M70,$M70+SUMIFS($M$13:$M$72,$C$13:$C$72,$C70,$D$13:$D$72,$D70,$R$13:$R$72,"Fermer")*$I70/SUMIFS($I$13:$I$72,$C$13:$C$72,$C70,$D$13:$D$72,$D70,$R$13:$R$72,"&lt;&gt;Fermer")))</f>
+        <f>IF(OR($C70="",COUNT($H70:$Q70)=0),"",IF($R70="Fermer","",IF(SUMIFS($I$13:$I$72,$C$13:$C$72,$C70,$D$13:$D$72,$D70,$R$13:$R$72,"&lt;&gt;Fermer")=0,$M70,$M70+SUMIFS($M$13:$M$72,$C$13:$C$72,$C70,$D$13:$D$72,$D70,$R$13:$R$72,"Fermer")*$I70/SUMIFS($I$13:$I$72,$C$13:$C$72,$C70,$D$13:$D$72,$D70,$R$13:$R$72,"&lt;&gt;Fermer"))))</f>
       </c>
       <c r="T70" s="75">
-        <f>IF($R70="Fermer","",$J70-$K70-$S70)</f>
+        <f>IF(OR($C70="",COUNT($H70:$Q70)=0),"",IF($R70="Fermer","",$J70-$K70-$S70))</f>
       </c>
       <c r="U70" s="74">
-        <f>IF($R70="Fermer",-$L70,0)</f>
+        <f>IF(OR($C70="",COUNT($H70:$Q70)=0),"",IF($R70="Fermer",-$L70,0))</f>
       </c>
       <c r="V70" s="76">
-        <f>IF($R70="Fermer","Fermer = perdre "&amp;TEXT($L70,"#,##0")&amp;" € de contribution. Le fixe, lui, reste.",IF(AND($O70&gt;=0,$T70&lt;0),"BASCULE : saine avant, en déficit à cause d'une fermeture voisine.",IF(AND($O70&lt;0,$L70&gt;0),"Déficit au coût complet mais contribution positive : ne pas fermer, c'est un artefact d'allocation.",IF($O70&lt;0,"Contribution négative : vrai point dur.","Rentable. Point mort "&amp;TEXT($P70,"#,##0")&amp;" étudiants, marge de sécurité "&amp;TEXT($Q70,"0%")&amp;"."))))</f>
+        <f>IF(OR($C70="",COUNT($H70:$Q70)=0),"",IF($R70="Fermer","Fermer = perdre "&amp;TEXT($L70,"#,##0")&amp;" € de contribution. Le fixe, lui, reste.",IF(AND($O70&gt;=0,$T70&lt;0),"BASCULE : saine avant, en déficit à cause d'une fermeture voisine.",IF(AND($O70&lt;0,$L70&gt;0),"Déficit au coût complet mais contribution positive : ne pas fermer, c'est un artefact d'allocation.",IF($O70&lt;0,"Contribution négative : vrai point dur.","Rentable. Point mort "&amp;TEXT($P70,"#,##0")&amp;" étudiants, marge de sécurité "&amp;TEXT($Q70,"0%")&amp;".")))))</f>
       </c>
     </row>
     <row r="71" ht="14.25" customHeight="1">
@@ -15741,16 +15741,16 @@
         <v>115</v>
       </c>
       <c r="S71" s="74">
-        <f>IF($R71="Fermer","",IF(SUMIFS($I$13:$I$72,$C$13:$C$72,$C71,$D$13:$D$72,$D71,$R$13:$R$72,"&lt;&gt;Fermer")=0,$M71,$M71+SUMIFS($M$13:$M$72,$C$13:$C$72,$C71,$D$13:$D$72,$D71,$R$13:$R$72,"Fermer")*$I71/SUMIFS($I$13:$I$72,$C$13:$C$72,$C71,$D$13:$D$72,$D71,$R$13:$R$72,"&lt;&gt;Fermer")))</f>
+        <f>IF(OR($C71="",COUNT($H71:$Q71)=0),"",IF($R71="Fermer","",IF(SUMIFS($I$13:$I$72,$C$13:$C$72,$C71,$D$13:$D$72,$D71,$R$13:$R$72,"&lt;&gt;Fermer")=0,$M71,$M71+SUMIFS($M$13:$M$72,$C$13:$C$72,$C71,$D$13:$D$72,$D71,$R$13:$R$72,"Fermer")*$I71/SUMIFS($I$13:$I$72,$C$13:$C$72,$C71,$D$13:$D$72,$D71,$R$13:$R$72,"&lt;&gt;Fermer"))))</f>
       </c>
       <c r="T71" s="75">
-        <f>IF($R71="Fermer","",$J71-$K71-$S71)</f>
+        <f>IF(OR($C71="",COUNT($H71:$Q71)=0),"",IF($R71="Fermer","",$J71-$K71-$S71))</f>
       </c>
       <c r="U71" s="74">
-        <f>IF($R71="Fermer",-$L71,0)</f>
+        <f>IF(OR($C71="",COUNT($H71:$Q71)=0),"",IF($R71="Fermer",-$L71,0))</f>
       </c>
       <c r="V71" s="76">
-        <f>IF($R71="Fermer","Fermer = perdre "&amp;TEXT($L71,"#,##0")&amp;" € de contribution. Le fixe, lui, reste.",IF(AND($O71&gt;=0,$T71&lt;0),"BASCULE : saine avant, en déficit à cause d'une fermeture voisine.",IF(AND($O71&lt;0,$L71&gt;0),"Déficit au coût complet mais contribution positive : ne pas fermer, c'est un artefact d'allocation.",IF($O71&lt;0,"Contribution négative : vrai point dur.","Rentable. Point mort "&amp;TEXT($P71,"#,##0")&amp;" étudiants, marge de sécurité "&amp;TEXT($Q71,"0%")&amp;"."))))</f>
+        <f>IF(OR($C71="",COUNT($H71:$Q71)=0),"",IF($R71="Fermer","Fermer = perdre "&amp;TEXT($L71,"#,##0")&amp;" € de contribution. Le fixe, lui, reste.",IF(AND($O71&gt;=0,$T71&lt;0),"BASCULE : saine avant, en déficit à cause d'une fermeture voisine.",IF(AND($O71&lt;0,$L71&gt;0),"Déficit au coût complet mais contribution positive : ne pas fermer, c'est un artefact d'allocation.",IF($O71&lt;0,"Contribution négative : vrai point dur.","Rentable. Point mort "&amp;TEXT($P71,"#,##0")&amp;" étudiants, marge de sécurité "&amp;TEXT($Q71,"0%")&amp;".")))))</f>
       </c>
     </row>
     <row r="72" ht="14.25" customHeight="1">
@@ -15804,16 +15804,16 @@
         <v>115</v>
       </c>
       <c r="S72" s="74">
-        <f>IF($R72="Fermer","",IF(SUMIFS($I$13:$I$72,$C$13:$C$72,$C72,$D$13:$D$72,$D72,$R$13:$R$72,"&lt;&gt;Fermer")=0,$M72,$M72+SUMIFS($M$13:$M$72,$C$13:$C$72,$C72,$D$13:$D$72,$D72,$R$13:$R$72,"Fermer")*$I72/SUMIFS($I$13:$I$72,$C$13:$C$72,$C72,$D$13:$D$72,$D72,$R$13:$R$72,"&lt;&gt;Fermer")))</f>
+        <f>IF(OR($C72="",COUNT($H72:$Q72)=0),"",IF($R72="Fermer","",IF(SUMIFS($I$13:$I$72,$C$13:$C$72,$C72,$D$13:$D$72,$D72,$R$13:$R$72,"&lt;&gt;Fermer")=0,$M72,$M72+SUMIFS($M$13:$M$72,$C$13:$C$72,$C72,$D$13:$D$72,$D72,$R$13:$R$72,"Fermer")*$I72/SUMIFS($I$13:$I$72,$C$13:$C$72,$C72,$D$13:$D$72,$D72,$R$13:$R$72,"&lt;&gt;Fermer"))))</f>
       </c>
       <c r="T72" s="75">
-        <f>IF($R72="Fermer","",$J72-$K72-$S72)</f>
+        <f>IF(OR($C72="",COUNT($H72:$Q72)=0),"",IF($R72="Fermer","",$J72-$K72-$S72))</f>
       </c>
       <c r="U72" s="74">
-        <f>IF($R72="Fermer",-$L72,0)</f>
+        <f>IF(OR($C72="",COUNT($H72:$Q72)=0),"",IF($R72="Fermer",-$L72,0))</f>
       </c>
       <c r="V72" s="76">
-        <f>IF($R72="Fermer","Fermer = perdre "&amp;TEXT($L72,"#,##0")&amp;" € de contribution. Le fixe, lui, reste.",IF(AND($O72&gt;=0,$T72&lt;0),"BASCULE : saine avant, en déficit à cause d'une fermeture voisine.",IF(AND($O72&lt;0,$L72&gt;0),"Déficit au coût complet mais contribution positive : ne pas fermer, c'est un artefact d'allocation.",IF($O72&lt;0,"Contribution négative : vrai point dur.","Rentable. Point mort "&amp;TEXT($P72,"#,##0")&amp;" étudiants, marge de sécurité "&amp;TEXT($Q72,"0%")&amp;"."))))</f>
+        <f>IF(OR($C72="",COUNT($H72:$Q72)=0),"",IF($R72="Fermer","Fermer = perdre "&amp;TEXT($L72,"#,##0")&amp;" € de contribution. Le fixe, lui, reste.",IF(AND($O72&gt;=0,$T72&lt;0),"BASCULE : saine avant, en déficit à cause d'une fermeture voisine.",IF(AND($O72&lt;0,$L72&gt;0),"Déficit au coût complet mais contribution positive : ne pas fermer, c'est un artefact d'allocation.",IF($O72&lt;0,"Contribution négative : vrai point dur.","Rentable. Point mort "&amp;TEXT($P72,"#,##0")&amp;" étudiants, marge de sécurité "&amp;TEXT($Q72,"0%")&amp;".")))))</f>
       </c>
     </row>
     <row r="73" ht="14.25" customHeight="1">

</xml_diff>